<commit_message>
Reconcile 184 export artifacts and approved population targets in production workbook
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R3ba83cf42f084380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R1d68e4be90014be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rbfedc4d5c63245cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R9651bb0dff654338"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R4c15516a8a3244e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R4e2265908d894948"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243746"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -75,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -116,6 +121,14 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -445,15 +458,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$163,Assets!$C$6:$C$163,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A7,Assets!$B$6:$B$163,"Character",Assets!$H$6:$H$163,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A7,Assets!$B$6:$B$163,"Character",Assets!$I$6:$I$163,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -461,7 +474,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -479,20 +492,25 @@
       <x:c r="C8" s="8" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="D8" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="E8" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="F8" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="G8" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="H8" s="2" t="str">
-        <x:v>Awaiting report</x:v>
+      <x:c r="D8" s="2" t="n">
+        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A8)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="2" t="n">
+        <x:f>C8-D8</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H8" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8)</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
@@ -510,15 +528,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$163,Assets!$C$6:$C$163,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A9,Assets!$B$6:$B$163,"Character",Assets!$H$6:$H$163,"Validated")</x:f>
-        <x:v>64</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A9,Assets!$B$6:$B$163,"Character",Assets!$I$6:$I$163,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -526,8 +544,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$163,A9)</x:f>
-        <x:v>91</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9)</x:f>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
       <x:c r="J9" s="2"/>
@@ -544,20 +562,25 @@
       <x:c r="C10" s="8" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="D10" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="E10" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="F10" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="G10" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="H10" s="2" t="str">
-        <x:v>Awaiting report</x:v>
+      <x:c r="D10" s="2" t="n">
+        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="n">
+        <x:f>C10-D10</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H10" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
@@ -574,20 +597,25 @@
       <x:c r="C11" s="8" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="D11" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="E11" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="F11" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="G11" s="2" t="str">
-        <x:v>Awaiting report</x:v>
-      </x:c>
-      <x:c r="H11" s="2" t="str">
-        <x:v>Awaiting report</x:v>
+      <x:c r="D11" s="2" t="n">
+        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A11)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="2" t="n">
+        <x:f>C11-D11</x:f>
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H11" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
@@ -627,8 +655,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E163)</x:f>
-        <x:v>85636</x:v>
+        <x:f>SUM(Assets!E6:E189)</x:f>
+        <x:v>179758</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -646,7 +674,7 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B163,"Prop")+COUNTIFS(Assets!B6:B163,"Item")</x:f>
+        <x:f>COUNTIFS(Assets!B6:B189,"Prop")+COUNTIFS(Assets!B6:B189,"Item")</x:f>
         <x:v>59</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
@@ -676,7 +704,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Role counts exclude palette tiers and duplicate dragon growth stages. Gallery/Parcels/Bricks upgrade batches remain queued.</x:v>
+        <x:v>Codex kit only. Refined hero/slime individuals and LODs add exports without new role types.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -719,11 +747,21 @@
       <x:c r="L19" s="2"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="2"/>
-      <x:c r="B20" s="2"/>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2"/>
-      <x:c r="E20" s="2"/>
+      <x:c r="A20" s="21" t="str">
+        <x:v>Approved population</x:v>
+      </x:c>
+      <x:c r="B20" s="21" t="str">
+        <x:v>Target individuals</x:v>
+      </x:c>
+      <x:c r="C20" s="21" t="str">
+        <x:v>Validated candidates</x:v>
+      </x:c>
+      <x:c r="D20" s="21" t="str">
+        <x:v>Play proven</x:v>
+      </x:c>
+      <x:c r="E20" s="21" t="str">
+        <x:v>Remaining art</x:v>
+      </x:c>
       <x:c r="F20" s="2"/>
       <x:c r="G20" s="2"/>
       <x:c r="H20" s="2"/>
@@ -733,11 +771,21 @@
       <x:c r="L20" s="2"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
+      <x:c r="A21" s="2" t="str">
+        <x:v>Enemies</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="n">
+        <x:v>490</x:v>
+      </x:c>
       <x:c r="F21" s="2"/>
       <x:c r="G21" s="2"/>
       <x:c r="H21" s="2"/>
@@ -747,11 +795,21 @@
       <x:c r="L21" s="2"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
+      <x:c r="A22" s="2" t="str">
+        <x:v>Friendlies</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="n">
+        <x:v>500</x:v>
+      </x:c>
       <x:c r="F22" s="2"/>
       <x:c r="G22" s="2"/>
       <x:c r="H22" s="2"/>
@@ -775,7 +833,9 @@
       <x:c r="L23" s="2"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="2"/>
+      <x:c r="A24" s="2" t="str">
+        <x:v>50 types × 10 each per side. Population IDs linked to ten slime candidates. Boss designs are separate proposals.</x:v>
+      </x:c>
       <x:c r="B24" s="2"/>
       <x:c r="C24" s="2"/>
       <x:c r="D24" s="2"/>
@@ -1433,7 +1493,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>Sources: validated Labyrinth/Portal exports and RetroMonster source hash. Art prototypes; Unreal acceptance pending.</x:v>
+        <x:v>Codex export register; excludes other teams. Validation is not visual approval or Play proof. LODs count as exports, not new roles.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1490,6 +1550,12 @@
       <x:c r="N5" s="15" t="str">
         <x:v>Source monster</x:v>
       </x:c>
+      <x:c r="O5" s="19" t="str">
+        <x:v>Population ID</x:v>
+      </x:c>
+      <x:c r="P5" s="19" t="str">
+        <x:v>LOD level</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="2" t="str">
@@ -8325,8 +8391,1308 @@
         <x:v>n.a.</x:v>
       </x:c>
     </x:row>
+    <x:row r="164" ht="38" customHeight="1">
+      <x:c r="A164" s="1" t="str">
+        <x:v>Mob_Gallery_Sketcher</x:v>
+      </x:c>
+      <x:c r="B164" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C164" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D164" s="5" t="str">
+        <x:v>Hero brush and palette</x:v>
+      </x:c>
+      <x:c r="E164" s="7" t="n">
+        <x:v>1040</x:v>
+      </x:c>
+      <x:c r="F164" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G164" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H164" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I164" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J164" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K164" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_Sketcher.glb</x:v>
+      </x:c>
+      <x:c r="L164" s="1" t="str">
+        <x:v>1792bb1f054ecaf3a277be125184bdfe01b1c6fa7a265ab886691ff480cb065b</x:v>
+      </x:c>
+      <x:c r="M164" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N164" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O164" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P164" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="38" customHeight="1">
+      <x:c r="A165" s="1" t="str">
+        <x:v>Mob_Gallery_CuratorVell</x:v>
+      </x:c>
+      <x:c r="B165" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C165" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D165" s="5" t="str">
+        <x:v>Gallery quest presentation</x:v>
+      </x:c>
+      <x:c r="E165" s="7" t="n">
+        <x:v>1408</x:v>
+      </x:c>
+      <x:c r="F165" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G165" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H165" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I165" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J165" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K165" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_CuratorVell.glb</x:v>
+      </x:c>
+      <x:c r="L165" s="1" t="str">
+        <x:v>26655f7f6a3722d583b65d90fb37485a7ff3176621ecdf6f8a5b53f4f5b9666a</x:v>
+      </x:c>
+      <x:c r="M165" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N165" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O165" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P165" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="38" customHeight="1">
+      <x:c r="A166" s="1" t="str">
+        <x:v>Mob_Gallery_FrameHangerTwins</x:v>
+      </x:c>
+      <x:c r="B166" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C166" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D166" s="5" t="str">
+        <x:v>Frame pulley crew role</x:v>
+      </x:c>
+      <x:c r="E166" s="7" t="n">
+        <x:v>1120</x:v>
+      </x:c>
+      <x:c r="F166" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G166" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H166" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I166" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J166" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K166" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_FrameHangerTwins.glb</x:v>
+      </x:c>
+      <x:c r="L166" s="1" t="str">
+        <x:v>9c4baea7ba6e8ca2a327da95a4181f9b4d42ce28a77787859e93fab8ade539ac</x:v>
+      </x:c>
+      <x:c r="M166" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N166" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O166" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P166" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="38" customHeight="1">
+      <x:c r="A167" s="1" t="str">
+        <x:v>Mob_Gallery_VarnishMonk</x:v>
+      </x:c>
+      <x:c r="B167" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C167" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D167" s="5" t="str">
+        <x:v>Painting protection supplies proposal</x:v>
+      </x:c>
+      <x:c r="E167" s="7" t="n">
+        <x:v>920</x:v>
+      </x:c>
+      <x:c r="F167" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G167" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H167" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I167" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J167" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K167" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_VarnishMonk.glb</x:v>
+      </x:c>
+      <x:c r="L167" s="1" t="str">
+        <x:v>8ca2428428c93e844720df47a5db03ce91ac7a238e9a68d2b03cc757a75d5048</x:v>
+      </x:c>
+      <x:c r="M167" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N167" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O167" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P167" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="38" customHeight="1">
+      <x:c r="A168" s="1" t="str">
+        <x:v>Mob_Gallery_RestorerAma</x:v>
+      </x:c>
+      <x:c r="B168" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C168" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D168" s="5" t="str">
+        <x:v>Mural restoration guidance</x:v>
+      </x:c>
+      <x:c r="E168" s="7" t="n">
+        <x:v>928</x:v>
+      </x:c>
+      <x:c r="F168" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G168" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H168" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I168" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J168" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K168" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_RestorerAma.glb</x:v>
+      </x:c>
+      <x:c r="L168" s="1" t="str">
+        <x:v>887f80d5e0e4a8f2ac2d36e04f4ac840a2f9ce2ad190ee980d2fe21a9a44be65</x:v>
+      </x:c>
+      <x:c r="M168" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N168" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O168" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P168" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="38" customHeight="1">
+      <x:c r="A169" s="1" t="str">
+        <x:v>Mob_Gallery_PigmentMiner</x:v>
+      </x:c>
+      <x:c r="B169" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C169" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D169" s="5" t="str">
+        <x:v>Pigment crafting guidance</x:v>
+      </x:c>
+      <x:c r="E169" s="7" t="n">
+        <x:v>928</x:v>
+      </x:c>
+      <x:c r="F169" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G169" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H169" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I169" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J169" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K169" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_PigmentMiner.glb</x:v>
+      </x:c>
+      <x:c r="L169" s="1" t="str">
+        <x:v>86707e4fcfa9b49a19de3693f7c69dff01670bf234503bf19ae7f2ae51404837</x:v>
+      </x:c>
+      <x:c r="M169" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N169" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O169" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P169" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="38" customHeight="1">
+      <x:c r="A170" s="1" t="str">
+        <x:v>Mob_Gallery_GalleryGuard</x:v>
+      </x:c>
+      <x:c r="B170" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C170" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D170" s="5" t="str">
+        <x:v>Gallery access guidance</x:v>
+      </x:c>
+      <x:c r="E170" s="7" t="n">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="F170" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G170" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H170" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I170" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J170" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K170" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_GalleryGuard.glb</x:v>
+      </x:c>
+      <x:c r="L170" s="1" t="str">
+        <x:v>0f28168765ec816655adec39dc767c2e32be18477bc3b71857743c406cfb5c26</x:v>
+      </x:c>
+      <x:c r="M170" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N170" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O170" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P170" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="38" customHeight="1">
+      <x:c r="A171" s="1" t="str">
+        <x:v>Mob_Gallery_StreetMuralist</x:v>
+      </x:c>
+      <x:c r="B171" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C171" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D171" s="5" t="str">
+        <x:v>Painted travel hints proposal</x:v>
+      </x:c>
+      <x:c r="E171" s="7" t="n">
+        <x:v>1040</x:v>
+      </x:c>
+      <x:c r="F171" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G171" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H171" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I171" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J171" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K171" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_StreetMuralist.glb</x:v>
+      </x:c>
+      <x:c r="L171" s="1" t="str">
+        <x:v>7786ec54dec04a5af1128e03f4c9126a09c32ad9bdcf12a15819694e7021b019</x:v>
+      </x:c>
+      <x:c r="M171" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N171" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O171" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P171" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="38" customHeight="1">
+      <x:c r="A172" s="1" t="str">
+        <x:v>Mob_Gallery_LightTailor</x:v>
+      </x:c>
+      <x:c r="B172" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C172" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D172" s="5" t="str">
+        <x:v>Realm cosmetic presentation</x:v>
+      </x:c>
+      <x:c r="E172" s="7" t="n">
+        <x:v>1120</x:v>
+      </x:c>
+      <x:c r="F172" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G172" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H172" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I172" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J172" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K172" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_LightTailor.glb</x:v>
+      </x:c>
+      <x:c r="L172" s="1" t="str">
+        <x:v>e1c319bf62eba64e0991e3f1c7439db85ec1ed98e2af1798bab38a25a659bdaa</x:v>
+      </x:c>
+      <x:c r="M172" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N172" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O172" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P172" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="38" customHeight="1">
+      <x:c r="A173" s="1" t="str">
+        <x:v>Mob_Gallery_DroneMechanicPell</x:v>
+      </x:c>
+      <x:c r="B173" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C173" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D173" s="5" t="str">
+        <x:v>Drone upgrade presentation</x:v>
+      </x:c>
+      <x:c r="E173" s="7" t="n">
+        <x:v>1216</x:v>
+      </x:c>
+      <x:c r="F173" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G173" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H173" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I173" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J173" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K173" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_DroneMechanicPell.glb</x:v>
+      </x:c>
+      <x:c r="L173" s="1" t="str">
+        <x:v>fb6316ec0fc8d5b62ae5cb1f0247df22116c704e0467951ccfceb001ee0fa029</x:v>
+      </x:c>
+      <x:c r="M173" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N173" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O173" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P173" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="38" customHeight="1">
+      <x:c r="A174" s="1" t="str">
+        <x:v>Mob_Gallery_CriticBloom</x:v>
+      </x:c>
+      <x:c r="B174" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C174" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D174" s="5" t="str">
+        <x:v>Build review quest proposal</x:v>
+      </x:c>
+      <x:c r="E174" s="7" t="n">
+        <x:v>936</x:v>
+      </x:c>
+      <x:c r="F174" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G174" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H174" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I174" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J174" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K174" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_CriticBloom.glb</x:v>
+      </x:c>
+      <x:c r="L174" s="1" t="str">
+        <x:v>95b8056c8639e451e66b06914b509fcc5e05851f61d31a2000e5a3549246c2d8</x:v>
+      </x:c>
+      <x:c r="M174" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N174" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O174" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P174" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="38" customHeight="1">
+      <x:c r="A175" s="1" t="str">
+        <x:v>Mob_Gallery_LostSelfPortrait</x:v>
+      </x:c>
+      <x:c r="B175" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C175" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D175" s="5" t="str">
+        <x:v>Missing frame quest proposal</x:v>
+      </x:c>
+      <x:c r="E175" s="7" t="n">
+        <x:v>1068</x:v>
+      </x:c>
+      <x:c r="F175" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G175" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H175" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I175" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J175" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K175" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_LostSelfPortrait.glb</x:v>
+      </x:c>
+      <x:c r="L175" s="1" t="str">
+        <x:v>183555ebd7a6c71f12365b020ebb37f5d34c794d915319d17ce4780a137d1b28</x:v>
+      </x:c>
+      <x:c r="M175" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N175" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O175" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P175" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="38" customHeight="1">
+      <x:c r="A176" s="1" t="str">
+        <x:v>Mob_Gallery_EchoChoir</x:v>
+      </x:c>
+      <x:c r="B176" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C176" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D176" s="5" t="str">
+        <x:v>Touring jukebox district cue proposal</x:v>
+      </x:c>
+      <x:c r="E176" s="7" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="F176" s="1" t="str">
+        <x:v>GalleryHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G176" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H176" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I176" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J176" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K176" s="1" t="str">
+        <x:v>gallery-buildout/cast/Mob_Gallery_EchoChoir.glb</x:v>
+      </x:c>
+      <x:c r="L176" s="1" t="str">
+        <x:v>0af6afef337936078e5776445ac3650b922912e62857ce3b3399d75b6196e9aa</x:v>
+      </x:c>
+      <x:c r="M176" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N176" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O176" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P176" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="38" customHeight="1">
+      <x:c r="A177" s="1" t="str">
+        <x:v>Mob_Portal_Knight_Polish</x:v>
+      </x:c>
+      <x:c r="B177" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C177" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D177" s="5" t="str">
+        <x:v>Hero polish review; existing knight rules</x:v>
+      </x:c>
+      <x:c r="E177" s="7" t="n">
+        <x:v>14252</x:v>
+      </x:c>
+      <x:c r="F177" s="1" t="str">
+        <x:v>PortalHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G177" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H177" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I177" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J177" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K177" s="1" t="str">
+        <x:v>portal-hero-polish/Mob_Portal_Knight_Polish.glb</x:v>
+      </x:c>
+      <x:c r="L177" s="1" t="str">
+        <x:v>bfa2f8479888a683d46e3d62ff145cb37072fe02c90241e3a9052050c2709c29</x:v>
+      </x:c>
+      <x:c r="M177" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N177" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O177" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P177" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="38" customHeight="1">
+      <x:c r="A178" s="1" t="str">
+        <x:v>Mob_Portal_Knight_Polish_LOD1</x:v>
+      </x:c>
+      <x:c r="B178" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C178" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D178" s="5" t="str">
+        <x:v>Hero visual LOD; same existing role</x:v>
+      </x:c>
+      <x:c r="E178" s="7" t="n">
+        <x:v>4988</x:v>
+      </x:c>
+      <x:c r="F178" s="1" t="str">
+        <x:v>PortalHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G178" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H178" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I178" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J178" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K178" s="1" t="str">
+        <x:v>portal-hero-lods/Mob_Portal_Knight_Polish_LOD1.glb</x:v>
+      </x:c>
+      <x:c r="L178" s="1" t="str">
+        <x:v>75632474a90a5775d8430b42db62f3139863d8fd36e4ad0422c6e1e9e87266ad</x:v>
+      </x:c>
+      <x:c r="M178" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N178" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O178" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P178" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="38" customHeight="1">
+      <x:c r="A179" s="1" t="str">
+        <x:v>Mob_Portal_Knight_Polish_LOD2</x:v>
+      </x:c>
+      <x:c r="B179" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C179" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D179" s="5" t="str">
+        <x:v>Hero visual LOD; same existing role</x:v>
+      </x:c>
+      <x:c r="E179" s="7" t="n">
+        <x:v>1706</x:v>
+      </x:c>
+      <x:c r="F179" s="1" t="str">
+        <x:v>PortalHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G179" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H179" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I179" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J179" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K179" s="1" t="str">
+        <x:v>portal-hero-lods/Mob_Portal_Knight_Polish_LOD2.glb</x:v>
+      </x:c>
+      <x:c r="L179" s="1" t="str">
+        <x:v>51bb21340145ae8a877250d4a0fcdf284b209e394e46da984aa06dc8adfa692b</x:v>
+      </x:c>
+      <x:c r="M179" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N179" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O179" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P179" s="1" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="38" customHeight="1">
+      <x:c r="A180" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_01</x:v>
+      </x:c>
+      <x:c r="B180" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C180" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D180" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E180" s="7" t="n">
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="F180" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G180" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H180" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I180" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J180" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K180" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_01.glb</x:v>
+      </x:c>
+      <x:c r="L180" s="1" t="str">
+        <x:v>5976d65cc6ad0bffe08a5cdb64a41adfa0e0cd3232ce72216b2c99705381c972</x:v>
+      </x:c>
+      <x:c r="M180" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N180" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O180" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_01</x:v>
+      </x:c>
+      <x:c r="P180" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="38" customHeight="1">
+      <x:c r="A181" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_02</x:v>
+      </x:c>
+      <x:c r="B181" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C181" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D181" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E181" s="7" t="n">
+        <x:v>5928</x:v>
+      </x:c>
+      <x:c r="F181" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G181" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H181" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I181" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J181" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K181" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_02.glb</x:v>
+      </x:c>
+      <x:c r="L181" s="1" t="str">
+        <x:v>78b7e9b3950acaded07cc7a2225286b2e14e710471f3fda7764d7fb73c054fe2</x:v>
+      </x:c>
+      <x:c r="M181" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N181" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O181" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_02</x:v>
+      </x:c>
+      <x:c r="P181" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="38" customHeight="1">
+      <x:c r="A182" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_03</x:v>
+      </x:c>
+      <x:c r="B182" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C182" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D182" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E182" s="7" t="n">
+        <x:v>5948</x:v>
+      </x:c>
+      <x:c r="F182" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G182" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H182" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I182" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J182" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K182" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_03.glb</x:v>
+      </x:c>
+      <x:c r="L182" s="1" t="str">
+        <x:v>8a15302a21e37852f071095ff31100f518cec5a718b3d0da786748a538fe9801</x:v>
+      </x:c>
+      <x:c r="M182" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N182" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O182" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_03</x:v>
+      </x:c>
+      <x:c r="P182" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="38" customHeight="1">
+      <x:c r="A183" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_04</x:v>
+      </x:c>
+      <x:c r="B183" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C183" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D183" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E183" s="7" t="n">
+        <x:v>5968</x:v>
+      </x:c>
+      <x:c r="F183" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G183" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H183" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I183" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J183" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K183" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_04.glb</x:v>
+      </x:c>
+      <x:c r="L183" s="1" t="str">
+        <x:v>dd3bd1f681454a5e05570345391290bc698ce06d063ab2c1556d3eeabcf807c0</x:v>
+      </x:c>
+      <x:c r="M183" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N183" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O183" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_04</x:v>
+      </x:c>
+      <x:c r="P183" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="38" customHeight="1">
+      <x:c r="A184" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_05</x:v>
+      </x:c>
+      <x:c r="B184" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C184" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D184" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E184" s="7" t="n">
+        <x:v>5988</x:v>
+      </x:c>
+      <x:c r="F184" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G184" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H184" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I184" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J184" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K184" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_05.glb</x:v>
+      </x:c>
+      <x:c r="L184" s="1" t="str">
+        <x:v>5824ddc6eb3d9088107be33b76221e18d7021e38872bf7223bf80cd4ee4e83b1</x:v>
+      </x:c>
+      <x:c r="M184" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N184" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O184" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_05</x:v>
+      </x:c>
+      <x:c r="P184" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="38" customHeight="1">
+      <x:c r="A185" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_06</x:v>
+      </x:c>
+      <x:c r="B185" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C185" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D185" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E185" s="7" t="n">
+        <x:v>5908</x:v>
+      </x:c>
+      <x:c r="F185" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G185" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H185" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I185" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J185" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K185" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_06.glb</x:v>
+      </x:c>
+      <x:c r="L185" s="1" t="str">
+        <x:v>a21bd14270587f96afb59193bd3deae46d14431f841b8d17b3cdabdaa2fd94ce</x:v>
+      </x:c>
+      <x:c r="M185" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N185" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O185" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_06</x:v>
+      </x:c>
+      <x:c r="P185" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="38" customHeight="1">
+      <x:c r="A186" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_07</x:v>
+      </x:c>
+      <x:c r="B186" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C186" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D186" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E186" s="7" t="n">
+        <x:v>5928</x:v>
+      </x:c>
+      <x:c r="F186" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G186" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H186" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I186" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J186" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K186" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_07.glb</x:v>
+      </x:c>
+      <x:c r="L186" s="1" t="str">
+        <x:v>dcc07fe1ca260fd7274f767c873cb84dbc7d07e09ab2ee011f2cb2b4476c214c</x:v>
+      </x:c>
+      <x:c r="M186" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N186" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O186" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_07</x:v>
+      </x:c>
+      <x:c r="P186" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="38" customHeight="1">
+      <x:c r="A187" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_08</x:v>
+      </x:c>
+      <x:c r="B187" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C187" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D187" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E187" s="7" t="n">
+        <x:v>5948</x:v>
+      </x:c>
+      <x:c r="F187" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G187" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H187" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I187" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J187" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K187" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_08.glb</x:v>
+      </x:c>
+      <x:c r="L187" s="1" t="str">
+        <x:v>5528a9f3cf8706f6adbaa9b2c6d29f09887eb3c2209e08923e5b89fabe11da2a</x:v>
+      </x:c>
+      <x:c r="M187" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N187" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O187" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_08</x:v>
+      </x:c>
+      <x:c r="P187" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="38" customHeight="1">
+      <x:c r="A188" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_09</x:v>
+      </x:c>
+      <x:c r="B188" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C188" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D188" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E188" s="7" t="n">
+        <x:v>5968</x:v>
+      </x:c>
+      <x:c r="F188" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G188" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H188" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I188" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J188" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K188" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_09.glb</x:v>
+      </x:c>
+      <x:c r="L188" s="1" t="str">
+        <x:v>03ed035dfdf5ec0ad1273b7127ed05864dc177fd691c560fdf0e522b0d1204b5</x:v>
+      </x:c>
+      <x:c r="M188" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N188" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O188" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_09</x:v>
+      </x:c>
+      <x:c r="P188" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="38" customHeight="1">
+      <x:c r="A189" s="1" t="str">
+        <x:v>Mob_Portal_BLIGHT_SLIME_Polish_10</x:v>
+      </x:c>
+      <x:c r="B189" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C189" s="1" t="str">
+        <x:v>Portal Realm</x:v>
+      </x:c>
+      <x:c r="D189" s="5" t="str">
+        <x:v>Existing Blight Slime encounter visual</x:v>
+      </x:c>
+      <x:c r="E189" s="7" t="n">
+        <x:v>5988</x:v>
+      </x:c>
+      <x:c r="F189" s="1" t="str">
+        <x:v>PortalCreatureV1</x:v>
+      </x:c>
+      <x:c r="G189" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H189" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I189" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J189" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K189" s="1" t="str">
+        <x:v>portal-slime-polish/Mob_Portal_BLIGHT_SLIME_Polish_10.glb</x:v>
+      </x:c>
+      <x:c r="L189" s="1" t="str">
+        <x:v>0646f6c8ad458b2ec9079cb31a683c0d660cc3eca1933d1fd078086047e22ac5</x:v>
+      </x:c>
+      <x:c r="M189" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N189" s="1" t="str">
+        <x:v>BLIGHT_SLIME</x:v>
+      </x:c>
+      <x:c r="O189" s="1" t="str">
+        <x:v>Portal_enemy_BLIGHT_SLIME_10</x:v>
+      </x:c>
+      <x:c r="P189" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="6">
     <x:dataValidation type="list" sqref="I6:I72">
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
@@ -8337,6 +9703,12 @@
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J73:J163">
+      <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I164:I189">
+      <x:formula1>"Pending,Imported,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J164:J189">
       <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -8895,12 +10267,22 @@
       <x:c r="K24" s="2"/>
       <x:c r="L24" s="2"/>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="2"/>
-      <x:c r="B25" s="2"/>
-      <x:c r="C25" s="2"/>
-      <x:c r="D25" s="2"/>
-      <x:c r="E25" s="2"/>
+    <x:row r="25" ht="52" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>PORT09</x:v>
+      </x:c>
+      <x:c r="B25" s="4" t="str">
+        <x:v>Kings favours, rescues, unicorn requests</x:v>
+      </x:c>
+      <x:c r="C25" s="4" t="str">
+        <x:v>Ordered quest core</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="str">
+        <x:v>Core tested; persistence and rewards pending</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="str">
+        <x:v>Royal roads connect rescued towns and helpful herds</x:v>
+      </x:c>
       <x:c r="F25" s="2"/>
       <x:c r="G25" s="2"/>
       <x:c r="H25" s="2"/>
@@ -8909,12 +10291,22 @@
       <x:c r="K25" s="2"/>
       <x:c r="L25" s="2"/>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="2"/>
-      <x:c r="B26" s="2"/>
-      <x:c r="C26" s="2"/>
-      <x:c r="D26" s="2"/>
-      <x:c r="E26" s="2"/>
+    <x:row r="26" ht="52" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>PORT10</x:v>
+      </x:c>
+      <x:c r="B26" s="4" t="str">
+        <x:v>Additive 3D battle presentation</x:v>
+      </x:c>
+      <x:c r="C26" s="4" t="str">
+        <x:v>Battle director + presentation actor</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="str">
+        <x:v>Isolated UE compile/link; live binding pending</x:v>
+      </x:c>
+      <x:c r="E26" s="4" t="str">
+        <x:v>Preserve classic rules and improve expressive battles</x:v>
+      </x:c>
       <x:c r="F26" s="2"/>
       <x:c r="G26" s="2"/>
       <x:c r="H26" s="2"/>
@@ -8923,12 +10315,22 @@
       <x:c r="K26" s="2"/>
       <x:c r="L26" s="2"/>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="2"/>
-      <x:c r="B27" s="2"/>
-      <x:c r="C27" s="2"/>
-      <x:c r="D27" s="2"/>
-      <x:c r="E27" s="2"/>
+    <x:row r="27" ht="52" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>PORT11</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="str">
+        <x:v>Hero/slime polish and hero detail levels</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="str">
+        <x:v>Hero + 10 slimes + 2 reduced exports</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="str">
+        <x:v>Exports validated; visual/native acceptance pending</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>Distinct silhouettes retain the raw realm identity</x:v>
+      </x:c>
       <x:c r="F27" s="2"/>
       <x:c r="G27" s="2"/>
       <x:c r="H27" s="2"/>
@@ -8937,12 +10339,22 @@
       <x:c r="K27" s="2"/>
       <x:c r="L27" s="2"/>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="2"/>
-      <x:c r="B28" s="2"/>
-      <x:c r="C28" s="2"/>
-      <x:c r="D28" s="2"/>
-      <x:c r="E28" s="2"/>
+    <x:row r="28" ht="52" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>PORT12</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="str">
+        <x:v>Dragon egg and configured land annotations</x:v>
+      </x:c>
+      <x:c r="C28" s="4" t="str">
+        <x:v>Java egg + DRR codec parity</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="str">
+        <x:v>Targeted Java parity tested; ownership authority pending</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="str">
+        <x:v>Native drake semantics preserved without demo deed authority</x:v>
+      </x:c>
       <x:c r="F28" s="2"/>
       <x:c r="G28" s="2"/>
       <x:c r="H28" s="2"/>
@@ -8951,12 +10363,22 @@
       <x:c r="K28" s="2"/>
       <x:c r="L28" s="2"/>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="2"/>
-      <x:c r="B29" s="2"/>
-      <x:c r="C29" s="2"/>
-      <x:c r="D29" s="2"/>
-      <x:c r="E29" s="2"/>
+    <x:row r="29" ht="52" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>SEA01</x:v>
+      </x:c>
+      <x:c r="B29" s="4" t="str">
+        <x:v>Boats/submarines enter ocean; shores return; underwater docks connect worlds</x:v>
+      </x:c>
+      <x:c r="C29" s="4" t="str">
+        <x:v>Dock route core</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="str">
+        <x:v>Core tested; vessels/live transitions pending</x:v>
+      </x:c>
+      <x:c r="E29" s="4" t="str">
+        <x:v>Explore sea routes and drowned settlements</x:v>
+      </x:c>
       <x:c r="F29" s="2"/>
       <x:c r="G29" s="2"/>
       <x:c r="H29" s="2"/>
@@ -8965,12 +10387,22 @@
       <x:c r="K29" s="2"/>
       <x:c r="L29" s="2"/>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
+    <x:row r="30" ht="52" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>LAND01</x:v>
+      </x:c>
+      <x:c r="B30" s="4" t="str">
+        <x:v>Long prairie range and submerged seabed</x:v>
+      </x:c>
+      <x:c r="C30" s="4" t="str">
+        <x:v>Terrain core + native actor</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="str">
+        <x:v>Isolated UE compile/link; placement pending</x:v>
+      </x:c>
+      <x:c r="E30" s="4" t="str">
+        <x:v>Buffalo ranges, travel corridors and ocean exploration</x:v>
+      </x:c>
       <x:c r="F30" s="2"/>
       <x:c r="G30" s="2"/>
       <x:c r="H30" s="2"/>
@@ -8979,12 +10411,22 @@
       <x:c r="K30" s="2"/>
       <x:c r="L30" s="2"/>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
+    <x:row r="31" ht="52" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>CAST01</x:v>
+      </x:c>
+      <x:c r="B31" s="4" t="str">
+        <x:v>50 enemy and 50 friendly types, 10 each</x:v>
+      </x:c>
+      <x:c r="C31" s="4" t="str">
+        <x:v>1000 individual production IDs</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="str">
+        <x:v>10 enemy candidates validated; others planned</x:v>
+      </x:c>
+      <x:c r="E31" s="4" t="str">
+        <x:v>Kings, rescues and unicorn biddings drive the cast</x:v>
+      </x:c>
       <x:c r="F31" s="2"/>
       <x:c r="G31" s="2"/>
       <x:c r="H31" s="2"/>

</xml_diff>

<commit_message>
Complete Gallery modular art kit and reconcile production register
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R9651bb0dff654338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R4c15516a8a3244e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R4e2265908d894948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Raadceb366b584e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R125713e2e28c4d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Ra0e1ac36088244e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,15 +458,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -474,7 +474,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -493,24 +493,24 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A8)</x:f>
-        <x:v>13</x:v>
+        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A8)</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="2" t="n">
         <x:f>C8-D8</x:f>
-        <x:v>19</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A8)</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
@@ -528,15 +528,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -544,7 +544,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A9)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9)</x:f>
         <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
@@ -563,15 +563,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A10)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="2" t="n">
@@ -579,7 +579,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A10)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
@@ -598,15 +598,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$189,Assets!$C$6:$C$189,A11)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11,Assets!$B$6:$B$189,"Character",Assets!$H$6:$H$189,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11,Assets!$B$6:$B$189,"Character",Assets!$I$6:$I$189,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="2" t="n">
@@ -614,7 +614,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$189,A11)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
@@ -655,8 +655,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E189)</x:f>
-        <x:v>179758</x:v>
+        <x:f>SUM(Assets!E6:E232)</x:f>
+        <x:v>217522</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -674,8 +674,8 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B189,"Prop")+COUNTIFS(Assets!B6:B189,"Item")</x:f>
-        <x:v>59</x:v>
+        <x:f>COUNTIFS(Assets!B6:B232,"Prop")+COUNTIFS(Assets!B6:B232,"Item")</x:f>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -704,7 +704,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Codex kit only. Refined hero/slime individuals and LODs add exports without new role types.</x:v>
+        <x:v>Codex first kits only. Gallery 56 exports; native behaviors/visual acceptance pending. LODs are not new roles.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -9691,8 +9691,2110 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="190" ht="38" customHeight="1">
+      <x:c r="A190" s="1" t="str">
+        <x:v>Mob_Gallery_Smudgeling</x:v>
+      </x:c>
+      <x:c r="B190" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C190" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D190" s="5" t="str">
+        <x:v>Ink creature</x:v>
+      </x:c>
+      <x:c r="E190" s="7" t="n">
+        <x:v>1792</x:v>
+      </x:c>
+      <x:c r="F190" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G190" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H190" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I190" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J190" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K190" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_Smudgeling.glb</x:v>
+      </x:c>
+      <x:c r="L190" s="1" t="str">
+        <x:v>5c9890d264e41ead8fa2384a6c96c60c59ee27be1443167405325b36e5a3e370</x:v>
+      </x:c>
+      <x:c r="M190" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N190" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O190" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P190" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="38" customHeight="1">
+      <x:c r="A191" s="1" t="str">
+        <x:v>Mob_Gallery_ThumbtackBeetle</x:v>
+      </x:c>
+      <x:c r="B191" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C191" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D191" s="5" t="str">
+        <x:v>Metal beetle</x:v>
+      </x:c>
+      <x:c r="E191" s="7" t="n">
+        <x:v>1788</x:v>
+      </x:c>
+      <x:c r="F191" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G191" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H191" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I191" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J191" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K191" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_ThumbtackBeetle.glb</x:v>
+      </x:c>
+      <x:c r="L191" s="1" t="str">
+        <x:v>f9879366ec38a649ddbed13a51a560f1806b9755e7112f05dba1c6b891bcdd7c</x:v>
+      </x:c>
+      <x:c r="M191" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N191" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O191" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P191" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="38" customHeight="1">
+      <x:c r="A192" s="1" t="str">
+        <x:v>Mob_Gallery_CanvasMoth</x:v>
+      </x:c>
+      <x:c r="B192" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C192" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D192" s="5" t="str">
+        <x:v>Canvas-wing creature</x:v>
+      </x:c>
+      <x:c r="E192" s="7" t="n">
+        <x:v>1916</x:v>
+      </x:c>
+      <x:c r="F192" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G192" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H192" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I192" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J192" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K192" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_CanvasMoth.glb</x:v>
+      </x:c>
+      <x:c r="L192" s="1" t="str">
+        <x:v>da33e970963d79b640564567bc471e56f3067471bfac778e64825bef1804d3d6</x:v>
+      </x:c>
+      <x:c r="M192" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N192" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O192" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P192" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="38" customHeight="1">
+      <x:c r="A193" s="1" t="str">
+        <x:v>Mob_Gallery_EaselStrider</x:v>
+      </x:c>
+      <x:c r="B193" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C193" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D193" s="5" t="str">
+        <x:v>Tripod creature</x:v>
+      </x:c>
+      <x:c r="E193" s="7" t="n">
+        <x:v>1048</x:v>
+      </x:c>
+      <x:c r="F193" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G193" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H193" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I193" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J193" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K193" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_EaselStrider.glb</x:v>
+      </x:c>
+      <x:c r="L193" s="1" t="str">
+        <x:v>00766cd978ba3445e0e3094cc77e6b4aa75c9873a814b8e9107be230e1c5dcc7</x:v>
+      </x:c>
+      <x:c r="M193" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N193" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O193" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P193" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="38" customHeight="1">
+      <x:c r="A194" s="1" t="str">
+        <x:v>Mob_Gallery_TurpentineToad</x:v>
+      </x:c>
+      <x:c r="B194" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C194" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D194" s="5" t="str">
+        <x:v>Toad creature</x:v>
+      </x:c>
+      <x:c r="E194" s="7" t="n">
+        <x:v>2232</x:v>
+      </x:c>
+      <x:c r="F194" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G194" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H194" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I194" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J194" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K194" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_TurpentineToad.glb</x:v>
+      </x:c>
+      <x:c r="L194" s="1" t="str">
+        <x:v>6e43b9f72852041df1b74dd583f857fef7c31711f53dd726293de7b481dbf7bd</x:v>
+      </x:c>
+      <x:c r="M194" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N194" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O194" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P194" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="38" customHeight="1">
+      <x:c r="A195" s="1" t="str">
+        <x:v>Mob_Gallery_MosaicHound</x:v>
+      </x:c>
+      <x:c r="B195" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C195" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D195" s="5" t="str">
+        <x:v>Tile hound</x:v>
+      </x:c>
+      <x:c r="E195" s="7" t="n">
+        <x:v>1788</x:v>
+      </x:c>
+      <x:c r="F195" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G195" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H195" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I195" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J195" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K195" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_MosaicHound.glb</x:v>
+      </x:c>
+      <x:c r="L195" s="1" t="str">
+        <x:v>865a2c47cf36f5fce326b7e2a0db990aa734342827a95040f51a1b3611ed0d6c</x:v>
+      </x:c>
+      <x:c r="M195" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N195" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O195" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P195" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="38" customHeight="1">
+      <x:c r="A196" s="1" t="str">
+        <x:v>Mob_Gallery_GildedFrameMimic</x:v>
+      </x:c>
+      <x:c r="B196" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C196" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D196" s="5" t="str">
+        <x:v>Living frame creature</x:v>
+      </x:c>
+      <x:c r="E196" s="7" t="n">
+        <x:v>1296</x:v>
+      </x:c>
+      <x:c r="F196" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G196" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H196" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I196" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J196" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K196" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_GildedFrameMimic.glb</x:v>
+      </x:c>
+      <x:c r="L196" s="1" t="str">
+        <x:v>ae02b5dd46ef21d397b175f2b371bf3dfcac77f4bf90e5021e909ee6c1a9cdb2</x:v>
+      </x:c>
+      <x:c r="M196" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N196" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O196" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P196" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="38" customHeight="1">
+      <x:c r="A197" s="1" t="str">
+        <x:v>Mob_Gallery_SentinelBust</x:v>
+      </x:c>
+      <x:c r="B197" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C197" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D197" s="5" t="str">
+        <x:v>Marble sentinel</x:v>
+      </x:c>
+      <x:c r="E197" s="7" t="n">
+        <x:v>2284</x:v>
+      </x:c>
+      <x:c r="F197" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G197" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H197" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I197" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J197" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K197" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_SentinelBust.glb</x:v>
+      </x:c>
+      <x:c r="L197" s="1" t="str">
+        <x:v>364e2856aca5677ba421415b771ab2be005145fb6aa362f4945306e462e027fe</x:v>
+      </x:c>
+      <x:c r="M197" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N197" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O197" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P197" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="38" customHeight="1">
+      <x:c r="A198" s="1" t="str">
+        <x:v>Mob_Gallery_LightProjection</x:v>
+      </x:c>
+      <x:c r="B198" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C198" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D198" s="5" t="str">
+        <x:v>Colour construct; replaces spooky wraith proposal</x:v>
+      </x:c>
+      <x:c r="E198" s="7" t="n">
+        <x:v>1094</x:v>
+      </x:c>
+      <x:c r="F198" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G198" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H198" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I198" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J198" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K198" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_LightProjection.glb</x:v>
+      </x:c>
+      <x:c r="L198" s="1" t="str">
+        <x:v>3dc0582f65739454caba05f6a894a125be692b63bf1dda185a118cdbe96ccae2</x:v>
+      </x:c>
+      <x:c r="M198" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N198" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O198" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P198" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="38" customHeight="1">
+      <x:c r="A199" s="1" t="str">
+        <x:v>Mob_Gallery_GreyWash</x:v>
+      </x:c>
+      <x:c r="B199" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C199" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D199" s="5" t="str">
+        <x:v>Colour-draining boss proposal</x:v>
+      </x:c>
+      <x:c r="E199" s="7" t="n">
+        <x:v>2688</x:v>
+      </x:c>
+      <x:c r="F199" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G199" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H199" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I199" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J199" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K199" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_GreyWash.glb</x:v>
+      </x:c>
+      <x:c r="L199" s="1" t="str">
+        <x:v>b9d62c02824c01b9cec55b5798884d7172fa0720655c1adfe9fb8ef95b4dfef2</x:v>
+      </x:c>
+      <x:c r="M199" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N199" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O199" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P199" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="38" customHeight="1">
+      <x:c r="A200" s="1" t="str">
+        <x:v>Mob_Gallery_PaperCrane</x:v>
+      </x:c>
+      <x:c r="B200" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C200" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D200" s="5" t="str">
+        <x:v>Ambient origami bird</x:v>
+      </x:c>
+      <x:c r="E200" s="7" t="n">
+        <x:v>1504</x:v>
+      </x:c>
+      <x:c r="F200" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G200" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H200" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I200" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J200" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K200" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_PaperCrane.glb</x:v>
+      </x:c>
+      <x:c r="L200" s="1" t="str">
+        <x:v>38c8b6eccee1d0aa7d0043f370f00c7fcc4d077dedefb9a500897600af734423</x:v>
+      </x:c>
+      <x:c r="M200" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N200" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O200" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P200" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="38" customHeight="1">
+      <x:c r="A201" s="1" t="str">
+        <x:v>Mob_Gallery_BrushtailSquirrel</x:v>
+      </x:c>
+      <x:c r="B201" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C201" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D201" s="5" t="str">
+        <x:v>Ambient brush-tailed animal</x:v>
+      </x:c>
+      <x:c r="E201" s="7" t="n">
+        <x:v>1616</x:v>
+      </x:c>
+      <x:c r="F201" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G201" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H201" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I201" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J201" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K201" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_BrushtailSquirrel.glb</x:v>
+      </x:c>
+      <x:c r="L201" s="1" t="str">
+        <x:v>9577e76109873fc3475ed8a86a4e36e164f187f7178695f126019c224ba08903</x:v>
+      </x:c>
+      <x:c r="M201" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N201" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O201" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P201" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="38" customHeight="1">
+      <x:c r="A202" s="1" t="str">
+        <x:v>Mob_Gallery_GalleryDrone</x:v>
+      </x:c>
+      <x:c r="B202" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C202" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D202" s="5" t="str">
+        <x:v>Realm mount; flight pending</x:v>
+      </x:c>
+      <x:c r="E202" s="7" t="n">
+        <x:v>1272</x:v>
+      </x:c>
+      <x:c r="F202" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G202" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H202" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I202" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J202" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K202" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_GalleryDrone.glb</x:v>
+      </x:c>
+      <x:c r="L202" s="1" t="str">
+        <x:v>490d1de4a25460846816441dd866036f7f018585824bbedcba00f10edb595fe1</x:v>
+      </x:c>
+      <x:c r="M202" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N202" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O202" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P202" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="38" customHeight="1">
+      <x:c r="A203" s="1" t="str">
+        <x:v>Mob_Gallery_KiteRay</x:v>
+      </x:c>
+      <x:c r="B203" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C203" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D203" s="5" t="str">
+        <x:v>Gliding companion</x:v>
+      </x:c>
+      <x:c r="E203" s="7" t="n">
+        <x:v>1476</x:v>
+      </x:c>
+      <x:c r="F203" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G203" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H203" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I203" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J203" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K203" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_KiteRay.glb</x:v>
+      </x:c>
+      <x:c r="L203" s="1" t="str">
+        <x:v>78bcc541f27646e0917fb1411b60ef7640dcb765f81408147ad5e5cfbf98701a</x:v>
+      </x:c>
+      <x:c r="M203" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N203" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O203" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P203" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="38" customHeight="1">
+      <x:c r="A204" s="1" t="str">
+        <x:v>Mob_Gallery_EaselMule</x:v>
+      </x:c>
+      <x:c r="B204" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C204" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D204" s="5" t="str">
+        <x:v>Pack companion</x:v>
+      </x:c>
+      <x:c r="E204" s="7" t="n">
+        <x:v>1480</x:v>
+      </x:c>
+      <x:c r="F204" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G204" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H204" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I204" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J204" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K204" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_EaselMule.glb</x:v>
+      </x:c>
+      <x:c r="L204" s="1" t="str">
+        <x:v>8eaf9937c50d8639e0de49bbb04ab90266a7a06180602621563058ee45eb0461</x:v>
+      </x:c>
+      <x:c r="M204" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N204" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O204" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P204" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="38" customHeight="1">
+      <x:c r="A205" s="1" t="str">
+        <x:v>Mob_Gallery_Inkpup</x:v>
+      </x:c>
+      <x:c r="B205" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C205" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D205" s="5" t="str">
+        <x:v>Friendly pet</x:v>
+      </x:c>
+      <x:c r="E205" s="7" t="n">
+        <x:v>1616</x:v>
+      </x:c>
+      <x:c r="F205" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G205" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H205" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I205" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J205" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K205" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_Inkpup.glb</x:v>
+      </x:c>
+      <x:c r="L205" s="1" t="str">
+        <x:v>95238d1ccb69ca58b82739a97af5eba416ce8d94fdb6c0bab6cc055656a33619</x:v>
+      </x:c>
+      <x:c r="M205" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N205" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O205" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P205" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="38" customHeight="1">
+      <x:c r="A206" s="1" t="str">
+        <x:v>Mob_Gallery_PrismFinch</x:v>
+      </x:c>
+      <x:c r="B206" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C206" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D206" s="5" t="str">
+        <x:v>Friendly pet</x:v>
+      </x:c>
+      <x:c r="E206" s="7" t="n">
+        <x:v>1474</x:v>
+      </x:c>
+      <x:c r="F206" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G206" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H206" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I206" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J206" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K206" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_PrismFinch.glb</x:v>
+      </x:c>
+      <x:c r="L206" s="1" t="str">
+        <x:v>09d0900bf54aa64fffaaf027bfb934f8d6db99b3301f8778c2d00141f3384781</x:v>
+      </x:c>
+      <x:c r="M206" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N206" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O206" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P206" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="38" customHeight="1">
+      <x:c r="A207" s="1" t="str">
+        <x:v>Mob_Gallery_CrayonGecko</x:v>
+      </x:c>
+      <x:c r="B207" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C207" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D207" s="5" t="str">
+        <x:v>Friendly pet</x:v>
+      </x:c>
+      <x:c r="E207" s="7" t="n">
+        <x:v>1416</x:v>
+      </x:c>
+      <x:c r="F207" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G207" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H207" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I207" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J207" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K207" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_CrayonGecko.glb</x:v>
+      </x:c>
+      <x:c r="L207" s="1" t="str">
+        <x:v>0ab21f5e561c845a15c26e38f0e303202a17b17df091e90a12ed36b5e55074ca</x:v>
+      </x:c>
+      <x:c r="M207" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N207" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O207" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P207" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="38" customHeight="1">
+      <x:c r="A208" s="1" t="str">
+        <x:v>Mob_Gallery_LampMoth</x:v>
+      </x:c>
+      <x:c r="B208" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C208" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D208" s="5" t="str">
+        <x:v>Friendly pet</x:v>
+      </x:c>
+      <x:c r="E208" s="7" t="n">
+        <x:v>2332</x:v>
+      </x:c>
+      <x:c r="F208" s="1" t="str">
+        <x:v>GalleryCreatureV1</x:v>
+      </x:c>
+      <x:c r="G208" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H208" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I208" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J208" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K208" s="1" t="str">
+        <x:v>gallery-buildout/creatures/Mob_Gallery_LampMoth.glb</x:v>
+      </x:c>
+      <x:c r="L208" s="1" t="str">
+        <x:v>e695dde4c6417c8abdc9a1bc3d996eadbe8c9a2ad1bbfc1ebdf9033299ded09a</x:v>
+      </x:c>
+      <x:c r="M208" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N208" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O208" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P208" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="38" customHeight="1">
+      <x:c r="A209" s="1" t="str">
+        <x:v>Prop_Gallery_FloorTile</x:v>
+      </x:c>
+      <x:c r="B209" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C209" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D209" s="5" t="str">
+        <x:v>Walkable floor module</x:v>
+      </x:c>
+      <x:c r="E209" s="7" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F209" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G209" s="5" t="str"/>
+      <x:c r="H209" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I209" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J209" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K209" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_FloorTile.glb</x:v>
+      </x:c>
+      <x:c r="L209" s="1" t="str">
+        <x:v>0d8a4d33c41589bca58342d9481326381c1b2f78a8a0c995cb1a1a3d101abf80</x:v>
+      </x:c>
+      <x:c r="M209" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N209" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O209" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P209" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="38" customHeight="1">
+      <x:c r="A210" s="1" t="str">
+        <x:v>Prop_Gallery_MosaicFloor</x:v>
+      </x:c>
+      <x:c r="B210" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C210" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D210" s="5" t="str">
+        <x:v>Colour tile floor</x:v>
+      </x:c>
+      <x:c r="E210" s="7" t="n">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="F210" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G210" s="5" t="str"/>
+      <x:c r="H210" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I210" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J210" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K210" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_MosaicFloor.glb</x:v>
+      </x:c>
+      <x:c r="L210" s="1" t="str">
+        <x:v>b0c176031f9b282815166ce4f2c4b7a74fb553da62c1c94bba7a86417a66cfee</x:v>
+      </x:c>
+      <x:c r="M210" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N210" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O210" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P210" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="38" customHeight="1">
+      <x:c r="A211" s="1" t="str">
+        <x:v>Prop_Gallery_Walkway</x:v>
+      </x:c>
+      <x:c r="B211" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C211" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D211" s="5" t="str">
+        <x:v>Hanging walkway</x:v>
+      </x:c>
+      <x:c r="E211" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F211" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G211" s="5" t="str"/>
+      <x:c r="H211" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I211" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J211" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K211" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_Walkway.glb</x:v>
+      </x:c>
+      <x:c r="L211" s="1" t="str">
+        <x:v>dafbaae399a08c8852a7357fab5043696c48e5111a9fd21ffb71a8682a398a73</x:v>
+      </x:c>
+      <x:c r="M211" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N211" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O211" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P211" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="38" customHeight="1">
+      <x:c r="A212" s="1" t="str">
+        <x:v>Prop_Gallery_FrameWall</x:v>
+      </x:c>
+      <x:c r="B212" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C212" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D212" s="5" t="str">
+        <x:v>Modular framed wall</x:v>
+      </x:c>
+      <x:c r="E212" s="7" t="n">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="F212" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G212" s="5" t="str"/>
+      <x:c r="H212" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I212" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J212" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K212" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_FrameWall.glb</x:v>
+      </x:c>
+      <x:c r="L212" s="1" t="str">
+        <x:v>9d5ae47dc5abc26930d7bafa9fcd11f7e5d1479843e64f892704be5e5b9cae0a</x:v>
+      </x:c>
+      <x:c r="M212" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N212" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O212" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P212" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="38" customHeight="1">
+      <x:c r="A213" s="1" t="str">
+        <x:v>Prop_Gallery_WindowWall</x:v>
+      </x:c>
+      <x:c r="B213" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C213" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D213" s="5" t="str">
+        <x:v>Window wall</x:v>
+      </x:c>
+      <x:c r="E213" s="7" t="n">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="F213" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G213" s="5" t="str"/>
+      <x:c r="H213" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I213" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J213" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K213" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_WindowWall.glb</x:v>
+      </x:c>
+      <x:c r="L213" s="1" t="str">
+        <x:v>0a487a806dd676c9c96fc529dddcdb551c17e8ae6f1e9f14dc6a60108cd7d93a</x:v>
+      </x:c>
+      <x:c r="M213" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N213" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O213" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P213" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="38" customHeight="1">
+      <x:c r="A214" s="1" t="str">
+        <x:v>Prop_Gallery_DoorFrame</x:v>
+      </x:c>
+      <x:c r="B214" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C214" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D214" s="5" t="str">
+        <x:v>Clear doorway module</x:v>
+      </x:c>
+      <x:c r="E214" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F214" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G214" s="5" t="str"/>
+      <x:c r="H214" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I214" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J214" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K214" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_DoorFrame.glb</x:v>
+      </x:c>
+      <x:c r="L214" s="1" t="str">
+        <x:v>d8cec4cccb4d9460441ae611e4c06bb58b509232aedf7dab40c5447cde903305</x:v>
+      </x:c>
+      <x:c r="M214" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N214" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O214" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P214" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="38" customHeight="1">
+      <x:c r="A215" s="1" t="str">
+        <x:v>Prop_Gallery_CornerColumn</x:v>
+      </x:c>
+      <x:c r="B215" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C215" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D215" s="5" t="str">
+        <x:v>Modular corner support</x:v>
+      </x:c>
+      <x:c r="E215" s="7" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="F215" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G215" s="5" t="str"/>
+      <x:c r="H215" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I215" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J215" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K215" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_CornerColumn.glb</x:v>
+      </x:c>
+      <x:c r="L215" s="1" t="str">
+        <x:v>1611123c9c7214068abb2fe1c41512221048b2e3122d8ce1316897fd02ba188d</x:v>
+      </x:c>
+      <x:c r="M215" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N215" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O215" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P215" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="38" customHeight="1">
+      <x:c r="A216" s="1" t="str">
+        <x:v>Prop_Gallery_Railing</x:v>
+      </x:c>
+      <x:c r="B216" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C216" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D216" s="5" t="str">
+        <x:v>Walkway boundary</x:v>
+      </x:c>
+      <x:c r="E216" s="7" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F216" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G216" s="5" t="str"/>
+      <x:c r="H216" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I216" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J216" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K216" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_Railing.glb</x:v>
+      </x:c>
+      <x:c r="L216" s="1" t="str">
+        <x:v>452e22c1743cbb9f1482bf3de7ee0b7a7c6c0be9d982fb288a5a555ee3b6bbb2</x:v>
+      </x:c>
+      <x:c r="M216" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N216" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O216" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P216" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="38" customHeight="1">
+      <x:c r="A217" s="1" t="str">
+        <x:v>Prop_Gallery_Ramp</x:v>
+      </x:c>
+      <x:c r="B217" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C217" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D217" s="5" t="str">
+        <x:v>Access ramp</x:v>
+      </x:c>
+      <x:c r="E217" s="7" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F217" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G217" s="5" t="str"/>
+      <x:c r="H217" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I217" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J217" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K217" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_Ramp.glb</x:v>
+      </x:c>
+      <x:c r="L217" s="1" t="str">
+        <x:v>06d35c586d5026e5aeb5c9efe4883530763b1333c99fd26758f99fdcb8ae437a</x:v>
+      </x:c>
+      <x:c r="M217" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N217" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O217" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P217" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="38" customHeight="1">
+      <x:c r="A218" s="1" t="str">
+        <x:v>Prop_Gallery_Stairs</x:v>
+      </x:c>
+      <x:c r="B218" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C218" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D218" s="5" t="str">
+        <x:v>Raised walkway access</x:v>
+      </x:c>
+      <x:c r="E218" s="7" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F218" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G218" s="5" t="str"/>
+      <x:c r="H218" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I218" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J218" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K218" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_Stairs.glb</x:v>
+      </x:c>
+      <x:c r="L218" s="1" t="str">
+        <x:v>13e07f9a7c25d8f7e3702d30d862dd391e6e5fe57ff7cbb5139f9734edc8382c</x:v>
+      </x:c>
+      <x:c r="M218" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N218" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O218" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P218" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="38" customHeight="1">
+      <x:c r="A219" s="1" t="str">
+        <x:v>Prop_Gallery_PaintingFrame</x:v>
+      </x:c>
+      <x:c r="B219" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C219" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D219" s="5" t="str">
+        <x:v>Art display frame</x:v>
+      </x:c>
+      <x:c r="E219" s="7" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="F219" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G219" s="5" t="str"/>
+      <x:c r="H219" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I219" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J219" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K219" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_PaintingFrame.glb</x:v>
+      </x:c>
+      <x:c r="L219" s="1" t="str">
+        <x:v>f92f63fe9c48924b46fe6e00beb0e2eff99c3f3be3671848bae518a0a9e14003</x:v>
+      </x:c>
+      <x:c r="M219" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N219" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O219" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P219" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="38" customHeight="1">
+      <x:c r="A220" s="1" t="str">
+        <x:v>Prop_Gallery_MuralPanel</x:v>
+      </x:c>
+      <x:c r="B220" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C220" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D220" s="5" t="str">
+        <x:v>Painted hint surface</x:v>
+      </x:c>
+      <x:c r="E220" s="7" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="F220" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G220" s="5" t="str"/>
+      <x:c r="H220" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I220" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J220" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K220" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_MuralPanel.glb</x:v>
+      </x:c>
+      <x:c r="L220" s="1" t="str">
+        <x:v>a2179351b6ef29e18a704160a3d3a7d660a3486d1be22ad4dbef9a7182b03e03</x:v>
+      </x:c>
+      <x:c r="M220" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N220" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O220" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P220" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="38" customHeight="1">
+      <x:c r="A221" s="1" t="str">
+        <x:v>Prop_Gallery_RestorationBench</x:v>
+      </x:c>
+      <x:c r="B221" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C221" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D221" s="5" t="str">
+        <x:v>Restoration station</x:v>
+      </x:c>
+      <x:c r="E221" s="7" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F221" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G221" s="5" t="str"/>
+      <x:c r="H221" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I221" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J221" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K221" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_RestorationBench.glb</x:v>
+      </x:c>
+      <x:c r="L221" s="1" t="str">
+        <x:v>70cb02477ea9bd06d39d3226cb9a2dc50219af30a4bcdb6579fa41e832f3fff9</x:v>
+      </x:c>
+      <x:c r="M221" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N221" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O221" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P221" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="38" customHeight="1">
+      <x:c r="A222" s="1" t="str">
+        <x:v>Prop_Gallery_PigmentCrate</x:v>
+      </x:c>
+      <x:c r="B222" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C222" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D222" s="5" t="str">
+        <x:v>Craft supplies presentation</x:v>
+      </x:c>
+      <x:c r="E222" s="7" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="F222" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G222" s="5" t="str"/>
+      <x:c r="H222" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I222" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J222" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K222" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_PigmentCrate.glb</x:v>
+      </x:c>
+      <x:c r="L222" s="1" t="str">
+        <x:v>8d1ff03c888a128481c798e51b48bca8ff2967930808c420bb520003e4921e61</x:v>
+      </x:c>
+      <x:c r="M222" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N222" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O222" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P222" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="38" customHeight="1">
+      <x:c r="A223" s="1" t="str">
+        <x:v>Prop_Gallery_BrushRack</x:v>
+      </x:c>
+      <x:c r="B223" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C223" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D223" s="5" t="str">
+        <x:v>Tool display</x:v>
+      </x:c>
+      <x:c r="E223" s="7" t="n">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="F223" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G223" s="5" t="str"/>
+      <x:c r="H223" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I223" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J223" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K223" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_BrushRack.glb</x:v>
+      </x:c>
+      <x:c r="L223" s="1" t="str">
+        <x:v>d743d839602ba389a380e8f1536cf282c897cd4f3a6d381a4cf106c96dab6bd3</x:v>
+      </x:c>
+      <x:c r="M223" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N223" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O223" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P223" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="38" customHeight="1">
+      <x:c r="A224" s="1" t="str">
+        <x:v>Prop_Gallery_VarnishStation</x:v>
+      </x:c>
+      <x:c r="B224" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C224" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D224" s="5" t="str">
+        <x:v>Painting protection station</x:v>
+      </x:c>
+      <x:c r="E224" s="7" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="F224" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G224" s="5" t="str"/>
+      <x:c r="H224" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I224" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J224" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K224" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_VarnishStation.glb</x:v>
+      </x:c>
+      <x:c r="L224" s="1" t="str">
+        <x:v>ca2a1e73e2b365823ccaf8f2baeb6c27fe9d5e8e195b102792eaff158c47cbe1</x:v>
+      </x:c>
+      <x:c r="M224" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N224" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O224" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P224" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="38" customHeight="1">
+      <x:c r="A225" s="1" t="str">
+        <x:v>Prop_Gallery_TailorStand</x:v>
+      </x:c>
+      <x:c r="B225" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C225" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D225" s="5" t="str">
+        <x:v>Cosmetic station</x:v>
+      </x:c>
+      <x:c r="E225" s="7" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="F225" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G225" s="5" t="str"/>
+      <x:c r="H225" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I225" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J225" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K225" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_TailorStand.glb</x:v>
+      </x:c>
+      <x:c r="L225" s="1" t="str">
+        <x:v>7efcdd22abaa7bb0e1c91bb2afe7df138d33291f84ad38911bdc07e0d59e9b18</x:v>
+      </x:c>
+      <x:c r="M225" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N225" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O225" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P225" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="38" customHeight="1">
+      <x:c r="A226" s="1" t="str">
+        <x:v>Prop_Gallery_CriticLectern</x:v>
+      </x:c>
+      <x:c r="B226" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C226" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D226" s="5" t="str">
+        <x:v>Build review station</x:v>
+      </x:c>
+      <x:c r="E226" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F226" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G226" s="5" t="str"/>
+      <x:c r="H226" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I226" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J226" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K226" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_CriticLectern.glb</x:v>
+      </x:c>
+      <x:c r="L226" s="1" t="str">
+        <x:v>76b0f7fd9e250e4eef6ef47f13c988a3a047c34fd174af3f6eb74117b1387f84</x:v>
+      </x:c>
+      <x:c r="M226" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N226" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O226" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P226" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="38" customHeight="1">
+      <x:c r="A227" s="1" t="str">
+        <x:v>Prop_Gallery_DroneDock</x:v>
+      </x:c>
+      <x:c r="B227" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C227" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D227" s="5" t="str">
+        <x:v>Mount pickup presentation</x:v>
+      </x:c>
+      <x:c r="E227" s="7" t="n">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="F227" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G227" s="5" t="str"/>
+      <x:c r="H227" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I227" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J227" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K227" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_DroneDock.glb</x:v>
+      </x:c>
+      <x:c r="L227" s="1" t="str">
+        <x:v>28d3e3b0170212303c90aed4b7194f8bb656990f8d3c2553bfc69612def727dc</x:v>
+      </x:c>
+      <x:c r="M227" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N227" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O227" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P227" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="38" customHeight="1">
+      <x:c r="A228" s="1" t="str">
+        <x:v>Prop_Gallery_DroneRepairBench</x:v>
+      </x:c>
+      <x:c r="B228" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C228" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D228" s="5" t="str">
+        <x:v>Mount repair station</x:v>
+      </x:c>
+      <x:c r="E228" s="7" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="F228" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G228" s="5" t="str"/>
+      <x:c r="H228" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I228" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J228" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K228" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_DroneRepairBench.glb</x:v>
+      </x:c>
+      <x:c r="L228" s="1" t="str">
+        <x:v>0a7959d54210842e0df385ff0bcd2afa424989900c7502148a74581891af9eb8</x:v>
+      </x:c>
+      <x:c r="M228" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N228" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O228" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P228" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="38" customHeight="1">
+      <x:c r="A229" s="1" t="str">
+        <x:v>Prop_Gallery_ConcertPlatform</x:v>
+      </x:c>
+      <x:c r="B229" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C229" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D229" s="5" t="str">
+        <x:v>Touring jukebox performance station</x:v>
+      </x:c>
+      <x:c r="E229" s="7" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="F229" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G229" s="5" t="str"/>
+      <x:c r="H229" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I229" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J229" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K229" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_ConcertPlatform.glb</x:v>
+      </x:c>
+      <x:c r="L229" s="1" t="str">
+        <x:v>25ce6a97e6b365052c3573d5c965a2b7d287baa45082bb5415735f201b4a447b</x:v>
+      </x:c>
+      <x:c r="M229" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N229" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O229" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P229" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="38" customHeight="1">
+      <x:c r="A230" s="1" t="str">
+        <x:v>Prop_Gallery_RainbowFrame</x:v>
+      </x:c>
+      <x:c r="B230" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C230" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D230" s="5" t="str">
+        <x:v>Rainbow departure frame</x:v>
+      </x:c>
+      <x:c r="E230" s="7" t="n">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="F230" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G230" s="5" t="str"/>
+      <x:c r="H230" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I230" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J230" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K230" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_RainbowFrame.glb</x:v>
+      </x:c>
+      <x:c r="L230" s="1" t="str">
+        <x:v>82d8cc1b21978e5e5d9b5196d20098b04cdebd84a439ea90541133470a9911db</x:v>
+      </x:c>
+      <x:c r="M230" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N230" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O230" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P230" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="38" customHeight="1">
+      <x:c r="A231" s="1" t="str">
+        <x:v>Prop_Gallery_AirlockEntry</x:v>
+      </x:c>
+      <x:c r="B231" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C231" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D231" s="5" t="str">
+        <x:v>Underwater dock arrival presentation</x:v>
+      </x:c>
+      <x:c r="E231" s="7" t="n">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="F231" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G231" s="5" t="str"/>
+      <x:c r="H231" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I231" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J231" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K231" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_AirlockEntry.glb</x:v>
+      </x:c>
+      <x:c r="L231" s="1" t="str">
+        <x:v>357d4200bfd5eff30d1dca6bf6124f7f393016cf60ba8950b3dededd3d92d609</x:v>
+      </x:c>
+      <x:c r="M231" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N231" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O231" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P231" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="38" customHeight="1">
+      <x:c r="A232" s="1" t="str">
+        <x:v>Prop_Gallery_QuestNoticeboard</x:v>
+      </x:c>
+      <x:c r="B232" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C232" s="1" t="str">
+        <x:v>Gallery City</x:v>
+      </x:c>
+      <x:c r="D232" s="5" t="str">
+        <x:v>Readable quest presentation</x:v>
+      </x:c>
+      <x:c r="E232" s="7" t="n">
+        <x:v>440</x:v>
+      </x:c>
+      <x:c r="F232" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G232" s="5" t="str"/>
+      <x:c r="H232" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I232" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J232" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K232" s="1" t="str">
+        <x:v>gallery-buildout/environment/Prop_Gallery_QuestNoticeboard.glb</x:v>
+      </x:c>
+      <x:c r="L232" s="1" t="str">
+        <x:v>70cd56651a278ebffee8f8728bae55b8ba932163ed4415512e33897634d2c414</x:v>
+      </x:c>
+      <x:c r="M232" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N232" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O232" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P232" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="6">
+  <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="I6:I72">
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
@@ -9709,6 +11811,12 @@
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J164:J189">
+      <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I190:I232">
+      <x:formula1>"Pending,Imported,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J190:J232">
       <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -10435,12 +12543,22 @@
       <x:c r="K31" s="2"/>
       <x:c r="L31" s="2"/>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
+    <x:row r="32" ht="52" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>GAL01</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>Living paintings and colour knowledge</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>32 role cast with 19 creature/mount/pet visuals</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="str">
+        <x:v>Art validated; abilities proposed</x:v>
+      </x:c>
+      <x:c r="E32" s="4" t="str">
+        <x:v>Restore city murals and make colour useful</x:v>
+      </x:c>
       <x:c r="F32" s="2"/>
       <x:c r="G32" s="2"/>
       <x:c r="H32" s="2"/>
@@ -10449,12 +12567,22 @@
       <x:c r="K32" s="2"/>
       <x:c r="L32" s="2"/>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-      <x:c r="D33" s="2"/>
-      <x:c r="E33" s="2"/>
+    <x:row r="33" ht="52" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:v>GAL02</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>Frame streets, workstations, drone/sea arrival docks</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>24 modular props, 2 m snap grid</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="str">
+        <x:v>Static validation; collision/interaction pending</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="str">
+        <x:v>Connect framed plazas, workshops and visiting realms</x:v>
+      </x:c>
       <x:c r="F33" s="2"/>
       <x:c r="G33" s="2"/>
       <x:c r="H33" s="2"/>
@@ -10463,12 +12591,22 @@
       <x:c r="K33" s="2"/>
       <x:c r="L33" s="2"/>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
-      <x:c r="D34" s="2"/>
-      <x:c r="E34" s="2"/>
+    <x:row r="34" ht="52" customHeight="1">
+      <x:c r="A34" s="2" t="str">
+        <x:v>GAL03</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>Curator reward must require actual objective proof</x:v>
+      </x:c>
+      <x:c r="C34" s="4" t="str">
+        <x:v>Existing DCS found choice + FRAME_PLATE</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="str">
+        <x:v>Owner notified; authoritative gating pending</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="str">
+        <x:v>Claims of a rescue/discovery must reflect completed actions</x:v>
+      </x:c>
       <x:c r="F34" s="2"/>
       <x:c r="G34" s="2"/>
       <x:c r="H34" s="2"/>

</xml_diff>

<commit_message>
Complete Parcels environment kit with provenance-preserving trough reuse
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Raadceb366b584e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R125713e2e28c4d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Ra0e1ac36088244e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R0d6ccfa970be4c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R95944fd561cf436b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Ra283ac5bb0944d1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243746"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -80,7 +85,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -130,6 +135,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -458,15 +468,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -474,7 +484,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -493,15 +503,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A8)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A8)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="2" t="n">
@@ -509,7 +519,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A8)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
@@ -528,15 +538,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -544,7 +554,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A9)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9)</x:f>
         <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
@@ -563,15 +573,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A10)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="2" t="n">
@@ -579,7 +589,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A10)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
@@ -598,24 +608,24 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$232,Assets!$C$6:$C$232,A11)</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A11)</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11,Assets!$B$6:$B$232,"Character",Assets!$H$6:$H$232,"Validated")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11,Assets!$B$6:$B$232,"Character",Assets!$I$6:$I$232,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="2" t="n">
         <x:f>C11-D11</x:f>
-        <x:v>32</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$232,A11)</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
@@ -655,8 +665,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E232)</x:f>
-        <x:v>217522</x:v>
+        <x:f>SUM(Assets!E6:E288)</x:f>
+        <x:v>265360</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -674,8 +684,8 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B232,"Prop")+COUNTIFS(Assets!B6:B232,"Item")</x:f>
-        <x:v>83</x:v>
+        <x:f>COUNTIFS(Assets!B6:B288,"Prop")+COUNTIFS(Assets!B6:B288,"Item")</x:f>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -704,7 +714,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Codex first kits only. Gallery 56 exports; native behaviors/visual acceptance pending. LODs are not new roles.</x:v>
+        <x:v>Codex kits: 283 unique asset references, including one unchanged AMF reuse. Export validation is not Play proof.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -1445,6 +1455,7 @@
     <x:col min="12" max="12" width="70" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="14" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1556,6 +1567,9 @@
       <x:c r="P5" s="19" t="str">
         <x:v>LOD level</x:v>
       </x:c>
+      <x:c r="Q5" s="23" t="str">
+        <x:v>Provenance</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="2" t="str">
@@ -11793,8 +11807,2928 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
+    <x:row r="233" ht="38" customHeight="1">
+      <x:c r="A233" s="1" t="str">
+        <x:v>Mob_Parcels_Courier</x:v>
+      </x:c>
+      <x:c r="B233" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C233" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D233" s="5" t="str">
+        <x:v>Hero parcel courier</x:v>
+      </x:c>
+      <x:c r="E233" s="7" t="n">
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="F233" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G233" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H233" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I233" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J233" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K233" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_Courier.glb</x:v>
+      </x:c>
+      <x:c r="L233" s="1" t="str">
+        <x:v>bf0996f414bc81cebfccd237517db84d357fca8112a212a4518ab13ad973fff3</x:v>
+      </x:c>
+      <x:c r="M233" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N233" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O233" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P233" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q233" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="38" customHeight="1">
+      <x:c r="A234" s="1" t="str">
+        <x:v>Mob_Parcels_PostmasterGrue</x:v>
+      </x:c>
+      <x:c r="B234" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C234" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D234" s="5" t="str">
+        <x:v>Delivery quest board</x:v>
+      </x:c>
+      <x:c r="E234" s="7" t="n">
+        <x:v>1088</x:v>
+      </x:c>
+      <x:c r="F234" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G234" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H234" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I234" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J234" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K234" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_PostmasterGrue.glb</x:v>
+      </x:c>
+      <x:c r="L234" s="1" t="str">
+        <x:v>cc9275a50174767d6064b410da673c812eea992c9a6575d94b6518912034345c</x:v>
+      </x:c>
+      <x:c r="M234" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N234" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O234" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P234" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q234" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="38" customHeight="1">
+      <x:c r="A235" s="1" t="str">
+        <x:v>Mob_Parcels_PlotSurveyorIlka</x:v>
+      </x:c>
+      <x:c r="B235" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C235" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D235" s="5" t="str">
+        <x:v>Survey presentation; no deed authority</x:v>
+      </x:c>
+      <x:c r="E235" s="7" t="n">
+        <x:v>1020</x:v>
+      </x:c>
+      <x:c r="F235" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G235" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H235" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I235" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J235" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K235" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_PlotSurveyorIlka.glb</x:v>
+      </x:c>
+      <x:c r="L235" s="1" t="str">
+        <x:v>6dc02e93053d5fc156e68d68745c0ca2b9c70334a7fffcfc7b917d330d53d364</x:v>
+      </x:c>
+      <x:c r="M235" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N235" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O235" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P235" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q235" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="38" customHeight="1">
+      <x:c r="A236" s="1" t="str">
+        <x:v>Mob_Parcels_FenceSmith</x:v>
+      </x:c>
+      <x:c r="B236" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C236" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D236" s="5" t="str">
+        <x:v>Fence crafting</x:v>
+      </x:c>
+      <x:c r="E236" s="7" t="n">
+        <x:v>936</x:v>
+      </x:c>
+      <x:c r="F236" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G236" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H236" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I236" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J236" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K236" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_FenceSmith.glb</x:v>
+      </x:c>
+      <x:c r="L236" s="1" t="str">
+        <x:v>c3c21555e0ed5cf354c44a5097e477dc3c387cceca78c191fb2aac2b887ffcae</x:v>
+      </x:c>
+      <x:c r="M236" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N236" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O236" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P236" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q236" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="38" customHeight="1">
+      <x:c r="A237" s="1" t="str">
+        <x:v>Mob_Parcels_SeedBrokerOtt</x:v>
+      </x:c>
+      <x:c r="B237" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C237" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D237" s="5" t="str">
+        <x:v>Seed supplies</x:v>
+      </x:c>
+      <x:c r="E237" s="7" t="n">
+        <x:v>1092</x:v>
+      </x:c>
+      <x:c r="F237" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G237" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H237" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I237" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J237" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K237" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_SeedBrokerOtt.glb</x:v>
+      </x:c>
+      <x:c r="L237" s="1" t="str">
+        <x:v>ba6f0121e58e93c664487bdbbe913de53b943cdc50f55ee35363e22324de9c55</x:v>
+      </x:c>
+      <x:c r="M237" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N237" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O237" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P237" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q237" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="38" customHeight="1">
+      <x:c r="A238" s="1" t="str">
+        <x:v>Mob_Parcels_ScarecrowElder</x:v>
+      </x:c>
+      <x:c r="B238" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C238" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D238" s="5" t="str">
+        <x:v>Helpful field guide</x:v>
+      </x:c>
+      <x:c r="E238" s="7" t="n">
+        <x:v>1080</x:v>
+      </x:c>
+      <x:c r="F238" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G238" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H238" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I238" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J238" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K238" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_ScarecrowElder.glb</x:v>
+      </x:c>
+      <x:c r="L238" s="1" t="str">
+        <x:v>072136d18cd624b7449acf69a1e126443ace76e47943123b82b8e5722159aa28</x:v>
+      </x:c>
+      <x:c r="M238" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N238" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O238" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P238" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q238" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="38" customHeight="1">
+      <x:c r="A239" s="1" t="str">
+        <x:v>Mob_Parcels_HelipadChiefRosa</x:v>
+      </x:c>
+      <x:c r="B239" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C239" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D239" s="5" t="str">
+        <x:v>Helicopter guidance</x:v>
+      </x:c>
+      <x:c r="E239" s="7" t="n">
+        <x:v>980</x:v>
+      </x:c>
+      <x:c r="F239" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G239" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H239" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I239" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J239" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K239" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_HelipadChiefRosa.glb</x:v>
+      </x:c>
+      <x:c r="L239" s="1" t="str">
+        <x:v>8f66d723b6da8197eeff1e86740ad3e1c42a446aab940349fa90dd0c6a4fae34</x:v>
+      </x:c>
+      <x:c r="M239" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N239" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O239" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P239" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q239" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="38" customHeight="1">
+      <x:c r="A240" s="1" t="str">
+        <x:v>Mob_Parcels_MilkCartTwins</x:v>
+      </x:c>
+      <x:c r="B240" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C240" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D240" s="5" t="str">
+        <x:v>Cart escort role representative</x:v>
+      </x:c>
+      <x:c r="E240" s="7" t="n">
+        <x:v>1164</x:v>
+      </x:c>
+      <x:c r="F240" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G240" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H240" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I240" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J240" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K240" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_MilkCartTwins.glb</x:v>
+      </x:c>
+      <x:c r="L240" s="1" t="str">
+        <x:v>dc3fd8dfd5dc8edad794d5b7e0b4bd8ae864f59b3cef1464b3e95a20f5caa5a5</x:v>
+      </x:c>
+      <x:c r="M240" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N240" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O240" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P240" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q240" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="38" customHeight="1">
+      <x:c r="A241" s="1" t="str">
+        <x:v>Mob_Parcels_LostLetterCourier</x:v>
+      </x:c>
+      <x:c r="B241" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C241" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D241" s="5" t="str">
+        <x:v>Lost letter quest; nonHalloween ghost reinterpretation</x:v>
+      </x:c>
+      <x:c r="E241" s="7" t="n">
+        <x:v>1052</x:v>
+      </x:c>
+      <x:c r="F241" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G241" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H241" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I241" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J241" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K241" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_LostLetterCourier.glb</x:v>
+      </x:c>
+      <x:c r="L241" s="1" t="str">
+        <x:v>b955a27486c3f020fc7e535fa6417dd0b0c6c255352662e44775c832a7fa243c</x:v>
+      </x:c>
+      <x:c r="M241" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N241" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O241" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P241" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q241" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="38" customHeight="1">
+      <x:c r="A242" s="1" t="str">
+        <x:v>Mob_Parcels_BeekeeperHollis</x:v>
+      </x:c>
+      <x:c r="B242" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C242" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D242" s="5" t="str">
+        <x:v>Bee and honey supplies</x:v>
+      </x:c>
+      <x:c r="E242" s="7" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="F242" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G242" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H242" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I242" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J242" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K242" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_BeekeeperHollis.glb</x:v>
+      </x:c>
+      <x:c r="L242" s="1" t="str">
+        <x:v>e76bdb218217fce1de5b68c338680041c2f2f1e739065f09c648062d61e8aa25</x:v>
+      </x:c>
+      <x:c r="M242" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N242" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O242" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P242" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q242" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="38" customHeight="1">
+      <x:c r="A243" s="1" t="str">
+        <x:v>Mob_Parcels_AuctionCrow</x:v>
+      </x:c>
+      <x:c r="B243" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C243" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D243" s="5" t="str">
+        <x:v>Market role</x:v>
+      </x:c>
+      <x:c r="E243" s="7" t="n">
+        <x:v>980</x:v>
+      </x:c>
+      <x:c r="F243" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G243" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H243" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I243" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J243" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K243" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_AuctionCrow.glb</x:v>
+      </x:c>
+      <x:c r="L243" s="1" t="str">
+        <x:v>49821ce09034ff47180e0eccdf52fbfbdd2fd09e6cfb1c756d656462fdda1c3c</x:v>
+      </x:c>
+      <x:c r="M243" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N243" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O243" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P243" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q243" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="38" customHeight="1">
+      <x:c r="A244" s="1" t="str">
+        <x:v>Mob_Parcels_WeatherVaneKeeper</x:v>
+      </x:c>
+      <x:c r="B244" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C244" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D244" s="5" t="str">
+        <x:v>Storm and crop guidance</x:v>
+      </x:c>
+      <x:c r="E244" s="7" t="n">
+        <x:v>964</x:v>
+      </x:c>
+      <x:c r="F244" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G244" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H244" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I244" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J244" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K244" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_WeatherVaneKeeper.glb</x:v>
+      </x:c>
+      <x:c r="L244" s="1" t="str">
+        <x:v>1013286ffb4fc52965e77f88dd8633d37c988911c68cc97007d0f2f22f7b6e11</x:v>
+      </x:c>
+      <x:c r="M244" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N244" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O244" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P244" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q244" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="38" customHeight="1">
+      <x:c r="A245" s="1" t="str">
+        <x:v>Mob_Parcels_NeighbourFeudPair</x:v>
+      </x:c>
+      <x:c r="B245" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C245" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D245" s="5" t="str">
+        <x:v>Boundary quest representative</x:v>
+      </x:c>
+      <x:c r="E245" s="7" t="n">
+        <x:v>1020</x:v>
+      </x:c>
+      <x:c r="F245" s="1" t="str">
+        <x:v>ParcelsHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G245" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H245" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I245" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J245" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K245" s="1" t="str">
+        <x:v>parcels-buildout/cast/Mob_Parcels_NeighbourFeudPair.glb</x:v>
+      </x:c>
+      <x:c r="L245" s="1" t="str">
+        <x:v>2651571ddbd7a1c629f8f7ce19ed9b3842ccbfb8e8153dc16c8c47df977a0cd4</x:v>
+      </x:c>
+      <x:c r="M245" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N245" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O245" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P245" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q245" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="38" customHeight="1">
+      <x:c r="A246" s="1" t="str">
+        <x:v>Mob_Parcels_MailboxMimic</x:v>
+      </x:c>
+      <x:c r="B246" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C246" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D246" s="5" t="str">
+        <x:v>Mailbox encounter</x:v>
+      </x:c>
+      <x:c r="E246" s="7" t="n">
+        <x:v>1072</x:v>
+      </x:c>
+      <x:c r="F246" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G246" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H246" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I246" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J246" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K246" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_MailboxMimic.glb</x:v>
+      </x:c>
+      <x:c r="L246" s="1" t="str">
+        <x:v>494fe5a93ef8d3d195c45d690b85308d5c056d3e549c523debd30fa9eea3c0d5</x:v>
+      </x:c>
+      <x:c r="M246" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N246" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O246" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P246" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q246" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="38" customHeight="1">
+      <x:c r="A247" s="1" t="str">
+        <x:v>Mob_Parcels_BurrowVole</x:v>
+      </x:c>
+      <x:c r="B247" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C247" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D247" s="5" t="str">
+        <x:v>Burrowing creature</x:v>
+      </x:c>
+      <x:c r="E247" s="7" t="n">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="F247" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G247" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H247" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I247" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J247" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K247" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_BurrowVole.glb</x:v>
+      </x:c>
+      <x:c r="L247" s="1" t="str">
+        <x:v>fa2fe721b3207185d1eb5725ef23029c388dfa4eb604fff67bfdbc85b622e6a7</x:v>
+      </x:c>
+      <x:c r="M247" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N247" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O247" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P247" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q247" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="38" customHeight="1">
+      <x:c r="A248" s="1" t="str">
+        <x:v>Mob_Parcels_HaySprite</x:v>
+      </x:c>
+      <x:c r="B248" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C248" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D248" s="5" t="str">
+        <x:v>Field creature</x:v>
+      </x:c>
+      <x:c r="E248" s="7" t="n">
+        <x:v>1360</x:v>
+      </x:c>
+      <x:c r="F248" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G248" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H248" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I248" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J248" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K248" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_HaySprite.glb</x:v>
+      </x:c>
+      <x:c r="L248" s="1" t="str">
+        <x:v>57aaf592025a532c3d7d955188c51b3d5d796389f1f88dc80ce7ae78f95faa1e</x:v>
+      </x:c>
+      <x:c r="M248" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N248" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O248" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P248" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q248" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="38" customHeight="1">
+      <x:c r="A249" s="1" t="str">
+        <x:v>Mob_Parcels_ThistleBoar</x:v>
+      </x:c>
+      <x:c r="B249" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C249" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D249" s="5" t="str">
+        <x:v>Briar boar</x:v>
+      </x:c>
+      <x:c r="E249" s="7" t="n">
+        <x:v>1606</x:v>
+      </x:c>
+      <x:c r="F249" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G249" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H249" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I249" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J249" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K249" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_ThistleBoar.glb</x:v>
+      </x:c>
+      <x:c r="L249" s="1" t="str">
+        <x:v>48480b340d372a2c2e1c357660a58d31d572822bcc65822543ac5c5528e4ab3a</x:v>
+      </x:c>
+      <x:c r="M249" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N249" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O249" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P249" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q249" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="38" customHeight="1">
+      <x:c r="A250" s="1" t="str">
+        <x:v>Mob_Parcels_TwineSnake</x:v>
+      </x:c>
+      <x:c r="B250" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C250" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D250" s="5" t="str">
+        <x:v>Twine serpent</x:v>
+      </x:c>
+      <x:c r="E250" s="7" t="n">
+        <x:v>2464</x:v>
+      </x:c>
+      <x:c r="F250" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G250" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H250" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I250" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J250" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K250" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_TwineSnake.glb</x:v>
+      </x:c>
+      <x:c r="L250" s="1" t="str">
+        <x:v>fdde0d64b8797fdfa65aa67978c5ee57e739514f578c32acc63968cc573ae914</x:v>
+      </x:c>
+      <x:c r="M250" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N250" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O250" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P250" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q250" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="38" customHeight="1">
+      <x:c r="A251" s="1" t="str">
+        <x:v>Mob_Parcels_WheelbarrowGolem</x:v>
+      </x:c>
+      <x:c r="B251" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C251" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D251" s="5" t="str">
+        <x:v>Cart creature</x:v>
+      </x:c>
+      <x:c r="E251" s="7" t="n">
+        <x:v>1428</x:v>
+      </x:c>
+      <x:c r="F251" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G251" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H251" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I251" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J251" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K251" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_WheelbarrowGolem.glb</x:v>
+      </x:c>
+      <x:c r="L251" s="1" t="str">
+        <x:v>a16d1d92b4ab43aaea6dda53709c56df0d2429a16118e0d5efff614fcd06c8c7</x:v>
+      </x:c>
+      <x:c r="M251" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N251" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O251" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P251" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q251" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="38" customHeight="1">
+      <x:c r="A252" s="1" t="str">
+        <x:v>Mob_Parcels_StampedeCalf</x:v>
+      </x:c>
+      <x:c r="B252" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C252" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D252" s="5" t="str">
+        <x:v>Field calf</x:v>
+      </x:c>
+      <x:c r="E252" s="7" t="n">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="F252" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G252" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H252" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I252" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J252" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K252" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_StampedeCalf.glb</x:v>
+      </x:c>
+      <x:c r="L252" s="1" t="str">
+        <x:v>01891efc6bc6fe6cd9c0bc1799e41ce0aa3f7a36334a74c2ae2ac82c8cd9477f</x:v>
+      </x:c>
+      <x:c r="M252" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N252" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O252" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P252" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q252" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="38" customHeight="1">
+      <x:c r="A253" s="1" t="str">
+        <x:v>Mob_Parcels_CombineCrab</x:v>
+      </x:c>
+      <x:c r="B253" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C253" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D253" s="5" t="str">
+        <x:v>Machine crab</x:v>
+      </x:c>
+      <x:c r="E253" s="7" t="n">
+        <x:v>1288</x:v>
+      </x:c>
+      <x:c r="F253" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G253" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H253" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I253" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J253" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K253" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_CombineCrab.glb</x:v>
+      </x:c>
+      <x:c r="L253" s="1" t="str">
+        <x:v>eea69b95ab34bd370d9ef3a2c2026cef6bee293371eef421eafe2e29b2b520b4</x:v>
+      </x:c>
+      <x:c r="M253" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N253" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O253" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P253" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q253" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="38" customHeight="1">
+      <x:c r="A254" s="1" t="str">
+        <x:v>Mob_Parcels_RustwingHawk</x:v>
+      </x:c>
+      <x:c r="B254" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C254" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D254" s="5" t="str">
+        <x:v>Field hunter</x:v>
+      </x:c>
+      <x:c r="E254" s="7" t="n">
+        <x:v>1570</x:v>
+      </x:c>
+      <x:c r="F254" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G254" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H254" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I254" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J254" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K254" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_RustwingHawk.glb</x:v>
+      </x:c>
+      <x:c r="L254" s="1" t="str">
+        <x:v>d0141fe508b6e5b4f64c1109f291869a4f6b2f8ad206c287234cab4d26fb2eaa</x:v>
+      </x:c>
+      <x:c r="M254" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N254" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O254" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P254" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q254" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255" ht="38" customHeight="1">
+      <x:c r="A255" s="1" t="str">
+        <x:v>Mob_Parcels_BlightBailiff</x:v>
+      </x:c>
+      <x:c r="B255" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C255" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D255" s="5" t="str">
+        <x:v>Boss proposal; no deed authority</x:v>
+      </x:c>
+      <x:c r="E255" s="7" t="n">
+        <x:v>1384</x:v>
+      </x:c>
+      <x:c r="F255" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G255" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H255" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I255" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J255" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K255" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_BlightBailiff.glb</x:v>
+      </x:c>
+      <x:c r="L255" s="1" t="str">
+        <x:v>c65c9fd63c9bed783edb1a313f1236d26327234fb38b51462eae8dcc6954f9ab</x:v>
+      </x:c>
+      <x:c r="M255" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N255" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O255" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P255" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q255" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256" ht="38" customHeight="1">
+      <x:c r="A256" s="1" t="str">
+        <x:v>Mob_Parcels_FenceLark</x:v>
+      </x:c>
+      <x:c r="B256" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C256" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D256" s="5" t="str">
+        <x:v>Ambient bird</x:v>
+      </x:c>
+      <x:c r="E256" s="7" t="n">
+        <x:v>1564</x:v>
+      </x:c>
+      <x:c r="F256" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G256" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H256" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I256" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J256" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K256" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_FenceLark.glb</x:v>
+      </x:c>
+      <x:c r="L256" s="1" t="str">
+        <x:v>b45e66850f77ba8011da8ff75fd8b759ddffb5f0a8e5af55336a229743fa483e</x:v>
+      </x:c>
+      <x:c r="M256" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N256" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O256" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P256" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q256" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257" ht="38" customHeight="1">
+      <x:c r="A257" s="1" t="str">
+        <x:v>Mob_Parcels_PuddleDuck</x:v>
+      </x:c>
+      <x:c r="B257" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C257" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D257" s="5" t="str">
+        <x:v>Ambient bird</x:v>
+      </x:c>
+      <x:c r="E257" s="7" t="n">
+        <x:v>1564</x:v>
+      </x:c>
+      <x:c r="F257" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G257" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H257" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I257" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J257" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K257" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_PuddleDuck.glb</x:v>
+      </x:c>
+      <x:c r="L257" s="1" t="str">
+        <x:v>d8f52452e7ab937f29ed37df5fd498653ceefb1f760a395182cd234ef62784d3</x:v>
+      </x:c>
+      <x:c r="M257" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N257" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O257" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P257" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q257" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258" ht="38" customHeight="1">
+      <x:c r="A258" s="1" t="str">
+        <x:v>Mob_Parcels_ParcelHelicopter</x:v>
+      </x:c>
+      <x:c r="B258" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C258" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D258" s="5" t="str">
+        <x:v>Realm mount; physics pending</x:v>
+      </x:c>
+      <x:c r="E258" s="7" t="n">
+        <x:v>740</x:v>
+      </x:c>
+      <x:c r="F258" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G258" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H258" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I258" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J258" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K258" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_ParcelHelicopter.glb</x:v>
+      </x:c>
+      <x:c r="L258" s="1" t="str">
+        <x:v>d894e2b0f2c50643b1be3c63770b641e5643879c3bc56b25792ee115b0b108ef</x:v>
+      </x:c>
+      <x:c r="M258" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N258" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O258" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P258" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q258" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259" ht="38" customHeight="1">
+      <x:c r="A259" s="1" t="str">
+        <x:v>Mob_Parcels_DraftOx</x:v>
+      </x:c>
+      <x:c r="B259" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C259" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D259" s="5" t="str">
+        <x:v>Pack companion</x:v>
+      </x:c>
+      <x:c r="E259" s="7" t="n">
+        <x:v>1644</x:v>
+      </x:c>
+      <x:c r="F259" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G259" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H259" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I259" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J259" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K259" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_DraftOx.glb</x:v>
+      </x:c>
+      <x:c r="L259" s="1" t="str">
+        <x:v>efb1d5768ded8834ede541efa70b51c15500a66810a3954e0ebe51fad0a26d35</x:v>
+      </x:c>
+      <x:c r="M259" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N259" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O259" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P259" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q259" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260" ht="38" customHeight="1">
+      <x:c r="A260" s="1" t="str">
+        <x:v>Mob_Parcels_GyroGoat</x:v>
+      </x:c>
+      <x:c r="B260" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C260" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D260" s="5" t="str">
+        <x:v>Climbing companion</x:v>
+      </x:c>
+      <x:c r="E260" s="7" t="n">
+        <x:v>1662</x:v>
+      </x:c>
+      <x:c r="F260" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G260" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H260" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I260" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J260" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K260" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_GyroGoat.glb</x:v>
+      </x:c>
+      <x:c r="L260" s="1" t="str">
+        <x:v>8d2ed1c3c0a8a31f508c51e43e2f5954a4431d5e3c8c891b9262fbd60971501f</x:v>
+      </x:c>
+      <x:c r="M260" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N260" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O260" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P260" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q260" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261" ht="38" customHeight="1">
+      <x:c r="A261" s="1" t="str">
+        <x:v>Mob_Parcels_ParcelPup</x:v>
+      </x:c>
+      <x:c r="B261" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C261" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D261" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E261" s="7" t="n">
+        <x:v>1796</x:v>
+      </x:c>
+      <x:c r="F261" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G261" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H261" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I261" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J261" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K261" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_ParcelPup.glb</x:v>
+      </x:c>
+      <x:c r="L261" s="1" t="str">
+        <x:v>728c140ffceb965ccee3428d6b978b8d41796931c6baf5d1bcb7621321f1c41a</x:v>
+      </x:c>
+      <x:c r="M261" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N261" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O261" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P261" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q261" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262" ht="38" customHeight="1">
+      <x:c r="A262" s="1" t="str">
+        <x:v>Mob_Parcels_CloverRabbit</x:v>
+      </x:c>
+      <x:c r="B262" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C262" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D262" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E262" s="7" t="n">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="F262" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G262" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H262" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I262" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J262" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K262" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_CloverRabbit.glb</x:v>
+      </x:c>
+      <x:c r="L262" s="1" t="str">
+        <x:v>df7d5262173fa734cde6ec1e5f1b3f6e0a997f83447297d1451fb905973a1b01</x:v>
+      </x:c>
+      <x:c r="M262" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N262" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O262" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P262" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q262" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263" ht="38" customHeight="1">
+      <x:c r="A263" s="1" t="str">
+        <x:v>Mob_Parcels_BarnOwlet</x:v>
+      </x:c>
+      <x:c r="B263" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C263" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D263" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E263" s="7" t="n">
+        <x:v>1948</x:v>
+      </x:c>
+      <x:c r="F263" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G263" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H263" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I263" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J263" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K263" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_BarnOwlet.glb</x:v>
+      </x:c>
+      <x:c r="L263" s="1" t="str">
+        <x:v>b90afe48015bed3ef9ea4e2f6eff5ad79ae5cbecf3fb2dd5b7d30396e48d6740</x:v>
+      </x:c>
+      <x:c r="M263" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N263" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O263" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P263" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q263" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264" ht="38" customHeight="1">
+      <x:c r="A264" s="1" t="str">
+        <x:v>Mob_Parcels_SeedMouse</x:v>
+      </x:c>
+      <x:c r="B264" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C264" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D264" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E264" s="7" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="F264" s="1" t="str">
+        <x:v>ParcelsCreatureV1</x:v>
+      </x:c>
+      <x:c r="G264" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H264" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I264" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J264" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K264" s="1" t="str">
+        <x:v>parcels-buildout/creatures/Mob_Parcels_SeedMouse.glb</x:v>
+      </x:c>
+      <x:c r="L264" s="1" t="str">
+        <x:v>f583b9ccf6db785a9866b0bbe6c5198d5c7079400f5ae40e2c8ca48153a0c071</x:v>
+      </x:c>
+      <x:c r="M264" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N264" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O264" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P264" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q264" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265" ht="38" customHeight="1">
+      <x:c r="A265" s="1" t="str">
+        <x:v>Prop_Parcels_FieldTile</x:v>
+      </x:c>
+      <x:c r="B265" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C265" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D265" s="5" t="str">
+        <x:v>Field module</x:v>
+      </x:c>
+      <x:c r="E265" s="7" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F265" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G265" s="5" t="str"/>
+      <x:c r="H265" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I265" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J265" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K265" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_FieldTile.glb</x:v>
+      </x:c>
+      <x:c r="L265" s="1" t="str">
+        <x:v>6c3e1cc89b9fe29409e4693d1197e7f2fb55126d812189a3088a3f65c178abdd</x:v>
+      </x:c>
+      <x:c r="M265" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N265" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O265" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P265" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q265" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266" ht="38" customHeight="1">
+      <x:c r="A266" s="1" t="str">
+        <x:v>Prop_Parcels_SoilBed</x:v>
+      </x:c>
+      <x:c r="B266" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C266" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D266" s="5" t="str">
+        <x:v>Crop bed</x:v>
+      </x:c>
+      <x:c r="E266" s="7" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F266" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G266" s="5" t="str"/>
+      <x:c r="H266" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I266" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J266" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K266" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_SoilBed.glb</x:v>
+      </x:c>
+      <x:c r="L266" s="1" t="str">
+        <x:v>79241dd7f293636556abf06db2d84bb9b1acca300ee38beb72b7efac205d4ea8</x:v>
+      </x:c>
+      <x:c r="M266" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N266" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O266" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P266" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q266" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267" ht="38" customHeight="1">
+      <x:c r="A267" s="1" t="str">
+        <x:v>Prop_Parcels_RoadTile</x:v>
+      </x:c>
+      <x:c r="B267" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C267" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D267" s="5" t="str">
+        <x:v>Travel road module</x:v>
+      </x:c>
+      <x:c r="E267" s="7" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F267" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G267" s="5" t="str"/>
+      <x:c r="H267" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I267" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J267" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K267" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_RoadTile.glb</x:v>
+      </x:c>
+      <x:c r="L267" s="1" t="str">
+        <x:v>545011c4a20f904b6ebf7c629ae278780f962a51e5d626eb795ae18deafb95c3</x:v>
+      </x:c>
+      <x:c r="M267" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N267" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O267" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P267" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q267" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268" ht="38" customHeight="1">
+      <x:c r="A268" s="1" t="str">
+        <x:v>Prop_Parcels_Fence</x:v>
+      </x:c>
+      <x:c r="B268" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C268" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D268" s="5" t="str">
+        <x:v>Boundary module</x:v>
+      </x:c>
+      <x:c r="E268" s="7" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F268" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G268" s="5" t="str"/>
+      <x:c r="H268" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I268" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J268" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K268" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Fence.glb</x:v>
+      </x:c>
+      <x:c r="L268" s="1" t="str">
+        <x:v>84f320a651da081a0d6ead2a1618cd795d8aa5f706ceba7b13243cab5398f1db</x:v>
+      </x:c>
+      <x:c r="M268" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N268" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O268" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P268" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q268" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269" ht="38" customHeight="1">
+      <x:c r="A269" s="1" t="str">
+        <x:v>Prop_Parcels_FarmGate</x:v>
+      </x:c>
+      <x:c r="B269" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C269" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D269" s="5" t="str">
+        <x:v>Farm entry</x:v>
+      </x:c>
+      <x:c r="E269" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F269" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G269" s="5" t="str"/>
+      <x:c r="H269" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I269" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J269" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K269" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_FarmGate.glb</x:v>
+      </x:c>
+      <x:c r="L269" s="1" t="str">
+        <x:v>afd5e0a2e760c0033a564700e739c29e8427d71ca7f7c5bedfcfbf28ab3d3c36</x:v>
+      </x:c>
+      <x:c r="M269" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N269" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O269" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P269" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q269" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270" ht="38" customHeight="1">
+      <x:c r="A270" s="1" t="str">
+        <x:v>Prop_Parcels_BarnWall</x:v>
+      </x:c>
+      <x:c r="B270" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C270" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D270" s="5" t="str">
+        <x:v>Farm wall</x:v>
+      </x:c>
+      <x:c r="E270" s="7" t="n">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="F270" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G270" s="5" t="str"/>
+      <x:c r="H270" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I270" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J270" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K270" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_BarnWall.glb</x:v>
+      </x:c>
+      <x:c r="L270" s="1" t="str">
+        <x:v>0a5b02bf8c296e9d5112b1db2cc15ccfd2e8062b886aa316fa1cf36825c5d50e</x:v>
+      </x:c>
+      <x:c r="M270" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N270" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O270" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P270" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q270" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="271" ht="38" customHeight="1">
+      <x:c r="A271" s="1" t="str">
+        <x:v>Prop_Parcels_BarnDoor</x:v>
+      </x:c>
+      <x:c r="B271" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C271" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D271" s="5" t="str">
+        <x:v>Clear farm doorway</x:v>
+      </x:c>
+      <x:c r="E271" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F271" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G271" s="5" t="str"/>
+      <x:c r="H271" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I271" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J271" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K271" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_BarnDoor.glb</x:v>
+      </x:c>
+      <x:c r="L271" s="1" t="str">
+        <x:v>b69acaecd3a941a67b2123106abc1a2b459e0ddb08edf9aa6d31a49b830a7ea9</x:v>
+      </x:c>
+      <x:c r="M271" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N271" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O271" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P271" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q271" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272" ht="38" customHeight="1">
+      <x:c r="A272" s="1" t="str">
+        <x:v>Prop_Parcels_HayBale</x:v>
+      </x:c>
+      <x:c r="B272" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C272" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D272" s="5" t="str">
+        <x:v>Farm supplies</x:v>
+      </x:c>
+      <x:c r="E272" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F272" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G272" s="5" t="str"/>
+      <x:c r="H272" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I272" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J272" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K272" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_HayBale.glb</x:v>
+      </x:c>
+      <x:c r="L272" s="1" t="str">
+        <x:v>9c5f842a704ffda5616e3432bb6b39d307384471890571ba531d2904a1c9cb99</x:v>
+      </x:c>
+      <x:c r="M272" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N272" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O272" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P272" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q272" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273" ht="38" customHeight="1">
+      <x:c r="A273" s="1" t="str">
+        <x:v>Prop_Parcels_SeedCrate</x:v>
+      </x:c>
+      <x:c r="B273" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C273" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D273" s="5" t="str">
+        <x:v>Seed supplies</x:v>
+      </x:c>
+      <x:c r="E273" s="7" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="F273" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G273" s="5" t="str"/>
+      <x:c r="H273" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I273" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J273" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K273" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_SeedCrate.glb</x:v>
+      </x:c>
+      <x:c r="L273" s="1" t="str">
+        <x:v>91922c867f8e5194a59ff4237670c6ae82fe7fd9f2563888a0b0020cb2af0388</x:v>
+      </x:c>
+      <x:c r="M273" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N273" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O273" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P273" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q273" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" ht="38" customHeight="1">
+      <x:c r="A274" s="1" t="str">
+        <x:v>Prop_Parcels_Mailbox</x:v>
+      </x:c>
+      <x:c r="B274" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C274" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D274" s="5" t="str">
+        <x:v>Delivery station</x:v>
+      </x:c>
+      <x:c r="E274" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F274" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G274" s="5" t="str"/>
+      <x:c r="H274" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I274" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J274" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K274" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Mailbox.glb</x:v>
+      </x:c>
+      <x:c r="L274" s="1" t="str">
+        <x:v>1c1666afc31eaee3a50bf69a1be634d705c7597d53a24289491f02168b2f67fc</x:v>
+      </x:c>
+      <x:c r="M274" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N274" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O274" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P274" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q274" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="275" ht="38" customHeight="1">
+      <x:c r="A275" s="1" t="str">
+        <x:v>Prop_Parcels_PostCounter</x:v>
+      </x:c>
+      <x:c r="B275" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C275" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D275" s="5" t="str">
+        <x:v>Mail station</x:v>
+      </x:c>
+      <x:c r="E275" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F275" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G275" s="5" t="str"/>
+      <x:c r="H275" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I275" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J275" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K275" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_PostCounter.glb</x:v>
+      </x:c>
+      <x:c r="L275" s="1" t="str">
+        <x:v>1594743955760261bc81d29ff121f673cd5a1cdef1f70e33da1b1209b1c51de3</x:v>
+      </x:c>
+      <x:c r="M275" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N275" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O275" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P275" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q275" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="276" ht="38" customHeight="1">
+      <x:c r="A276" s="1" t="str">
+        <x:v>Prop_Parcels_Noticeboard</x:v>
+      </x:c>
+      <x:c r="B276" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C276" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D276" s="5" t="str">
+        <x:v>Quest board</x:v>
+      </x:c>
+      <x:c r="E276" s="7" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F276" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G276" s="5" t="str"/>
+      <x:c r="H276" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I276" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J276" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K276" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Noticeboard.glb</x:v>
+      </x:c>
+      <x:c r="L276" s="1" t="str">
+        <x:v>97617bdf8438491654318c3185b3133bcd2754388f85fd0b4f58de438b4be2ae</x:v>
+      </x:c>
+      <x:c r="M276" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N276" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O276" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P276" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q276" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="277" ht="38" customHeight="1">
+      <x:c r="A277" s="1" t="str">
+        <x:v>Prop_Parcels_SurveyMarker</x:v>
+      </x:c>
+      <x:c r="B277" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C277" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D277" s="5" t="str">
+        <x:v>Survey presentation; no deed authority</x:v>
+      </x:c>
+      <x:c r="E277" s="7" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F277" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G277" s="5" t="str"/>
+      <x:c r="H277" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I277" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J277" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K277" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_SurveyMarker.glb</x:v>
+      </x:c>
+      <x:c r="L277" s="1" t="str">
+        <x:v>22144dc4804a9facc340c8187228a139abb22cb1d7d22d5bde258392e9d2cc26</x:v>
+      </x:c>
+      <x:c r="M277" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N277" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O277" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P277" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q277" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="278" ht="38" customHeight="1">
+      <x:c r="A278" s="1" t="str">
+        <x:v>Prop_Parcels_WeatherVane</x:v>
+      </x:c>
+      <x:c r="B278" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C278" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D278" s="5" t="str">
+        <x:v>Weather station</x:v>
+      </x:c>
+      <x:c r="E278" s="7" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="F278" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G278" s="5" t="str"/>
+      <x:c r="H278" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I278" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J278" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K278" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_WeatherVane.glb</x:v>
+      </x:c>
+      <x:c r="L278" s="1" t="str">
+        <x:v>370cbc1e1196234fb2190b1a33aeb03bbf1dbd87068e67c831a6ca16cf9675ea</x:v>
+      </x:c>
+      <x:c r="M278" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N278" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O278" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P278" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q278" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="279" ht="38" customHeight="1">
+      <x:c r="A279" s="1" t="str">
+        <x:v>Prop_Parcels_Beehive</x:v>
+      </x:c>
+      <x:c r="B279" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C279" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D279" s="5" t="str">
+        <x:v>Bee station</x:v>
+      </x:c>
+      <x:c r="E279" s="7" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F279" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G279" s="5" t="str"/>
+      <x:c r="H279" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I279" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J279" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K279" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Beehive.glb</x:v>
+      </x:c>
+      <x:c r="L279" s="1" t="str">
+        <x:v>d5d9c96eae2696b8d94da3b57a1ec836fd30f4e9338e327774850f1fda63305b</x:v>
+      </x:c>
+      <x:c r="M279" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N279" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O279" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P279" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q279" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="280" ht="38" customHeight="1">
+      <x:c r="A280" s="1" t="str">
+        <x:v>Prop_Parcels_MilkCart</x:v>
+      </x:c>
+      <x:c r="B280" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C280" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D280" s="5" t="str">
+        <x:v>Transport/cart station</x:v>
+      </x:c>
+      <x:c r="E280" s="7" t="n">
+        <x:v>536</x:v>
+      </x:c>
+      <x:c r="F280" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G280" s="5" t="str"/>
+      <x:c r="H280" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I280" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J280" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K280" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_MilkCart.glb</x:v>
+      </x:c>
+      <x:c r="L280" s="1" t="str">
+        <x:v>34e55e04d0387bf7bbf94113e356e2427ce3fc2f2a9ee5e89c8fdc6da0868d80</x:v>
+      </x:c>
+      <x:c r="M280" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N280" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O280" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P280" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q280" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="281" ht="38" customHeight="1">
+      <x:c r="A281" s="1" t="str">
+        <x:v>Prop_Parcels_RainCollector</x:v>
+      </x:c>
+      <x:c r="B281" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C281" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D281" s="5" t="str">
+        <x:v>Water collection presentation</x:v>
+      </x:c>
+      <x:c r="E281" s="7" t="n">
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="F281" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G281" s="5" t="str"/>
+      <x:c r="H281" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I281" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J281" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K281" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_RainCollector.glb</x:v>
+      </x:c>
+      <x:c r="L281" s="1" t="str">
+        <x:v>d82aa60833d2e457276cd17d7a2d2e4ff464b07ca5b93281290c4ee4106d5e47</x:v>
+      </x:c>
+      <x:c r="M281" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N281" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O281" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P281" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q281" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="282" ht="38" customHeight="1">
+      <x:c r="A282" s="1" t="str">
+        <x:v>Prop_Parcels_Well</x:v>
+      </x:c>
+      <x:c r="B282" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C282" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D282" s="5" t="str">
+        <x:v>Water source</x:v>
+      </x:c>
+      <x:c r="E282" s="7" t="n">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="F282" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G282" s="5" t="str"/>
+      <x:c r="H282" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I282" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J282" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K282" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Well.glb</x:v>
+      </x:c>
+      <x:c r="L282" s="1" t="str">
+        <x:v>09eef49d47939905c11c9f5641bbce56ff251794d92a12b21387540e78663e6f</x:v>
+      </x:c>
+      <x:c r="M282" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N282" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O282" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P282" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q282" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="283" ht="38" customHeight="1">
+      <x:c r="A283" s="1" t="str">
+        <x:v>Prop_Parcels_Helipad</x:v>
+      </x:c>
+      <x:c r="B283" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C283" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D283" s="5" t="str">
+        <x:v>Mount departure presentation</x:v>
+      </x:c>
+      <x:c r="E283" s="7" t="n">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="F283" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G283" s="5" t="str"/>
+      <x:c r="H283" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I283" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J283" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K283" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_Helipad.glb</x:v>
+      </x:c>
+      <x:c r="L283" s="1" t="str">
+        <x:v>f77149bf5c8241b551c574369ec597e6610c77d70da94e43c045339fe05ea207</x:v>
+      </x:c>
+      <x:c r="M283" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N283" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O283" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P283" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q283" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="284" ht="38" customHeight="1">
+      <x:c r="A284" s="1" t="str">
+        <x:v>Prop_Parcels_FuelPump</x:v>
+      </x:c>
+      <x:c r="B284" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C284" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D284" s="5" t="str">
+        <x:v>Vehicle service station</x:v>
+      </x:c>
+      <x:c r="E284" s="7" t="n">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="F284" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G284" s="5" t="str"/>
+      <x:c r="H284" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I284" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J284" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K284" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_FuelPump.glb</x:v>
+      </x:c>
+      <x:c r="L284" s="1" t="str">
+        <x:v>7ce8b4952c792f2f06b4b13ed34af2f7e1162b7ce20e069a724d9182bdc57683</x:v>
+      </x:c>
+      <x:c r="M284" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N284" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O284" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P284" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q284" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="285" ht="38" customHeight="1">
+      <x:c r="A285" s="1" t="str">
+        <x:v>Prop_Parcels_MarketStall</x:v>
+      </x:c>
+      <x:c r="B285" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C285" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D285" s="5" t="str">
+        <x:v>Market station</x:v>
+      </x:c>
+      <x:c r="E285" s="7" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F285" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G285" s="5" t="str"/>
+      <x:c r="H285" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I285" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J285" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K285" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_MarketStall.glb</x:v>
+      </x:c>
+      <x:c r="L285" s="1" t="str">
+        <x:v>5de855bfde4d528ff45f51d3093af4ff3b6f74e0b33eb8195f2dac96edae65cc</x:v>
+      </x:c>
+      <x:c r="M285" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N285" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O285" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P285" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q285" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="286" ht="38" customHeight="1">
+      <x:c r="A286" s="1" t="str">
+        <x:v>Prop_Parcels_BoatDock</x:v>
+      </x:c>
+      <x:c r="B286" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C286" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D286" s="5" t="str">
+        <x:v>Ocean departure dock</x:v>
+      </x:c>
+      <x:c r="E286" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F286" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G286" s="5" t="str"/>
+      <x:c r="H286" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I286" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J286" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K286" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_BoatDock.glb</x:v>
+      </x:c>
+      <x:c r="L286" s="1" t="str">
+        <x:v>225540ee703e522e8a85ce070936fb43240d32962ee67c7dac34c4096ae09a9b</x:v>
+      </x:c>
+      <x:c r="M286" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N286" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O286" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P286" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q286" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="287" ht="38" customHeight="1">
+      <x:c r="A287" s="1" t="str">
+        <x:v>Prop_Parcels_UnderwaterAirlock</x:v>
+      </x:c>
+      <x:c r="B287" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C287" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D287" s="5" t="str">
+        <x:v>Ocean arrival presentation</x:v>
+      </x:c>
+      <x:c r="E287" s="7" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="F287" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G287" s="5" t="str"/>
+      <x:c r="H287" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I287" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J287" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K287" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Parcels_UnderwaterAirlock.glb</x:v>
+      </x:c>
+      <x:c r="L287" s="1" t="str">
+        <x:v>7f229b166819f3fd95d3fa4cf030133bbda41e7f5b197fd75d029b5db8cbe6be</x:v>
+      </x:c>
+      <x:c r="M287" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N287" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O287" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P287" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q287" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="288" ht="38" customHeight="1">
+      <x:c r="A288" s="1" t="str">
+        <x:v>Prop_Water_AMF_Trough_V12</x:v>
+      </x:c>
+      <x:c r="B288" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C288" s="1" t="str">
+        <x:v>The Parcels</x:v>
+      </x:c>
+      <x:c r="D288" s="5" t="str">
+        <x:v>Existing AMF trough geometry reuse; behavior not copied</x:v>
+      </x:c>
+      <x:c r="E288" s="7" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F288" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G288" s="5" t="str"/>
+      <x:c r="H288" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I288" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J288" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K288" s="1" t="str">
+        <x:v>parcels-buildout/environment/Prop_Water_AMF_Trough_V12.glb</x:v>
+      </x:c>
+      <x:c r="L288" s="1" t="str">
+        <x:v>a8ad48d5354e7a08af59fcd08d173ab8dac655b576988eac525721dbff0720d6</x:v>
+      </x:c>
+      <x:c r="M288" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N288" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O288" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P288" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q288" s="5" t="str">
+        <x:v>Reused original AMF; owner retained</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="8">
+  <x:dataValidations count="10">
     <x:dataValidation type="list" sqref="I6:I72">
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
@@ -11817,6 +14751,12 @@
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J190:J232">
+      <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I233:I288">
+      <x:formula1>"Pending,Imported,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J233:J288">
       <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -12615,12 +15555,22 @@
       <x:c r="K34" s="2"/>
       <x:c r="L34" s="2"/>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="2"/>
-      <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
-      <x:c r="D35" s="2"/>
-      <x:c r="E35" s="2"/>
+    <x:row r="35" ht="52" customHeight="1">
+      <x:c r="A35" s="2" t="str">
+        <x:v>PAR01</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>Mail, farming and boundary guidance</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>32 cast/creature/mount/pet role models</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="str">
+        <x:v>Art validated; behaviors pending</x:v>
+      </x:c>
+      <x:c r="E35" s="4" t="str">
+        <x:v>Help neighbours and reconnect isolated plots</x:v>
+      </x:c>
       <x:c r="F35" s="2"/>
       <x:c r="G35" s="2"/>
       <x:c r="H35" s="2"/>
@@ -12629,12 +15579,22 @@
       <x:c r="K35" s="2"/>
       <x:c r="L35" s="2"/>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="2"/>
-      <x:c r="B36" s="2"/>
-      <x:c r="C36" s="2"/>
-      <x:c r="D36" s="2"/>
-      <x:c r="E36" s="2"/>
+    <x:row r="36" ht="52" customHeight="1">
+      <x:c r="A36" s="2" t="str">
+        <x:v>PAR02</x:v>
+      </x:c>
+      <x:c r="B36" s="4" t="str">
+        <x:v>Roads, fields, mail stations, helipad and ocean docks</x:v>
+      </x:c>
+      <x:c r="C36" s="4" t="str">
+        <x:v>23 original props + one reused AMF trough</x:v>
+      </x:c>
+      <x:c r="D36" s="4" t="str">
+        <x:v>Static validation; interactions/transport pending</x:v>
+      </x:c>
+      <x:c r="E36" s="4" t="str">
+        <x:v>Farm roads connect village work to wider journeys</x:v>
+      </x:c>
       <x:c r="F36" s="2"/>
       <x:c r="G36" s="2"/>
       <x:c r="H36" s="2"/>
@@ -12643,12 +15603,22 @@
       <x:c r="K36" s="2"/>
       <x:c r="L36" s="2"/>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="2"/>
-      <x:c r="B37" s="2"/>
-      <x:c r="C37" s="2"/>
-      <x:c r="D37" s="2"/>
-      <x:c r="E37" s="2"/>
+    <x:row r="37" ht="52" customHeight="1">
+      <x:c r="A37" s="2" t="str">
+        <x:v>PAR03</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>Reuse existing geometry without copying authority</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>Original AMF trough ID/SHA retained</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="str">
+        <x:v>No tonic transaction behavior inherited</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>Water supplies and companion care use explicit host rules</x:v>
+      </x:c>
       <x:c r="F37" s="2"/>
       <x:c r="G37" s="2"/>
       <x:c r="H37" s="2"/>

</xml_diff>

<commit_message>
Complete Brick modular art kit and production register
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R0d6ccfa970be4c07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R95944fd561cf436b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Ra283ac5bb0944d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R4588cbaccfdb4826"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R50679d0f83dd4d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R884ef78873444bf6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,7 +40,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,6 +50,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243746"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -85,7 +90,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -141,6 +146,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -468,15 +474,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -484,7 +490,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -503,15 +509,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A8)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A8)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="2" t="n">
@@ -519,7 +525,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A8)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
@@ -538,15 +544,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -554,7 +560,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A9)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9)</x:f>
         <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
@@ -573,24 +579,24 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A10)</x:f>
-        <x:v>0</x:v>
+        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A10)</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="2" t="n">
         <x:f>C10-D10</x:f>
-        <x:v>32</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A10)</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
@@ -608,15 +614,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$288,Assets!$C$6:$C$288,A11)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A11)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11,Assets!$B$6:$B$288,"Character",Assets!$H$6:$H$288,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11,Assets!$B$6:$B$288,"Character",Assets!$I$6:$I$288,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="2" t="n">
@@ -624,7 +630,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$288,A11)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
@@ -665,8 +671,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E288)</x:f>
-        <x:v>265360</x:v>
+        <x:f>SUM(Assets!E6:E344)</x:f>
+        <x:v>311464</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -684,8 +690,8 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B288,"Prop")+COUNTIFS(Assets!B6:B288,"Item")</x:f>
-        <x:v>107</x:v>
+        <x:f>COUNTIFS(Assets!B6:B344,"Prop")+COUNTIFS(Assets!B6:B344,"Item")</x:f>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -714,7 +720,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Codex kits: 283 unique asset references, including one unchanged AMF reuse. Export validation is not Play proof.</x:v>
+        <x:v>Codex kits: 339 unique asset references, including one unchanged AMF reuse. Export validation is not Play proof.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -1567,7 +1573,7 @@
       <x:c r="P5" s="19" t="str">
         <x:v>LOD level</x:v>
       </x:c>
-      <x:c r="Q5" s="23" t="str">
+      <x:c r="Q5" s="25" t="str">
         <x:v>Provenance</x:v>
       </x:c>
     </x:row>
@@ -14727,8 +14733,2928 @@
         <x:v>Reused original AMF; owner retained</x:v>
       </x:c>
     </x:row>
+    <x:row r="289" ht="38" customHeight="1">
+      <x:c r="A289" s="1" t="str">
+        <x:v>Mob_Bricks_Builder</x:v>
+      </x:c>
+      <x:c r="B289" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C289" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D289" s="5" t="str">
+        <x:v>Hero builder</x:v>
+      </x:c>
+      <x:c r="E289" s="7" t="n">
+        <x:v>1216</x:v>
+      </x:c>
+      <x:c r="F289" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G289" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H289" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I289" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J289" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K289" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_Builder.glb</x:v>
+      </x:c>
+      <x:c r="L289" s="1" t="str">
+        <x:v>cd0190074cb291f9c650970b0d51088b814afc511e2d7c12a411386a9877ce7c</x:v>
+      </x:c>
+      <x:c r="M289" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N289" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O289" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P289" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q289" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="290" ht="38" customHeight="1">
+      <x:c r="A290" s="1" t="str">
+        <x:v>Mob_Bricks_ForemanKip</x:v>
+      </x:c>
+      <x:c r="B290" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C290" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D290" s="5" t="str">
+        <x:v>Blueprint quest guide</x:v>
+      </x:c>
+      <x:c r="E290" s="7" t="n">
+        <x:v>1128</x:v>
+      </x:c>
+      <x:c r="F290" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G290" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H290" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I290" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J290" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K290" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_ForemanKip.glb</x:v>
+      </x:c>
+      <x:c r="L290" s="1" t="str">
+        <x:v>4c9ca83b0a83d80123cc39a1422a176663a60022836d72c1d4a5c0dd98ed2e79</x:v>
+      </x:c>
+      <x:c r="M290" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N290" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O290" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P290" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q290" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="291" ht="38" customHeight="1">
+      <x:c r="A291" s="1" t="str">
+        <x:v>Mob_Bricks_BrickBaker</x:v>
+      </x:c>
+      <x:c r="B291" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C291" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D291" s="5" t="str">
+        <x:v>Kiln crafting guide</x:v>
+      </x:c>
+      <x:c r="E291" s="7" t="n">
+        <x:v>1128</x:v>
+      </x:c>
+      <x:c r="F291" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G291" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H291" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I291" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J291" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K291" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_BrickBaker.glb</x:v>
+      </x:c>
+      <x:c r="L291" s="1" t="str">
+        <x:v>327660d01b75d19fc82df85f226bd706b4801000bca22e8e44e89ff295c50846</x:v>
+      </x:c>
+      <x:c r="M291" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N291" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O291" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P291" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q291" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="292" ht="38" customHeight="1">
+      <x:c r="A292" s="1" t="str">
+        <x:v>Mob_Bricks_BlueprintArchivist</x:v>
+      </x:c>
+      <x:c r="B292" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C292" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D292" s="5" t="str">
+        <x:v>Recipe archive</x:v>
+      </x:c>
+      <x:c r="E292" s="7" t="n">
+        <x:v>1136</x:v>
+      </x:c>
+      <x:c r="F292" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G292" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H292" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I292" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J292" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K292" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_BlueprintArchivist.glb</x:v>
+      </x:c>
+      <x:c r="L292" s="1" t="str">
+        <x:v>75f0115befab85399b25695b811c775d7bf9e1f147b37b79f36eb7356c27640d</x:v>
+      </x:c>
+      <x:c r="M292" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N292" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O292" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P292" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q292" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="293" ht="38" customHeight="1">
+      <x:c r="A293" s="1" t="str">
+        <x:v>Mob_Bricks_CraneOperatorSal</x:v>
+      </x:c>
+      <x:c r="B293" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C293" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D293" s="5" t="str">
+        <x:v>Structure crew</x:v>
+      </x:c>
+      <x:c r="E293" s="7" t="n">
+        <x:v>1164</x:v>
+      </x:c>
+      <x:c r="F293" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G293" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H293" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I293" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J293" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K293" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_CraneOperatorSal.glb</x:v>
+      </x:c>
+      <x:c r="L293" s="1" t="str">
+        <x:v>9f2b31bcdeb009de16b2bc261697a992bf3cc8fcc86f7e8686011eb2400efd38</x:v>
+      </x:c>
+      <x:c r="M293" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N293" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O293" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P293" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q293" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="294" ht="38" customHeight="1">
+      <x:c r="A294" s="1" t="str">
+        <x:v>Mob_Bricks_DemolitionDuo</x:v>
+      </x:c>
+      <x:c r="B294" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C294" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D294" s="5" t="str">
+        <x:v>Demolition challenge representative</x:v>
+      </x:c>
+      <x:c r="E294" s="7" t="n">
+        <x:v>1172</x:v>
+      </x:c>
+      <x:c r="F294" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G294" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H294" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I294" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J294" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K294" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_DemolitionDuo.glb</x:v>
+      </x:c>
+      <x:c r="L294" s="1" t="str">
+        <x:v>fdc73301fa1c5b2c51d0806c5dd3a79989783151d76d7aa0a6405201cc1557c2</x:v>
+      </x:c>
+      <x:c r="M294" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N294" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O294" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P294" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q294" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="295" ht="38" customHeight="1">
+      <x:c r="A295" s="1" t="str">
+        <x:v>Mob_Bricks_MayorMinifold</x:v>
+      </x:c>
+      <x:c r="B295" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C295" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D295" s="5" t="str">
+        <x:v>Town quest guide</x:v>
+      </x:c>
+      <x:c r="E295" s="7" t="n">
+        <x:v>1164</x:v>
+      </x:c>
+      <x:c r="F295" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G295" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H295" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I295" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J295" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K295" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_MayorMinifold.glb</x:v>
+      </x:c>
+      <x:c r="L295" s="1" t="str">
+        <x:v>06af1f551ac265140945ed4f7a19775b9a6a540ee403efb4028698d00a651b42</x:v>
+      </x:c>
+      <x:c r="M295" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N295" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O295" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P295" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q295" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296" ht="38" customHeight="1">
+      <x:c r="A296" s="1" t="str">
+        <x:v>Mob_Bricks_AirfieldAceNova</x:v>
+      </x:c>
+      <x:c r="B296" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C296" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D296" s="5" t="str">
+        <x:v>Plane mount guide</x:v>
+      </x:c>
+      <x:c r="E296" s="7" t="n">
+        <x:v>1136</x:v>
+      </x:c>
+      <x:c r="F296" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G296" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H296" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I296" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J296" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K296" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_AirfieldAceNova.glb</x:v>
+      </x:c>
+      <x:c r="L296" s="1" t="str">
+        <x:v>c7e86e1cd87d62f4dff6b259d02c82dd712b0985288876cc19d0481088aab34f</x:v>
+      </x:c>
+      <x:c r="M296" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N296" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O296" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P296" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q296" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="297" ht="38" customHeight="1">
+      <x:c r="A297" s="1" t="str">
+        <x:v>Mob_Bricks_ToySoldierSergeant</x:v>
+      </x:c>
+      <x:c r="B297" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C297" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D297" s="5" t="str">
+        <x:v>Tactics guide</x:v>
+      </x:c>
+      <x:c r="E297" s="7" t="n">
+        <x:v>1154</x:v>
+      </x:c>
+      <x:c r="F297" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G297" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H297" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I297" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J297" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K297" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_ToySoldierSergeant.glb</x:v>
+      </x:c>
+      <x:c r="L297" s="1" t="str">
+        <x:v>69d78a3423f860743e4529cdf1e700f858e085861d9a2195262f1acf0836b792</x:v>
+      </x:c>
+      <x:c r="M297" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N297" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O297" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P297" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q297" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="38" customHeight="1">
+      <x:c r="A298" s="1" t="str">
+        <x:v>Mob_Bricks_MissingPieceCollector</x:v>
+      </x:c>
+      <x:c r="B298" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C298" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D298" s="5" t="str">
+        <x:v>Collection quests</x:v>
+      </x:c>
+      <x:c r="E298" s="7" t="n">
+        <x:v>1328</x:v>
+      </x:c>
+      <x:c r="F298" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G298" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H298" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I298" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J298" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K298" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_MissingPieceCollector.glb</x:v>
+      </x:c>
+      <x:c r="L298" s="1" t="str">
+        <x:v>1a6c00909fd8912660abf1abf0b95a89a4a026e61e135b36e2bda54ce05728c6</x:v>
+      </x:c>
+      <x:c r="M298" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N298" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O298" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P298" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q298" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="38" customHeight="1">
+      <x:c r="A299" s="1" t="str">
+        <x:v>Mob_Bricks_AdhesiveAlchemist</x:v>
+      </x:c>
+      <x:c r="B299" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C299" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D299" s="5" t="str">
+        <x:v>NonHalloween Glue Witch art reinterpretation</x:v>
+      </x:c>
+      <x:c r="E299" s="7" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="F299" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G299" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H299" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I299" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J299" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K299" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_AdhesiveAlchemist.glb</x:v>
+      </x:c>
+      <x:c r="L299" s="1" t="str">
+        <x:v>fa368584812713c48cda24cfe165d3501eed4f46793614ef6d1a84f6637e92d4</x:v>
+      </x:c>
+      <x:c r="M299" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N299" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O299" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P299" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q299" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="38" customHeight="1">
+      <x:c r="A300" s="1" t="str">
+        <x:v>Mob_Bricks_Studmonger</x:v>
+      </x:c>
+      <x:c r="B300" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C300" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D300" s="5" t="str">
+        <x:v>Realm game-currency exchange presentation</x:v>
+      </x:c>
+      <x:c r="E300" s="7" t="n">
+        <x:v>1276</x:v>
+      </x:c>
+      <x:c r="F300" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G300" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H300" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I300" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J300" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K300" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_Studmonger.glb</x:v>
+      </x:c>
+      <x:c r="L300" s="1" t="str">
+        <x:v>dac3022f30e5c97288f2f2bf9b04ad166e5b8ddcbf5a83d2615f43442ed3c692</x:v>
+      </x:c>
+      <x:c r="M300" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N300" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O300" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P300" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q300" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="38" customHeight="1">
+      <x:c r="A301" s="1" t="str">
+        <x:v>Mob_Bricks_BuilderKidsClub</x:v>
+      </x:c>
+      <x:c r="B301" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C301" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D301" s="5" t="str">
+        <x:v>Club representative</x:v>
+      </x:c>
+      <x:c r="E301" s="7" t="n">
+        <x:v>1128</x:v>
+      </x:c>
+      <x:c r="F301" s="1" t="str">
+        <x:v>BrickHumanoidV1</x:v>
+      </x:c>
+      <x:c r="G301" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H301" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I301" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J301" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K301" s="1" t="str">
+        <x:v>bricks-buildout/cast/Mob_Bricks_BuilderKidsClub.glb</x:v>
+      </x:c>
+      <x:c r="L301" s="1" t="str">
+        <x:v>c7ad6614e1334918da565cd27a9ee4a61321cc38a56216c89a573eefd18c58ca</x:v>
+      </x:c>
+      <x:c r="M301" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N301" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O301" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P301" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q301" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="38" customHeight="1">
+      <x:c r="A302" s="1" t="str">
+        <x:v>Mob_Bricks_Brickbug</x:v>
+      </x:c>
+      <x:c r="B302" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C302" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D302" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E302" s="7" t="n">
+        <x:v>1448</x:v>
+      </x:c>
+      <x:c r="F302" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G302" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H302" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I302" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J302" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K302" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_Brickbug.glb</x:v>
+      </x:c>
+      <x:c r="L302" s="1" t="str">
+        <x:v>91a5cb0c754180222f2b2f841f5824acd48fd6fed4c38e29e323da3e490e7516</x:v>
+      </x:c>
+      <x:c r="M302" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N302" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O302" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P302" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q302" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="38" customHeight="1">
+      <x:c r="A303" s="1" t="str">
+        <x:v>Mob_Bricks_LooseStud</x:v>
+      </x:c>
+      <x:c r="B303" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C303" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D303" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E303" s="7" t="n">
+        <x:v>1128</x:v>
+      </x:c>
+      <x:c r="F303" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G303" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H303" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I303" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J303" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K303" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_LooseStud.glb</x:v>
+      </x:c>
+      <x:c r="L303" s="1" t="str">
+        <x:v>28a87b1a8b1e1fe1359f65f3becd3e8909e37fe26fd22ff6d373ec6d3f6b0877</x:v>
+      </x:c>
+      <x:c r="M303" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N303" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O303" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P303" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q303" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="38" customHeight="1">
+      <x:c r="A304" s="1" t="str">
+        <x:v>Mob_Bricks_PlateCrab</x:v>
+      </x:c>
+      <x:c r="B304" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C304" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D304" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E304" s="7" t="n">
+        <x:v>1560</x:v>
+      </x:c>
+      <x:c r="F304" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G304" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H304" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I304" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J304" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K304" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_PlateCrab.glb</x:v>
+      </x:c>
+      <x:c r="L304" s="1" t="str">
+        <x:v>37df4b8ff849f1bacacfb26b8c77e3a7ebc119d03adaba6d001ed6505e5fdd3f</x:v>
+      </x:c>
+      <x:c r="M304" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N304" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O304" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P304" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q304" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="38" customHeight="1">
+      <x:c r="A305" s="1" t="str">
+        <x:v>Mob_Bricks_HingeHound</x:v>
+      </x:c>
+      <x:c r="B305" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C305" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D305" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E305" s="7" t="n">
+        <x:v>1448</x:v>
+      </x:c>
+      <x:c r="F305" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G305" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H305" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I305" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J305" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K305" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_HingeHound.glb</x:v>
+      </x:c>
+      <x:c r="L305" s="1" t="str">
+        <x:v>68e9781ee2167d8b376f50d5571154ee9c9408ba1f32ac407046133fffb21e73</x:v>
+      </x:c>
+      <x:c r="M305" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N305" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O305" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P305" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q305" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="38" customHeight="1">
+      <x:c r="A306" s="1" t="str">
+        <x:v>Mob_Bricks_SlopeSlug</x:v>
+      </x:c>
+      <x:c r="B306" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C306" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D306" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E306" s="7" t="n">
+        <x:v>1228</x:v>
+      </x:c>
+      <x:c r="F306" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G306" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H306" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I306" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J306" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K306" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_SlopeSlug.glb</x:v>
+      </x:c>
+      <x:c r="L306" s="1" t="str">
+        <x:v>b2fcd6a2d8a18c1a901a7afb9129bb1d8708788c13597d5883d52cd7172d5d38</x:v>
+      </x:c>
+      <x:c r="M306" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N306" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O306" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P306" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q306" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="38" customHeight="1">
+      <x:c r="A307" s="1" t="str">
+        <x:v>Mob_Bricks_RebuildRex</x:v>
+      </x:c>
+      <x:c r="B307" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C307" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D307" s="5" t="str">
+        <x:v>Boss proposal</x:v>
+      </x:c>
+      <x:c r="E307" s="7" t="n">
+        <x:v>1466</x:v>
+      </x:c>
+      <x:c r="F307" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G307" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H307" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I307" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J307" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K307" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_RebuildRex.glb</x:v>
+      </x:c>
+      <x:c r="L307" s="1" t="str">
+        <x:v>c22f01f3e5352f0e28c502431f08434831c05379999dc9e5bb4b04635f1f1f3c</x:v>
+      </x:c>
+      <x:c r="M307" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N307" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O307" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P307" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q307" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="38" customHeight="1">
+      <x:c r="A308" s="1" t="str">
+        <x:v>Mob_Bricks_WindUpKnight</x:v>
+      </x:c>
+      <x:c r="B308" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C308" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D308" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E308" s="7" t="n">
+        <x:v>1508</x:v>
+      </x:c>
+      <x:c r="F308" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G308" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H308" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I308" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J308" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K308" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_WindUpKnight.glb</x:v>
+      </x:c>
+      <x:c r="L308" s="1" t="str">
+        <x:v>73b6a5e92cb63f4f1673e53f69810023bea7afd2c7d6b3ecbfa4a220d023f32b</x:v>
+      </x:c>
+      <x:c r="M308" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N308" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O308" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P308" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q308" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="38" customHeight="1">
+      <x:c r="A309" s="1" t="str">
+        <x:v>Mob_Bricks_TowerTitan</x:v>
+      </x:c>
+      <x:c r="B309" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C309" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D309" s="5" t="str">
+        <x:v>Boss proposal</x:v>
+      </x:c>
+      <x:c r="E309" s="7" t="n">
+        <x:v>1504</x:v>
+      </x:c>
+      <x:c r="F309" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G309" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H309" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I309" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J309" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K309" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_TowerTitan.glb</x:v>
+      </x:c>
+      <x:c r="L309" s="1" t="str">
+        <x:v>6f74988f38257a1fe828e62d4cb61fb8d9c701ae0c6c59af58dad8cc2338e7df</x:v>
+      </x:c>
+      <x:c r="M309" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N309" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O309" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P309" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q309" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="310" ht="38" customHeight="1">
+      <x:c r="A310" s="1" t="str">
+        <x:v>Mob_Bricks_MagnetMoth</x:v>
+      </x:c>
+      <x:c r="B310" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C310" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D310" s="5" t="str">
+        <x:v>Construct encounter</x:v>
+      </x:c>
+      <x:c r="E310" s="7" t="n">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="F310" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G310" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H310" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I310" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J310" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K310" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_MagnetMoth.glb</x:v>
+      </x:c>
+      <x:c r="L310" s="1" t="str">
+        <x:v>dcefaa4c4251ed626a41dcfe88b5a4b132212dab61bdfc7b1dea24840ce3c807</x:v>
+      </x:c>
+      <x:c r="M310" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N310" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O310" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P310" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q310" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="311" ht="38" customHeight="1">
+      <x:c r="A311" s="1" t="str">
+        <x:v>Mob_Bricks_Unmaker</x:v>
+      </x:c>
+      <x:c r="B311" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C311" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D311" s="5" t="str">
+        <x:v>Boss proposal; visual only, no structure authority</x:v>
+      </x:c>
+      <x:c r="E311" s="7" t="n">
+        <x:v>1260</x:v>
+      </x:c>
+      <x:c r="F311" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G311" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H311" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I311" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J311" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K311" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_Unmaker.glb</x:v>
+      </x:c>
+      <x:c r="L311" s="1" t="str">
+        <x:v>3357f980c0f10f7b072a006d3996d55ee160aabdc7d3a3d9bed30d11b4a97a96</x:v>
+      </x:c>
+      <x:c r="M311" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N311" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O311" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P311" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q311" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="312" ht="38" customHeight="1">
+      <x:c r="A312" s="1" t="str">
+        <x:v>Mob_Bricks_ClockworkPigeon</x:v>
+      </x:c>
+      <x:c r="B312" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C312" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D312" s="5" t="str">
+        <x:v>Ambient bird</x:v>
+      </x:c>
+      <x:c r="E312" s="7" t="n">
+        <x:v>1484</x:v>
+      </x:c>
+      <x:c r="F312" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G312" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H312" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I312" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J312" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K312" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_ClockworkPigeon.glb</x:v>
+      </x:c>
+      <x:c r="L312" s="1" t="str">
+        <x:v>b2384620d57338f37b06ab1bbcce36ccdc2546f8a20080ce656af388c7d224ca</x:v>
+      </x:c>
+      <x:c r="M312" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N312" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O312" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P312" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q312" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="313" ht="38" customHeight="1">
+      <x:c r="A313" s="1" t="str">
+        <x:v>Mob_Bricks_SpringFrog</x:v>
+      </x:c>
+      <x:c r="B313" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C313" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D313" s="5" t="str">
+        <x:v>Ambient creature</x:v>
+      </x:c>
+      <x:c r="E313" s="7" t="n">
+        <x:v>1360</x:v>
+      </x:c>
+      <x:c r="F313" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G313" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H313" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I313" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J313" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K313" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_SpringFrog.glb</x:v>
+      </x:c>
+      <x:c r="L313" s="1" t="str">
+        <x:v>b45e929a445f028cea430c0310872093fb64a48cc41103b11a24e78e260f060f</x:v>
+      </x:c>
+      <x:c r="M313" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N313" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O313" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P313" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q313" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="314" ht="38" customHeight="1">
+      <x:c r="A314" s="1" t="str">
+        <x:v>Mob_Bricks_BrickPlane</x:v>
+      </x:c>
+      <x:c r="B314" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C314" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D314" s="5" t="str">
+        <x:v>Realm vehicle; flight pending</x:v>
+      </x:c>
+      <x:c r="E314" s="7" t="n">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="F314" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G314" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H314" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I314" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J314" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K314" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_BrickPlane.glb</x:v>
+      </x:c>
+      <x:c r="L314" s="1" t="str">
+        <x:v>a6f637b505a7dab8169a6ee9950a55b3c734fc60eb2735ce2916d8c730a50b39</x:v>
+      </x:c>
+      <x:c r="M314" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N314" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O314" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P314" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q314" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="315" ht="38" customHeight="1">
+      <x:c r="A315" s="1" t="str">
+        <x:v>Mob_Bricks_BrickPony</x:v>
+      </x:c>
+      <x:c r="B315" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C315" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D315" s="5" t="str">
+        <x:v>Realm mount</x:v>
+      </x:c>
+      <x:c r="E315" s="7" t="n">
+        <x:v>1492</x:v>
+      </x:c>
+      <x:c r="F315" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G315" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H315" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I315" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J315" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K315" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_BrickPony.glb</x:v>
+      </x:c>
+      <x:c r="L315" s="1" t="str">
+        <x:v>e0ca8af130705a5a9fd9581a737fed746f03ecc7b2ae3cf0bf9960ee7b5feccb</x:v>
+      </x:c>
+      <x:c r="M315" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N315" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O315" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P315" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q315" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="316" ht="38" customHeight="1">
+      <x:c r="A316" s="1" t="str">
+        <x:v>Mob_Bricks_HoverCart</x:v>
+      </x:c>
+      <x:c r="B316" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C316" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D316" s="5" t="str">
+        <x:v>Realm vehicle; hover physics pending</x:v>
+      </x:c>
+      <x:c r="E316" s="7" t="n">
+        <x:v>1252</x:v>
+      </x:c>
+      <x:c r="F316" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G316" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H316" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I316" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J316" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K316" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_HoverCart.glb</x:v>
+      </x:c>
+      <x:c r="L316" s="1" t="str">
+        <x:v>cba865393a63861b0776503533b8689820606bf2032bdf31beb7a39e06db6cf7</x:v>
+      </x:c>
+      <x:c r="M316" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N316" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O316" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P316" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q316" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="317" ht="38" customHeight="1">
+      <x:c r="A317" s="1" t="str">
+        <x:v>Mob_Bricks_Studpup</x:v>
+      </x:c>
+      <x:c r="B317" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C317" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D317" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E317" s="7" t="n">
+        <x:v>1640</x:v>
+      </x:c>
+      <x:c r="F317" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G317" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H317" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I317" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J317" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K317" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_Studpup.glb</x:v>
+      </x:c>
+      <x:c r="L317" s="1" t="str">
+        <x:v>16f989ff1118a967c6650449e8df03f2882d73a90dc9b8acc74c7b8179fabb56</x:v>
+      </x:c>
+      <x:c r="M317" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N317" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O317" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P317" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q317" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="318" ht="38" customHeight="1">
+      <x:c r="A318" s="1" t="str">
+        <x:v>Mob_Bricks_TileTurtle</x:v>
+      </x:c>
+      <x:c r="B318" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C318" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D318" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E318" s="7" t="n">
+        <x:v>1372</x:v>
+      </x:c>
+      <x:c r="F318" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G318" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H318" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I318" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J318" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K318" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_TileTurtle.glb</x:v>
+      </x:c>
+      <x:c r="L318" s="1" t="str">
+        <x:v>581bff04404792e130d727a90faab45cdb35fc0d2c8a7f2d6d2ff897c7118a8c</x:v>
+      </x:c>
+      <x:c r="M318" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N318" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O318" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P318" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q318" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="319" ht="38" customHeight="1">
+      <x:c r="A319" s="1" t="str">
+        <x:v>Mob_Bricks_SpinnerTop</x:v>
+      </x:c>
+      <x:c r="B319" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C319" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D319" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E319" s="7" t="n">
+        <x:v>1068</x:v>
+      </x:c>
+      <x:c r="F319" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G319" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H319" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I319" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J319" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K319" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_SpinnerTop.glb</x:v>
+      </x:c>
+      <x:c r="L319" s="1" t="str">
+        <x:v>45de044480d15c69fb398c6634bff382fff0decf0bcbf8ca5beb4593e223587b</x:v>
+      </x:c>
+      <x:c r="M319" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N319" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O319" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P319" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q319" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="320" ht="38" customHeight="1">
+      <x:c r="A320" s="1" t="str">
+        <x:v>Mob_Bricks_PocketBot</x:v>
+      </x:c>
+      <x:c r="B320" s="1" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="C320" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D320" s="5" t="str">
+        <x:v>Helpful pet</x:v>
+      </x:c>
+      <x:c r="E320" s="7" t="n">
+        <x:v>1300</x:v>
+      </x:c>
+      <x:c r="F320" s="1" t="str">
+        <x:v>BrickCreatureV1</x:v>
+      </x:c>
+      <x:c r="G320" s="5" t="str">
+        <x:v>Idle, Walk, Attack, Hurt</x:v>
+      </x:c>
+      <x:c r="H320" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I320" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J320" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K320" s="1" t="str">
+        <x:v>bricks-buildout/creatures/Mob_Bricks_PocketBot.glb</x:v>
+      </x:c>
+      <x:c r="L320" s="1" t="str">
+        <x:v>cb59f6b15eb89dbc57a9d7b164eba707a531b7a1cdc318c8844c67f7bb0fbab3</x:v>
+      </x:c>
+      <x:c r="M320" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N320" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O320" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P320" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q320" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321" ht="38" customHeight="1">
+      <x:c r="A321" s="1" t="str">
+        <x:v>Prop_Bricks_MeadowTile</x:v>
+      </x:c>
+      <x:c r="B321" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C321" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D321" s="5" t="str">
+        <x:v>Continuous meadow module</x:v>
+      </x:c>
+      <x:c r="E321" s="7" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F321" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G321" s="5" t="str"/>
+      <x:c r="H321" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I321" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J321" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K321" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_MeadowTile.glb</x:v>
+      </x:c>
+      <x:c r="L321" s="1" t="str">
+        <x:v>5cd9a36506b1a5e62fa35a2ea3e78b272906f177f950462b8b2082eecd6d167c</x:v>
+      </x:c>
+      <x:c r="M321" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N321" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O321" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P321" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q321" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322" ht="38" customHeight="1">
+      <x:c r="A322" s="1" t="str">
+        <x:v>Prop_Bricks_Baseplate</x:v>
+      </x:c>
+      <x:c r="B322" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C322" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D322" s="5" t="str">
+        <x:v>Construction floor</x:v>
+      </x:c>
+      <x:c r="E322" s="7" t="n">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="F322" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G322" s="5" t="str"/>
+      <x:c r="H322" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I322" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J322" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K322" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Baseplate.glb</x:v>
+      </x:c>
+      <x:c r="L322" s="1" t="str">
+        <x:v>a9f42f446dd6906ce27b36c20a7ba31693b4a7dc53cf8e222b5ecf17ea734dfc</x:v>
+      </x:c>
+      <x:c r="M322" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N322" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O322" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P322" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q322" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323" ht="38" customHeight="1">
+      <x:c r="A323" s="1" t="str">
+        <x:v>Prop_Bricks_RoadTile</x:v>
+      </x:c>
+      <x:c r="B323" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C323" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D323" s="5" t="str">
+        <x:v>Continuous vehicle road</x:v>
+      </x:c>
+      <x:c r="E323" s="7" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F323" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G323" s="5" t="str"/>
+      <x:c r="H323" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I323" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J323" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K323" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_RoadTile.glb</x:v>
+      </x:c>
+      <x:c r="L323" s="1" t="str">
+        <x:v>2014f4008a825dec8e000f7eee041063e898fc4c16dca704fc7c409ef616df99</x:v>
+      </x:c>
+      <x:c r="M323" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N323" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O323" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P323" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q323" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324" ht="38" customHeight="1">
+      <x:c r="A324" s="1" t="str">
+        <x:v>Prop_Bricks_Wall</x:v>
+      </x:c>
+      <x:c r="B324" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C324" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D324" s="5" t="str">
+        <x:v>Construction wall</x:v>
+      </x:c>
+      <x:c r="E324" s="7" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="F324" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G324" s="5" t="str"/>
+      <x:c r="H324" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I324" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J324" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K324" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Wall.glb</x:v>
+      </x:c>
+      <x:c r="L324" s="1" t="str">
+        <x:v>24277edf78515ec6271a2a80778758b864af5e1157e5a357f38d604a4712fff0</x:v>
+      </x:c>
+      <x:c r="M324" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N324" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O324" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P324" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q324" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325" ht="38" customHeight="1">
+      <x:c r="A325" s="1" t="str">
+        <x:v>Prop_Bricks_WindowWall</x:v>
+      </x:c>
+      <x:c r="B325" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C325" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D325" s="5" t="str">
+        <x:v>Window module</x:v>
+      </x:c>
+      <x:c r="E325" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F325" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G325" s="5" t="str"/>
+      <x:c r="H325" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I325" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J325" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K325" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_WindowWall.glb</x:v>
+      </x:c>
+      <x:c r="L325" s="1" t="str">
+        <x:v>03c83847a7d1d76edc2ad1cd0a48361e316e8735b9d8e6b54af2120954c2601f</x:v>
+      </x:c>
+      <x:c r="M325" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N325" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O325" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P325" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q325" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326" ht="38" customHeight="1">
+      <x:c r="A326" s="1" t="str">
+        <x:v>Prop_Bricks_DoorFrame</x:v>
+      </x:c>
+      <x:c r="B326" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C326" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D326" s="5" t="str">
+        <x:v>Clear doorway</x:v>
+      </x:c>
+      <x:c r="E326" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F326" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G326" s="5" t="str"/>
+      <x:c r="H326" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I326" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J326" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K326" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_DoorFrame.glb</x:v>
+      </x:c>
+      <x:c r="L326" s="1" t="str">
+        <x:v>764b6daa0a8baf3952eab7397d4bf86bea2170ae69effe75b863989a7d7a3468</x:v>
+      </x:c>
+      <x:c r="M326" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N326" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O326" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P326" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q326" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327" ht="38" customHeight="1">
+      <x:c r="A327" s="1" t="str">
+        <x:v>Prop_Bricks_Column</x:v>
+      </x:c>
+      <x:c r="B327" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C327" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D327" s="5" t="str">
+        <x:v>Corner support</x:v>
+      </x:c>
+      <x:c r="E327" s="7" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F327" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G327" s="5" t="str"/>
+      <x:c r="H327" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I327" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J327" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K327" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Column.glb</x:v>
+      </x:c>
+      <x:c r="L327" s="1" t="str">
+        <x:v>a5c5ab57f686fdee644bb0b6b0f9ed29546b35e89015069083b1fd3ac1bcea0a</x:v>
+      </x:c>
+      <x:c r="M327" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N327" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O327" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P327" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q327" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328" ht="38" customHeight="1">
+      <x:c r="A328" s="1" t="str">
+        <x:v>Prop_Bricks_Rail</x:v>
+      </x:c>
+      <x:c r="B328" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C328" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D328" s="5" t="str">
+        <x:v>Raised platform boundary</x:v>
+      </x:c>
+      <x:c r="E328" s="7" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F328" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G328" s="5" t="str"/>
+      <x:c r="H328" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I328" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J328" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K328" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Rail.glb</x:v>
+      </x:c>
+      <x:c r="L328" s="1" t="str">
+        <x:v>34a92d75f8d2c7b15ff388d7929e7d85c5c18023057a0e4d33a7014fcf93edd5</x:v>
+      </x:c>
+      <x:c r="M328" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N328" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O328" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P328" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q328" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329" ht="38" customHeight="1">
+      <x:c r="A329" s="1" t="str">
+        <x:v>Prop_Bricks_Ramp</x:v>
+      </x:c>
+      <x:c r="B329" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C329" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D329" s="5" t="str">
+        <x:v>Continuous access slope</x:v>
+      </x:c>
+      <x:c r="E329" s="7" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F329" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G329" s="5" t="str"/>
+      <x:c r="H329" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I329" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J329" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K329" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Ramp.glb</x:v>
+      </x:c>
+      <x:c r="L329" s="1" t="str">
+        <x:v>12e211ea909f59f9a8f21e305872991da8c0cbc479e94375c4132e716b465c5a</x:v>
+      </x:c>
+      <x:c r="M329" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N329" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O329" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P329" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q329" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330" ht="38" customHeight="1">
+      <x:c r="A330" s="1" t="str">
+        <x:v>Prop_Bricks_Stairs</x:v>
+      </x:c>
+      <x:c r="B330" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C330" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D330" s="5" t="str">
+        <x:v>Raised platform access</x:v>
+      </x:c>
+      <x:c r="E330" s="7" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F330" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G330" s="5" t="str"/>
+      <x:c r="H330" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I330" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J330" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K330" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Stairs.glb</x:v>
+      </x:c>
+      <x:c r="L330" s="1" t="str">
+        <x:v>a02432fddb1f68f770ff83fdad7daf1bdcc2322a14a3ee4e0c53e71268678ccd</x:v>
+      </x:c>
+      <x:c r="M330" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N330" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O330" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P330" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q330" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331" ht="38" customHeight="1">
+      <x:c r="A331" s="1" t="str">
+        <x:v>Prop_Bricks_Workbench</x:v>
+      </x:c>
+      <x:c r="B331" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C331" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D331" s="5" t="str">
+        <x:v>Repair station</x:v>
+      </x:c>
+      <x:c r="E331" s="7" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="F331" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G331" s="5" t="str"/>
+      <x:c r="H331" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I331" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J331" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K331" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Workbench.glb</x:v>
+      </x:c>
+      <x:c r="L331" s="1" t="str">
+        <x:v>1af99022ebe83b4b46abcd2f5a6fb0642d413ee4ac76c88ae7236472eebb2007</x:v>
+      </x:c>
+      <x:c r="M331" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N331" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O331" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P331" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q331" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332" ht="38" customHeight="1">
+      <x:c r="A332" s="1" t="str">
+        <x:v>Prop_Bricks_Kiln</x:v>
+      </x:c>
+      <x:c r="B332" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C332" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D332" s="5" t="str">
+        <x:v>Crafting station</x:v>
+      </x:c>
+      <x:c r="E332" s="7" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="F332" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G332" s="5" t="str"/>
+      <x:c r="H332" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I332" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J332" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K332" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Kiln.glb</x:v>
+      </x:c>
+      <x:c r="L332" s="1" t="str">
+        <x:v>928c25ee5b6463c0055f2912e97330a79fa191cd2c1d264b87f3373bc500785c</x:v>
+      </x:c>
+      <x:c r="M332" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N332" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O332" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P332" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q332" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333" ht="38" customHeight="1">
+      <x:c r="A333" s="1" t="str">
+        <x:v>Prop_Bricks_RecipeArchive</x:v>
+      </x:c>
+      <x:c r="B333" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C333" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D333" s="5" t="str">
+        <x:v>Blueprint archive</x:v>
+      </x:c>
+      <x:c r="E333" s="7" t="n">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="F333" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G333" s="5" t="str"/>
+      <x:c r="H333" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I333" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J333" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K333" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_RecipeArchive.glb</x:v>
+      </x:c>
+      <x:c r="L333" s="1" t="str">
+        <x:v>9366096d23023d33b6a65e7cfce46ba1db38ee791c50814a91d0e638bf4aef54</x:v>
+      </x:c>
+      <x:c r="M333" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N333" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O333" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P333" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q333" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334" ht="38" customHeight="1">
+      <x:c r="A334" s="1" t="str">
+        <x:v>Prop_Bricks_CraneBase</x:v>
+      </x:c>
+      <x:c r="B334" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C334" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D334" s="5" t="str">
+        <x:v>Crane station</x:v>
+      </x:c>
+      <x:c r="E334" s="7" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="F334" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G334" s="5" t="str"/>
+      <x:c r="H334" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I334" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J334" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K334" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_CraneBase.glb</x:v>
+      </x:c>
+      <x:c r="L334" s="1" t="str">
+        <x:v>6abced73aac2e1694db6446aacd9398a110783cdf86595eb08ff569b01dd6501</x:v>
+      </x:c>
+      <x:c r="M334" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N334" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O334" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P334" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q334" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335" ht="38" customHeight="1">
+      <x:c r="A335" s="1" t="str">
+        <x:v>Prop_Bricks_SalvageBin</x:v>
+      </x:c>
+      <x:c r="B335" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C335" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D335" s="5" t="str">
+        <x:v>Parts recovery station</x:v>
+      </x:c>
+      <x:c r="E335" s="7" t="n">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="F335" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G335" s="5" t="str"/>
+      <x:c r="H335" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I335" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J335" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K335" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_SalvageBin.glb</x:v>
+      </x:c>
+      <x:c r="L335" s="1" t="str">
+        <x:v>8c51974edc8381da75111884ff1d8a5fcfa5c1562a56d3143bacba642d28abef</x:v>
+      </x:c>
+      <x:c r="M335" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N335" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O335" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P335" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q335" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336" ht="38" customHeight="1">
+      <x:c r="A336" s="1" t="str">
+        <x:v>Prop_Bricks_Noticeboard</x:v>
+      </x:c>
+      <x:c r="B336" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C336" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D336" s="5" t="str">
+        <x:v>Quest presentation</x:v>
+      </x:c>
+      <x:c r="E336" s="7" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F336" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G336" s="5" t="str"/>
+      <x:c r="H336" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I336" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J336" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K336" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_Noticeboard.glb</x:v>
+      </x:c>
+      <x:c r="L336" s="1" t="str">
+        <x:v>fcd740d267dd4e658e546719b90b80143545222b0cdb18725c12b6e2f7b509f3</x:v>
+      </x:c>
+      <x:c r="M336" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N336" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O336" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P336" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q336" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337" ht="38" customHeight="1">
+      <x:c r="A337" s="1" t="str">
+        <x:v>Prop_Bricks_TradeCounter</x:v>
+      </x:c>
+      <x:c r="B337" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C337" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D337" s="5" t="str">
+        <x:v>Realm trade station</x:v>
+      </x:c>
+      <x:c r="E337" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F337" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G337" s="5" t="str"/>
+      <x:c r="H337" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I337" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J337" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K337" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_TradeCounter.glb</x:v>
+      </x:c>
+      <x:c r="L337" s="1" t="str">
+        <x:v>9c1da27731fb3abe55c4aa8c6b3019acd42546e173192de1460a4fa8ba88ee2e</x:v>
+      </x:c>
+      <x:c r="M337" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N337" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O337" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P337" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q337" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" ht="38" customHeight="1">
+      <x:c r="A338" s="1" t="str">
+        <x:v>Prop_Bricks_RunwayTile</x:v>
+      </x:c>
+      <x:c r="B338" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C338" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D338" s="5" t="str">
+        <x:v>Continuous airfield strip</x:v>
+      </x:c>
+      <x:c r="E338" s="7" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F338" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G338" s="5" t="str"/>
+      <x:c r="H338" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I338" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J338" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K338" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_RunwayTile.glb</x:v>
+      </x:c>
+      <x:c r="L338" s="1" t="str">
+        <x:v>96b22fa4ca23e55097cd5f3a691addb8fe94dd03d05c6b30e8b476f11302fca6</x:v>
+      </x:c>
+      <x:c r="M338" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N338" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O338" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P338" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q338" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" ht="38" customHeight="1">
+      <x:c r="A339" s="1" t="str">
+        <x:v>Prop_Bricks_HangarFrame</x:v>
+      </x:c>
+      <x:c r="B339" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C339" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D339" s="5" t="str">
+        <x:v>Clear aircraft shelter entry</x:v>
+      </x:c>
+      <x:c r="E339" s="7" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F339" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G339" s="5" t="str"/>
+      <x:c r="H339" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I339" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J339" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K339" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_HangarFrame.glb</x:v>
+      </x:c>
+      <x:c r="L339" s="1" t="str">
+        <x:v>18ba51d9b7f9e2c8c99927cf196b91ef9409b246a1e323988e05eb4c75e6c7e1</x:v>
+      </x:c>
+      <x:c r="M339" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N339" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O339" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P339" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q339" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340" ht="38" customHeight="1">
+      <x:c r="A340" s="1" t="str">
+        <x:v>Prop_Bricks_RepairBay</x:v>
+      </x:c>
+      <x:c r="B340" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C340" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D340" s="5" t="str">
+        <x:v>Vehicle service platform</x:v>
+      </x:c>
+      <x:c r="E340" s="7" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F340" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G340" s="5" t="str"/>
+      <x:c r="H340" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I340" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J340" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K340" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_RepairBay.glb</x:v>
+      </x:c>
+      <x:c r="L340" s="1" t="str">
+        <x:v>f4b9d10a3248ce8630d35c07f6011b5906816c8e9d27be379b902638b93663a8</x:v>
+      </x:c>
+      <x:c r="M340" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N340" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O340" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P340" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q340" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341" ht="38" customHeight="1">
+      <x:c r="A341" s="1" t="str">
+        <x:v>Prop_Bricks_ConcertPlatform</x:v>
+      </x:c>
+      <x:c r="B341" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C341" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D341" s="5" t="str">
+        <x:v>Touring jukebox station</x:v>
+      </x:c>
+      <x:c r="E341" s="7" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F341" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G341" s="5" t="str"/>
+      <x:c r="H341" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I341" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J341" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K341" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_ConcertPlatform.glb</x:v>
+      </x:c>
+      <x:c r="L341" s="1" t="str">
+        <x:v>31102687d8885126c13bc0f366a94b869977526e75f8e5f609c35da90c8212f1</x:v>
+      </x:c>
+      <x:c r="M341" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N341" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O341" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P341" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q341" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342" ht="38" customHeight="1">
+      <x:c r="A342" s="1" t="str">
+        <x:v>Prop_Bricks_RainbowFrame</x:v>
+      </x:c>
+      <x:c r="B342" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C342" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D342" s="5" t="str">
+        <x:v>Rainbow departure presentation</x:v>
+      </x:c>
+      <x:c r="E342" s="7" t="n">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="F342" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G342" s="5" t="str"/>
+      <x:c r="H342" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I342" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J342" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K342" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_RainbowFrame.glb</x:v>
+      </x:c>
+      <x:c r="L342" s="1" t="str">
+        <x:v>94cca53c4069b7b60f7ab84e12bb1624f9824e23c6fe167b287456251e9a7883</x:v>
+      </x:c>
+      <x:c r="M342" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N342" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O342" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P342" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q342" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343" ht="38" customHeight="1">
+      <x:c r="A343" s="1" t="str">
+        <x:v>Prop_Bricks_BoatDock</x:v>
+      </x:c>
+      <x:c r="B343" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C343" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D343" s="5" t="str">
+        <x:v>Ocean departure dock</x:v>
+      </x:c>
+      <x:c r="E343" s="7" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F343" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G343" s="5" t="str"/>
+      <x:c r="H343" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I343" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J343" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K343" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_BoatDock.glb</x:v>
+      </x:c>
+      <x:c r="L343" s="1" t="str">
+        <x:v>4137281a4839f22bb66497e77746ed5aee2d421a472bff3eae0defb39734ce3f</x:v>
+      </x:c>
+      <x:c r="M343" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N343" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O343" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P343" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q343" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344" ht="38" customHeight="1">
+      <x:c r="A344" s="1" t="str">
+        <x:v>Prop_Bricks_UnderwaterAirlock</x:v>
+      </x:c>
+      <x:c r="B344" s="1" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C344" s="1" t="str">
+        <x:v>Brick Realm</x:v>
+      </x:c>
+      <x:c r="D344" s="5" t="str">
+        <x:v>Ocean arrival presentation</x:v>
+      </x:c>
+      <x:c r="E344" s="7" t="n">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="F344" s="1" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G344" s="5" t="str"/>
+      <x:c r="H344" s="1" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I344" s="1" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J344" s="1" t="str">
+        <x:v>Binding pending</x:v>
+      </x:c>
+      <x:c r="K344" s="1" t="str">
+        <x:v>bricks-buildout/environment/Prop_Bricks_UnderwaterAirlock.glb</x:v>
+      </x:c>
+      <x:c r="L344" s="1" t="str">
+        <x:v>02adaf1fe703e98aeca152ac866c2df55a8c485a7cc14aa0510eb041bc9cb7a5</x:v>
+      </x:c>
+      <x:c r="M344" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N344" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O344" s="1" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P344" s="1" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q344" s="5" t="str">
+        <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="10">
+  <x:dataValidations count="12">
     <x:dataValidation type="list" sqref="I6:I72">
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
@@ -14757,6 +17683,12 @@
       <x:formula1>"Pending,Imported,Play proven"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J233:J288">
+      <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I289:I344">
+      <x:formula1>"Pending,Imported,Play proven"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="J289:J344">
       <x:formula1>"Binding pending,Core tested,Play proven"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -15627,12 +18559,22 @@
       <x:c r="K37" s="2"/>
       <x:c r="L37" s="2"/>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="2"/>
-      <x:c r="B38" s="2"/>
-      <x:c r="C38" s="2"/>
-      <x:c r="D38" s="2"/>
-      <x:c r="E38" s="2"/>
+    <x:row r="38" ht="52" customHeight="1">
+      <x:c r="A38" s="2" t="str">
+        <x:v>BRK01</x:v>
+      </x:c>
+      <x:c r="B38" s="4" t="str">
+        <x:v>Repair scattered assemblies and restore the airfield</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="str">
+        <x:v>32 cast/construct/mount/pet role models</x:v>
+      </x:c>
+      <x:c r="D38" s="4" t="str">
+        <x:v>Art validated; host objective gates pending</x:v>
+      </x:c>
+      <x:c r="E38" s="4" t="str">
+        <x:v>Missing Piece Collector guides repairs after Unmaker</x:v>
+      </x:c>
       <x:c r="F38" s="2"/>
       <x:c r="G38" s="2"/>
       <x:c r="H38" s="2"/>
@@ -15641,12 +18583,22 @@
       <x:c r="K38" s="2"/>
       <x:c r="L38" s="2"/>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="2"/>
-      <x:c r="B39" s="2"/>
-      <x:c r="C39" s="2"/>
-      <x:c r="D39" s="2"/>
-      <x:c r="E39" s="2"/>
+    <x:row r="39" ht="52" customHeight="1">
+      <x:c r="A39" s="2" t="str">
+        <x:v>BRK02</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>Meadow, road, runway and workshop modules</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>24 original modular props</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="str">
+        <x:v>Static validation; collision and interactions pending</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="str">
+        <x:v>Long routes connect builders, workshops and sea docks</x:v>
+      </x:c>
       <x:c r="F39" s="2"/>
       <x:c r="G39" s="2"/>
       <x:c r="H39" s="2"/>
@@ -15655,12 +18607,22 @@
       <x:c r="K39" s="2"/>
       <x:c r="L39" s="2"/>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="2"/>
-      <x:c r="B40" s="2"/>
-      <x:c r="C40" s="2"/>
-      <x:c r="D40" s="2"/>
-      <x:c r="E40" s="2"/>
+    <x:row r="40" ht="52" customHeight="1">
+      <x:c r="A40" s="2" t="str">
+        <x:v>BRK03</x:v>
+      </x:c>
+      <x:c r="B40" s="4" t="str">
+        <x:v>Plane, hover cart and companion travel</x:v>
+      </x:c>
+      <x:c r="C40" s="4" t="str">
+        <x:v>Three mount/vehicle models and four pets</x:v>
+      </x:c>
+      <x:c r="D40" s="4" t="str">
+        <x:v>Native possession, physics and rewards pending</x:v>
+      </x:c>
+      <x:c r="E40" s="4" t="str">
+        <x:v>Repair transport to reach new exploration routes</x:v>
+      </x:c>
       <x:c r="F40" s="2"/>
       <x:c r="G40" s="2"/>
       <x:c r="H40" s="2"/>

</xml_diff>

<commit_message>
Verify remote dock boarding and record measured runtime checks
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R4588cbaccfdb4826"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R50679d0f83dd4d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R884ef78873444bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R549d44a51f254c04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rae2193682cf8474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rfd78cdb171e241f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R7e709991c17b4dfe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -39,8 +41,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -77,6 +84,21 @@
         <x:fgColor rgb="FF243746"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF243746"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -90,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -147,6 +169,18 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -18631,12 +18665,22 @@
       <x:c r="K40" s="2"/>
       <x:c r="L40" s="2"/>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="2"/>
-      <x:c r="B41" s="2"/>
-      <x:c r="C41" s="2"/>
-      <x:c r="D41" s="2"/>
-      <x:c r="E41" s="2"/>
+    <x:row r="41" ht="58" customHeight="1">
+      <x:c r="A41" s="2" t="str">
+        <x:v>OCE01</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>Board/exit at configured docks</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>Native possession, hull and camera checks</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="str">
+        <x:v>Headless native verification; art/remote exit pending</x:v>
+      </x:c>
+      <x:c r="E41" s="4" t="str">
+        <x:v>Boats and submarines support journeys from docks</x:v>
+      </x:c>
       <x:c r="F41" s="2"/>
       <x:c r="G41" s="2"/>
       <x:c r="H41" s="2"/>
@@ -18645,12 +18689,22 @@
       <x:c r="K41" s="2"/>
       <x:c r="L41" s="2"/>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="2"/>
-      <x:c r="B42" s="2"/>
-      <x:c r="C42" s="2"/>
-      <x:c r="D42" s="2"/>
-      <x:c r="E42" s="2"/>
+    <x:row r="42" ht="58" customHeight="1">
+      <x:c r="A42" s="2" t="str">
+        <x:v>OCE02</x:v>
+      </x:c>
+      <x:c r="B42" s="4" t="str">
+        <x:v>Owned remote boarding request</x:v>
+      </x:c>
+      <x:c r="C42" s="4" t="str">
+        <x:v>Server derives Hero from component owner</x:v>
+      </x:c>
+      <x:c r="D42" s="4" t="str">
+        <x:v>Localhost boat/submarine function paths passed</x:v>
+      </x:c>
+      <x:c r="E42" s="4" t="str">
+        <x:v>Host session permissions still need integration</x:v>
+      </x:c>
       <x:c r="F42" s="2"/>
       <x:c r="G42" s="2"/>
       <x:c r="H42" s="2"/>
@@ -18659,12 +18713,22 @@
       <x:c r="K42" s="2"/>
       <x:c r="L42" s="2"/>
     </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="2"/>
-      <x:c r="B43" s="2"/>
-      <x:c r="C43" s="2"/>
-      <x:c r="D43" s="2"/>
-      <x:c r="E43" s="2"/>
+    <x:row r="43" ht="58" customHeight="1">
+      <x:c r="A43" s="2" t="str">
+        <x:v>OCE03</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>Sea realm travel and shore return</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>Approved boat/submarine and underwater dock rules</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>Route core exists; loader/persistence integration pending</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="str">
+        <x:v>Dragon Warrior shores return to land; underwater docks link realms</x:v>
+      </x:c>
       <x:c r="F43" s="2"/>
       <x:c r="G43" s="2"/>
       <x:c r="H43" s="2"/>
@@ -18984,4 +19048,446 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="39" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="45" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="26" t="str">
+        <x:v>Native ocean verification runs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Scoped evidence, not every Unreal action. Seconds cover the stated scope; no mixed-scope total.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Verified runs</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:f>COUNTIF(D8:D22,"Verified")</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Pending checks</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:f>COUNTIF(D8:D22,"Pending")</x:f>
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="28" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="str">
+        <x:v>Behavior / run</x:v>
+      </x:c>
+      <x:c r="C7" s="28" t="str">
+        <x:v>Realm</x:v>
+      </x:c>
+      <x:c r="D7" s="28" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="E7" s="28" t="str">
+        <x:v>Seconds</x:v>
+      </x:c>
+      <x:c r="F7" s="28" t="str">
+        <x:v>Measured scope</x:v>
+      </x:c>
+      <x:c r="G7" s="28" t="str">
+        <x:v>Evidence in docs/production</x:v>
+      </x:c>
+      <x:c r="H7" s="28" t="str">
+        <x:v>Limit / remaining work</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="1" t="str">
+        <x:v>BUILD</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>Complete plugin reflection/compile/link</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E8" s="29" t="n">
+        <x:v>187.98</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="str">
+        <x:v>44 build actions; full process</x:v>
+      </x:c>
+      <x:c r="G8" s="5" t="str">
+        <x:v>ocean-owned-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H8" s="5" t="str">
+        <x:v>Compilation is not shipped gameplay</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="1" t="str">
+        <x:v>HERO</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="str">
+        <x:v>Daedalus.Ocean.HeroDockInteraction</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D9" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E9" s="29" t="n">
+        <x:v>0.011751800775527954</x:v>
+      </x:c>
+      <x:c r="F9" s="5" t="str">
+        <x:v>Automation test body; excludes engine startup</x:v>
+      </x:c>
+      <x:c r="G9" s="5" t="str">
+        <x:v>ocean-owned-runtime-proof.json</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="str">
+        <x:v>Headless function path, not physical device input</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="1" t="str">
+        <x:v>NATIVE</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>Daedalus.Ocean.HostEligibility</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E10" s="29" t="n">
+        <x:v>0.016099803149700165</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="str">
+        <x:v>Automation test body; excludes engine startup</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="str">
+        <x:v>ocean-owned-runtime-proof.json</x:v>
+      </x:c>
+      <x:c r="H10" s="5" t="str">
+        <x:v>Headless function path, not physical device input</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="1" t="str">
+        <x:v>BOARD-boat</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>Remote Hero interaction boards vessel — boat</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D11" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E11" s="29" t="n">
+        <x:v>17.625</x:v>
+      </x:c>
+      <x:c r="F11" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G11" s="5" t="str">
+        <x:v>ocean-owned-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H11" s="5" t="str">
+        <x:v>No physical E/X dispatch or realm transfer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="1" t="str">
+        <x:v>BOARD-submarine</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="str">
+        <x:v>Remote Hero interaction boards vessel — submarine</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D12" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E12" s="29" t="n">
+        <x:v>17.61</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G12" s="5" t="str">
+        <x:v>ocean-owned-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H12" s="5" t="str">
+        <x:v>No physical E/X dispatch or realm transfer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="1" t="str">
+        <x:v>KEY-boat</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="str">
+        <x:v>Keyboard event propulsion — boat</x:v>
+      </x:c>
+      <x:c r="C13" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D13" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E13" s="29" t="n">
+        <x:v>24.172</x:v>
+      </x:c>
+      <x:c r="F13" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G13" s="5" t="str">
+        <x:v>ocean-keyboard-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H13" s="5" t="str">
+        <x:v>Engine events; no physical hardware or rendered acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
+      <x:c r="A14" s="1" t="str">
+        <x:v>KEY-submarine</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="str">
+        <x:v>Keyboard event propulsion/dive — submarine</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D14" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E14" s="29" t="n">
+        <x:v>24.187</x:v>
+      </x:c>
+      <x:c r="F14" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G14" s="5" t="str">
+        <x:v>ocean-keyboard-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H14" s="5" t="str">
+        <x:v>Engine events; no physical hardware or rendered acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="1" t="str">
+        <x:v>PAD-boat</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="str">
+        <x:v>Analog event propulsion — boat</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E15" s="29" t="n">
+        <x:v>23.656</x:v>
+      </x:c>
+      <x:c r="F15" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="str">
+        <x:v>ocean-gamepad-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H15" s="5" t="str">
+        <x:v>Engine events; no physical hardware or rendered acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="1" t="str">
+        <x:v>PAD-submarine</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="str">
+        <x:v>Analog event propulsion/dive — submarine</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E16" s="29" t="n">
+        <x:v>24.406</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="str">
+        <x:v>Server/client startup, handshake and scenario</x:v>
+      </x:c>
+      <x:c r="G16" s="5" t="str">
+        <x:v>ocean-gamepad-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H16" s="5" t="str">
+        <x:v>Engine events; no physical hardware or rendered acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="1" t="str">
+        <x:v>HW</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="str">
+        <x:v>Physical Interact/controller hardware</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D17" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E17" s="29"/>
+      <x:c r="F17" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G17" s="5"/>
+      <x:c r="H17" s="5" t="str">
+        <x:v>Requires actual device/viewport run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="58" customHeight="1">
+      <x:c r="A18" s="1" t="str">
+        <x:v>EXIT</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>Remote exit input and restoration</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D18" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E18" s="29"/>
+      <x:c r="F18" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G18" s="5"/>
+      <x:c r="H18" s="5" t="str">
+        <x:v>Local exit tested; remote input not wired</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="58" customHeight="1">
+      <x:c r="A19" s="1" t="str">
+        <x:v>REALM</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="str">
+        <x:v>Portal ↔ Ocean / underwater realm transfer</x:v>
+      </x:c>
+      <x:c r="C19" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D19" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E19" s="29"/>
+      <x:c r="F19" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G19" s="5"/>
+      <x:c r="H19" s="5" t="str">
+        <x:v>Loader, anchors and persistent session integration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="1" t="str">
+        <x:v>ART</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="str">
+        <x:v>Live vessel/dock art and camera composition</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D20" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E20" s="29"/>
+      <x:c r="F20" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G20" s="5"/>
+      <x:c r="H20" s="5" t="str">
+        <x:v>Export/model assignment is not live acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="1" t="str">
+        <x:v>AUTH</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="str">
+        <x:v>Production login and travel permissions</x:v>
+      </x:c>
+      <x:c r="C21" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D21" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E21" s="29"/>
+      <x:c r="F21" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G21" s="5"/>
+      <x:c r="H21" s="5" t="str">
+        <x:v>Test fixtures do not prove real account policy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="58" customHeight="1">
+      <x:c r="A22" s="1" t="str">
+        <x:v>HOST</x:v>
+      </x:c>
+      <x:c r="B22" s="5" t="str">
+        <x:v>Public hosting, restart and recovery</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D22" s="31" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="E22" s="29"/>
+      <x:c r="F22" s="5" t="str">
+        <x:v>Not measured</x:v>
+      </x:c>
+      <x:c r="G22" s="5"/>
+      <x:c r="H22" s="5" t="str">
+        <x:v>Requires deployment and end-to-end verification</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="D8:D22">
+      <x:formula1>"Verified,Pending"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify remote vessel round trips through E input and record evidence
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R549d44a51f254c04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rae2193682cf8474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rfd78cdb171e241f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R7e709991c17b4dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R72402fdea0b5440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R1bab0b18469b4661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R80a8d9c25b824987"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R12271c568cbf4b7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,6 +99,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -112,7 +117,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -179,6 +184,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -18676,7 +18687,7 @@
         <x:v>Native possession, hull and camera checks</x:v>
       </x:c>
       <x:c r="D41" s="4" t="str">
-        <x:v>Headless native verification; art/remote exit pending</x:v>
+        <x:v>Native and localhost E-key exit verified; art/physical controls pending</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
         <x:v>Boats and submarines support journeys from docks</x:v>
@@ -18700,7 +18711,7 @@
         <x:v>Server derives Hero from component owner</x:v>
       </x:c>
       <x:c r="D42" s="4" t="str">
-        <x:v>Localhost boat/submarine function paths passed</x:v>
+        <x:v>Localhost boat/submarine boarding and exit passed</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
         <x:v>Host session permissions still need integration</x:v>
@@ -19079,15 +19090,15 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D22,"Verified")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF(D8:D23,"Verified")</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D22,"Pending")</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIF(D8:D23,"Pending")</x:f>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -19372,26 +19383,30 @@
         <x:v>Requires actual device/viewport run</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="58" customHeight="1">
+    <x:row r="18" ht="70" customHeight="1">
       <x:c r="A18" s="1" t="str">
-        <x:v>EXIT</x:v>
+        <x:v>EXIT-boat</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>Remote exit input and restoration</x:v>
+        <x:v>Remote boat boarding and E-key exit</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
         <x:v>Ocean</x:v>
       </x:c>
-      <x:c r="D18" s="31" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E18" s="29"/>
+      <x:c r="D18" s="33" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E18" s="29" t="n">
+        <x:v>18.359</x:v>
+      </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>Not measured</x:v>
-      </x:c>
-      <x:c r="G18" s="5"/>
+        <x:v>Startup, handshake and round trip</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="str">
+        <x:v>ocean-exit-network-proof.json</x:v>
+      </x:c>
       <x:c r="H18" s="5" t="str">
-        <x:v>Local exit tested; remote input not wired</x:v>
+        <x:v>Engine key event; physical device, art and realm loading pending</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
@@ -19482,9 +19497,38 @@
         <x:v>Requires deployment and end-to-end verification</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="70" customHeight="1">
+      <x:c r="A23" s="1" t="str">
+        <x:v>EXIT-submarine</x:v>
+      </x:c>
+      <x:c r="B23" s="5" t="str">
+        <x:v>Remote submarine boarding and E-key exit</x:v>
+      </x:c>
+      <x:c r="C23" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D23" s="33" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E23" s="29" t="n">
+        <x:v>18.375</x:v>
+      </x:c>
+      <x:c r="F23" s="5" t="str">
+        <x:v>Startup, handshake and round trip</x:v>
+      </x:c>
+      <x:c r="G23" s="5" t="str">
+        <x:v>ocean-exit-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H23" s="5" t="str">
+        <x:v>Engine key event; physical device, art and realm loading pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D8:D22">
+      <x:formula1>"Verified,Pending"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D23">
       <x:formula1>"Verified,Pending"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
Track Ocean terrain delivery and add portable export CI
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R72402fdea0b5440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R1bab0b18469b4661"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R80a8d9c25b824987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R12271c568cbf4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Raed22c646ad5460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R12a348e388f6442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R5a7410576e0a41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R4fbdffd0bec84686"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +104,11 @@
         <x:fgColor rgb="FFE8F5E9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -117,7 +122,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="34">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -190,6 +195,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -519,15 +527,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -535,7 +543,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -554,15 +562,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A8)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A8)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="2" t="n">
@@ -570,7 +578,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A8)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
@@ -589,15 +597,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -605,7 +613,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A9)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9)</x:f>
         <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
@@ -624,15 +632,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A10)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A10)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="2" t="n">
@@ -640,7 +648,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A10)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
@@ -659,15 +667,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$344,Assets!$C$6:$C$344,A11)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A11)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11,Assets!$B$6:$B$344,"Character",Assets!$H$6:$H$344,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11,Assets!$B$6:$B$344,"Character",Assets!$I$6:$I$344,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="2" t="n">
@@ -675,7 +683,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$344,A11)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
@@ -684,14 +692,32 @@
       <x:c r="L11" s="2"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="2"/>
-      <x:c r="C12" s="2"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
-      <x:c r="G12" s="2"/>
-      <x:c r="H12" s="2"/>
+      <x:c r="A12" s="2" t="str">
+        <x:v>Ocean Realm</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>Sol / Codex</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str"/>
+      <x:c r="D12" s="2" t="n">
+        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A12,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="n">
+        <x:f>COUNTIFS(Assets!$C$6:$C$345,A12,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="2" t="str">
+        <x:f>IF(C12="","",C12-D12)</x:f>
+      </x:c>
+      <x:c r="H12" s="2" t="n">
+        <x:f>COUNTIF(Assets!C6:C345,A12)</x:f>
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I12" s="2"/>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -716,8 +742,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E344)</x:f>
-        <x:v>311464</x:v>
+        <x:f>SUM(Assets!E6:E345)</x:f>
+        <x:v>362614</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -735,7 +761,7 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B344,"Prop")+COUNTIFS(Assets!B6:B344,"Item")</x:f>
+        <x:f>COUNTIFS(Assets!B6:B345,"Prop")+COUNTIFS(Assets!B6:B345,"Item")</x:f>
         <x:v>131</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
@@ -765,7 +791,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>Codex kits: 339 unique asset references, including one unchanged AMF reuse. Export validation is not Play proof.</x:v>
+        <x:v>340 unique asset references, including one unchanged AMF reuse and one generated Ocean sector. Export is not Play proof.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -780,7 +806,9 @@
       <x:c r="L17" s="2"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="2"/>
+      <x:c r="A18" s="2" t="str">
+        <x:v>Ocean character-role target is not set yet; the generated terrain adds no character roles.</x:v>
+      </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
       <x:c r="D18" s="2"/>
@@ -17696,6 +17724,59 @@
       </x:c>
       <x:c r="Q344" s="5" t="str">
         <x:v>Codex original</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345" ht="96" customHeight="1">
+      <x:c r="A345" s="5" t="str">
+        <x:v>Terrain_Ocean_Seed42013_Sector</x:v>
+      </x:c>
+      <x:c r="B345" s="5" t="str">
+        <x:v>Terrain</x:v>
+      </x:c>
+      <x:c r="C345" s="5" t="str">
+        <x:v>Ocean Realm</x:v>
+      </x:c>
+      <x:c r="D345" s="5" t="str">
+        <x:v>Seeded sea sector and floating dock</x:v>
+      </x:c>
+      <x:c r="E345" s="5" t="n">
+        <x:v>51150</x:v>
+      </x:c>
+      <x:c r="F345" s="5" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G345" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H345" s="34" t="str">
+        <x:v>Generated</x:v>
+      </x:c>
+      <x:c r="I345" s="34" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J345" s="5" t="str">
+        <x:v>Server registration and realm loading pending</x:v>
+      </x:c>
+      <x:c r="K345" s="5" t="str">
+        <x:v>C:/Users/730ri/Documents/Codex/2026-10-13/ocean-terrain-2/ocean.glb</x:v>
+      </x:c>
+      <x:c r="L345" s="5" t="str">
+        <x:v>727b3b436bcd8929eb67c6d6687d54e00e9cf21937b2c5d14a31b4faa3cf7ee0</x:v>
+      </x:c>
+      <x:c r="M345" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N345" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O345" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P345" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q345" s="5" t="str">
+        <x:v>Codex procedural terrain; generator v1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18748,12 +18829,22 @@
       <x:c r="K43" s="2"/>
       <x:c r="L43" s="2"/>
     </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="2"/>
-      <x:c r="B44" s="2"/>
-      <x:c r="C44" s="2"/>
-      <x:c r="D44" s="2"/>
-      <x:c r="E44" s="2"/>
+    <x:row r="44" ht="76" customHeight="1">
+      <x:c r="A44" s="4" t="str">
+        <x:v>OCE04</x:v>
+      </x:c>
+      <x:c r="B44" s="4" t="str">
+        <x:v>Seeded open sea and floating dock</x:v>
+      </x:c>
+      <x:c r="C44" s="4" t="str">
+        <x:v>Chunk generation; existing save/mesh formats</x:v>
+      </x:c>
+      <x:c r="D44" s="4" t="str">
+        <x:v>706 core tests passed; server registration and Unreal acceptance pending</x:v>
+      </x:c>
+      <x:c r="E44" s="4" t="str">
+        <x:v>Generate nearby sea chunks; preserve player edits before regeneration</x:v>
+      </x:c>
       <x:c r="F44" s="2"/>
       <x:c r="G44" s="2"/>
       <x:c r="H44" s="2"/>

</xml_diff>

<commit_message>
Record Ocean persistence evidence and update mechanics tracker
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Raed22c646ad5460e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R12a348e388f6442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R5a7410576e0a41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R4fbdffd0bec84686"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R8786bb3c0f0b4961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R94ef51e070a44646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R25add719869e4445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rf2cbe6acb97c4696"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18853,12 +18853,22 @@
       <x:c r="K44" s="2"/>
       <x:c r="L44" s="2"/>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="2"/>
-      <x:c r="B45" s="2"/>
-      <x:c r="C45" s="2"/>
-      <x:c r="D45" s="2"/>
-      <x:c r="E45" s="2"/>
+    <x:row r="45" ht="88" customHeight="1">
+      <x:c r="A45" s="4" t="str">
+        <x:v>OCE05</x:v>
+      </x:c>
+      <x:c r="B45" s="4" t="str">
+        <x:v>Visited sea chunks retain edits, including empty chunks</x:v>
+      </x:c>
+      <x:c r="C45" s="4" t="str">
+        <x:v>Exclusive writer; seed/version checks; staged atomic saves</x:v>
+      </x:c>
+      <x:c r="D45" s="4" t="str">
+        <x:v>712 core tests and separate-JVM restart/OS lock probe passed</x:v>
+      </x:c>
+      <x:c r="E45" s="4" t="str">
+        <x:v>Local storage verified; host integration, public recovery and realm loading pending</x:v>
+      </x:c>
       <x:c r="F45" s="2"/>
       <x:c r="G45" s="2"/>
       <x:c r="H45" s="2"/>

</xml_diff>

<commit_message>
Record bounded Ocean window evidence and mechanics
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R8786bb3c0f0b4961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R94ef51e070a44646"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R25add719869e4445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rf2cbe6acb97c4696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R704f21bd1abf4658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R4c254b2171c34229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R642269c41f334446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R36ac1a57be5b4c75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18877,12 +18877,22 @@
       <x:c r="K45" s="2"/>
       <x:c r="L45" s="2"/>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="2"/>
-      <x:c r="B46" s="2"/>
-      <x:c r="C46" s="2"/>
-      <x:c r="D46" s="2"/>
-      <x:c r="E46" s="2"/>
+    <x:row r="46" ht="88" customHeight="1">
+      <x:c r="A46" s="4" t="str">
+        <x:v>OCE06</x:v>
+      </x:c>
+      <x:c r="B46" s="4" t="str">
+        <x:v>Nearby sea chunks use a bounded resident window</x:v>
+      </x:c>
+      <x:c r="C46" s="4" t="str">
+        <x:v>Nearest-first warmup; write-through edits; safe eviction</x:v>
+      </x:c>
+      <x:c r="D46" s="4" t="str">
+        <x:v>718 core tests and separate-process cache restart probe passed</x:v>
+      </x:c>
+      <x:c r="E46" s="4" t="str">
+        <x:v>Local cache verified; authenticated host routes and Unreal streaming pending</x:v>
+      </x:c>
       <x:c r="F46" s="2"/>
       <x:c r="G46" s="2"/>
       <x:c r="H46" s="2"/>

</xml_diff>

<commit_message>
Record Ocean HTTP auth and restart evidence in production tracker
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R704f21bd1abf4658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R4c254b2171c34229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R642269c41f334446"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R36ac1a57be5b4c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R14576a31197b4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rcf7e9350f8bd4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdd046ccf8d244dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rfb2344d520eb4bc7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18901,12 +18901,22 @@
       <x:c r="K46" s="2"/>
       <x:c r="L46" s="2"/>
     </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="2"/>
-      <x:c r="B47" s="2"/>
-      <x:c r="C47" s="2"/>
-      <x:c r="D47" s="2"/>
-      <x:c r="E47" s="2"/>
+    <x:row r="47" ht="88" customHeight="1">
+      <x:c r="A47" s="4" t="str">
+        <x:v>OCE07</x:v>
+      </x:c>
+      <x:c r="B47" s="4" t="str">
+        <x:v>Authenticated sea-sector chunk reads</x:v>
+      </x:c>
+      <x:c r="C47" s="4" t="str">
+        <x:v>Existing chunk DTO; bounded sector; per-key quota</x:v>
+      </x:c>
+      <x:c r="D47" s="4" t="str">
+        <x:v>18 Ocean core + 14 server/auth tests; real prod HTTP/restart passed</x:v>
+      </x:c>
+      <x:c r="E47" s="4" t="str">
+        <x:v>Opt-in API verified; native client, realm registration and public hosting pending</x:v>
+      </x:c>
       <x:c r="F47" s="2"/>
       <x:c r="G47" s="2"/>
       <x:c r="H47" s="2"/>

</xml_diff>

<commit_message>
Verify packaged Java to native Ocean transport and record timings
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R14576a31197b4917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rcf7e9350f8bd4873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdd046ccf8d244dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rfb2344d520eb4bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Rc71e514588184602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R97fbd2f64f9b4d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R22d2399d561848c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rb6498d421f61448d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +109,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -122,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -198,6 +203,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -18925,12 +18933,22 @@
       <x:c r="K47" s="2"/>
       <x:c r="L47" s="2"/>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="2"/>
-      <x:c r="B48" s="2"/>
-      <x:c r="C48" s="2"/>
-      <x:c r="D48" s="2"/>
-      <x:c r="E48" s="2"/>
+    <x:row r="48" ht="88" customHeight="1">
+      <x:c r="A48" s="4" t="str">
+        <x:v>OCE08</x:v>
+      </x:c>
+      <x:c r="B48" s="4" t="str">
+        <x:v>Native client receives authenticated sea chunks</x:v>
+      </x:c>
+      <x:c r="C48" s="4" t="str">
+        <x:v>One in flight; bounded receive; strict DTO; stale-session guard</x:v>
+      </x:c>
+      <x:c r="D48" s="4" t="str">
+        <x:v>131-file plugin and 3 native tests pass; real Java/native HTTP passed</x:v>
+      </x:c>
+      <x:c r="E48" s="4" t="str">
+        <x:v>Local transport verified; scene meshes, TLS/redirect audit and travel pending</x:v>
+      </x:c>
       <x:c r="F48" s="2"/>
       <x:c r="G48" s="2"/>
       <x:c r="H48" s="2"/>
@@ -19211,14 +19229,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D23,"Verified")</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTIF(D8:D27,"Verified")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D23,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D27,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -19644,14 +19662,121 @@
         <x:v>Engine key event; physical device, art and realm loading pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="88" customHeight="1">
+      <x:c r="A24" s="5" t="str">
+        <x:v>BUILD-CLIENT</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="str">
+        <x:v>Complete 131-file plugin build</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D24" s="35" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E24" s="29" t="n">
+        <x:v>193.26</x:v>
+      </x:c>
+      <x:c r="F24" s="5" t="str">
+        <x:v>46 build/link actions; full process</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="str">
+        <x:v>ocean-client-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H24" s="5" t="str">
+        <x:v>Fresh base plus separately recorded lifecycle rebuild</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="88" customHeight="1">
+      <x:c r="A25" s="5" t="str">
+        <x:v>LIFECYCLE</x:v>
+      </x:c>
+      <x:c r="B25" s="5" t="str">
+        <x:v>Final EndPlay session-cancellation rebuild</x:v>
+      </x:c>
+      <x:c r="C25" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E25" s="29" t="n">
+        <x:v>12.4</x:v>
+      </x:c>
+      <x:c r="F25" s="5" t="str">
+        <x:v>5 incremental compile/link actions</x:v>
+      </x:c>
+      <x:c r="G25" s="5" t="str">
+        <x:v>ocean-client-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H25" s="5" t="str">
+        <x:v>All final production input hashes verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="88" customHeight="1">
+      <x:c r="A26" s="5" t="str">
+        <x:v>DECODE</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="str">
+        <x:v>Daedalus.Ocean.HostChunkDecoder</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D26" s="35" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E26" s="29" t="n">
+        <x:v>0.009295500814914703</x:v>
+      </x:c>
+      <x:c r="F26" s="5" t="str">
+        <x:v>Native test body; excludes engine startup</x:v>
+      </x:c>
+      <x:c r="G26" s="5" t="str">
+        <x:v>ocean-client-runtime-proof.json</x:v>
+      </x:c>
+      <x:c r="H26" s="5" t="str">
+        <x:v>Headless DTO/session validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="88" customHeight="1">
+      <x:c r="A27" s="5" t="str">
+        <x:v>HTTP-CLIENT</x:v>
+      </x:c>
+      <x:c r="B27" s="5" t="str">
+        <x:v>Packaged Java to native Ocean client</x:v>
+      </x:c>
+      <x:c r="C27" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E27" s="29" t="n">
+        <x:v>21.188</x:v>
+      </x:c>
+      <x:c r="F27" s="5" t="str">
+        <x:v>Java server startup plus native engine startup and HTTP scenario</x:v>
+      </x:c>
+      <x:c r="G27" s="5" t="str">
+        <x:v>ocean-client-http-proof.json</x:v>
+      </x:c>
+      <x:c r="H27" s="5" t="str">
+        <x:v>TLS/redirect, rendered gameplay and realm transfer pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D8:D22">
       <x:formula1>"Verified,Pending"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D23">
       <x:formula1>"Verified,Pending"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="D24:D27">
+      <x:formula1>"Verified,Pending"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Verify persisted Java chunks create and clear native Ocean geometry
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Rc71e514588184602"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R97fbd2f64f9b4d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R22d2399d561848c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rb6498d421f61448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R3a49aa8c3e674d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R659a8efa52dc48d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Re1775bc39ae342c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R5084e03c7bd148f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -47,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -114,6 +114,11 @@
         <x:fgColor rgb="FFE8F5E9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5E9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -127,7 +132,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -206,6 +211,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -18957,12 +18965,22 @@
       <x:c r="K48" s="2"/>
       <x:c r="L48" s="2"/>
     </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="2"/>
-      <x:c r="B49" s="2"/>
-      <x:c r="C49" s="2"/>
-      <x:c r="D49" s="2"/>
-      <x:c r="E49" s="2"/>
+    <x:row r="49" ht="88" customHeight="1">
+      <x:c r="A49" s="4" t="str">
+        <x:v>OCE09</x:v>
+      </x:c>
+      <x:c r="B49" s="4" t="str">
+        <x:v>Server sea chunks become native scene geometry</x:v>
+      </x:c>
+      <x:c r="C49" s="4" t="str">
+        <x:v>Canonical palette; neighbour remesh; local offsets; revisions preserved</x:v>
+      </x:c>
+      <x:c r="D49" s="4" t="str">
+        <x:v>135-file plugin / 4 native / 719 core tests pass; real geometry HTTP proof</x:v>
+      </x:c>
+      <x:c r="E49" s="4" t="str">
+        <x:v>Geometry verified; material appearance, rendered Play and realm travel pending</x:v>
+      </x:c>
       <x:c r="F49" s="2"/>
       <x:c r="G49" s="2"/>
       <x:c r="H49" s="2"/>
@@ -19229,14 +19247,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D27,"Verified")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIF(D8:D30,"Verified")</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D27,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D30,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -19766,8 +19784,86 @@
         <x:v>TLS/redirect, rendered gameplay and realm transfer pending</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="88" customHeight="1">
+      <x:c r="A28" s="5" t="str">
+        <x:v>BUILD-VIEW</x:v>
+      </x:c>
+      <x:c r="B28" s="5" t="str">
+        <x:v>Complete 135-file plugin build</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D28" s="36" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E28" s="29" t="n">
+        <x:v>202.42</x:v>
+      </x:c>
+      <x:c r="F28" s="5" t="str">
+        <x:v>48 build/link actions; full process</x:v>
+      </x:c>
+      <x:c r="G28" s="5" t="str">
+        <x:v>ocean-view-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H28" s="5" t="str">
+        <x:v>Full source hashes and production DLL recorded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="88" customHeight="1">
+      <x:c r="A29" s="5" t="str">
+        <x:v>GEOMETRY</x:v>
+      </x:c>
+      <x:c r="B29" s="5" t="str">
+        <x:v>Daedalus.Ocean.SectorGeometry</x:v>
+      </x:c>
+      <x:c r="C29" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D29" s="36" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E29" s="29" t="n">
+        <x:v>0.011793497949838638</x:v>
+      </x:c>
+      <x:c r="F29" s="5" t="str">
+        <x:v>Native test body; excludes engine startup</x:v>
+      </x:c>
+      <x:c r="G29" s="5" t="str">
+        <x:v>ocean-view-runtime-proof.json</x:v>
+      </x:c>
+      <x:c r="H29" s="5" t="str">
+        <x:v>Seams/capacity/revisions/collision flags; no rendered acceptance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="88" customHeight="1">
+      <x:c r="A30" s="5" t="str">
+        <x:v>HTTP-VIEW</x:v>
+      </x:c>
+      <x:c r="B30" s="5" t="str">
+        <x:v>Java saved terrain to native procedural mesh</x:v>
+      </x:c>
+      <x:c r="C30" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D30" s="36" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E30" s="29" t="n">
+        <x:v>20.766</x:v>
+      </x:c>
+      <x:c r="F30" s="5" t="str">
+        <x:v>Java server startup plus native engine startup and HTTP scenario</x:v>
+      </x:c>
+      <x:c r="G30" s="5" t="str">
+        <x:v>ocean-view-http-proof.json</x:v>
+      </x:c>
+      <x:c r="H30" s="5" t="str">
+        <x:v>Clear revision removes old mesh; appearance/travel pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="D8:D22">
       <x:formula1>"Verified,Pending"</x:formula1>
     </x:dataValidation>
@@ -19777,6 +19873,9 @@
     <x:dataValidation type="list" sqref="D24:D27">
       <x:formula1>"Verified,Pending"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="D28:D30">
+      <x:formula1>"Verified,Pending"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add original Ocean harbor assets and rendered native inspection delivery
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R3a49aa8c3e674d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R659a8efa52dc48d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Re1775bc39ae342c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R5084e03c7bd148f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R0a1380cdfba0446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R8f3663ecf7064541"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rbf9a92559ed64729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R9b3a8cafae154b11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -543,15 +543,15 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A7)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A7)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A7,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A7,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
@@ -559,7 +559,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A7)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A7)</x:f>
         <x:v>67</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
@@ -578,15 +578,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D8" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A8)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A8)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A8,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A8,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="2" t="n">
@@ -594,7 +594,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A8)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A8)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
@@ -613,15 +613,15 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="D9" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A9)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A9)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="E9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A9,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="F9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A9,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="2" t="n">
@@ -629,7 +629,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A9)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A9)</x:f>
         <x:v>104</x:v>
       </x:c>
       <x:c r="I9" s="2"/>
@@ -648,15 +648,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D10" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A10)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A10)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A10,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A10,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="2" t="n">
@@ -664,7 +664,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A10)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A10)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
@@ -683,15 +683,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D11" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A11)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A11)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A11,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="F11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A11,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="2" t="n">
@@ -699,7 +699,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A11)</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A11)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="I11" s="2"/>
@@ -716,23 +716,23 @@
       </x:c>
       <x:c r="C12" s="2" t="str"/>
       <x:c r="D12" s="2" t="n">
-        <x:f>SUMIFS(Assets!$M$6:$M$345,Assets!$C$6:$C$345,A12)</x:f>
+        <x:f>SUMIFS(Assets!$M$6:$M$348,Assets!$C$6:$C$348,A12)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A12,Assets!$B$6:$B$345,"Character",Assets!$H$6:$H$345,"Validated")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A12,Assets!$B$6:$B$348,"Character",Assets!$H$6:$H$348,"Validated")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="2" t="n">
-        <x:f>COUNTIFS(Assets!$C$6:$C$345,A12,Assets!$B$6:$B$345,"Character",Assets!$I$6:$I$345,"Play proven")</x:f>
+        <x:f>COUNTIFS(Assets!$C$6:$C$348,A12,Assets!$B$6:$B$348,"Character",Assets!$I$6:$I$348,"Play proven")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="2" t="str">
         <x:f>IF(C12="","",C12-D12)</x:f>
       </x:c>
       <x:c r="H12" s="2" t="n">
-        <x:f>COUNTIF(Assets!C6:C345,A12)</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF(Assets!C6:C348,A12)</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I12" s="2"/>
       <x:c r="J12" s="2"/>
@@ -758,8 +758,8 @@
         <x:v>Delivered triangles</x:v>
       </x:c>
       <x:c r="B14" s="6" t="n">
-        <x:f>SUM(Assets!E6:E345)</x:f>
-        <x:v>362614</x:v>
+        <x:f>SUM(Assets!E6:E348)</x:f>
+        <x:v>379408</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2"/>
@@ -777,8 +777,8 @@
         <x:v>Static meshes delivered</x:v>
       </x:c>
       <x:c r="B15" s="6" t="n">
-        <x:f>COUNTIFS(Assets!B6:B345,"Prop")+COUNTIFS(Assets!B6:B345,"Item")</x:f>
-        <x:v>131</x:v>
+        <x:f>COUNTIFS(Assets!B6:B348,"Prop")+COUNTIFS(Assets!B6:B348,"Item")</x:f>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
       <x:c r="D15" s="2"/>
@@ -807,7 +807,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="str">
-        <x:v>340 unique asset references, including one unchanged AMF reuse and one generated Ocean sector. Export is not Play proof.</x:v>
+        <x:v>343 unique asset references. Three Ocean props add no character roles. Export and inspection are not Play proof.</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -823,7 +823,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>Ocean character-role target is not set yet; the generated terrain adds no character roles.</x:v>
+        <x:v>Ocean character-role target is not set yet; terrain and vessel props add no character roles.</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
@@ -17793,6 +17793,165 @@
       </x:c>
       <x:c r="Q345" s="5" t="str">
         <x:v>Codex procedural terrain; generator v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346">
+      <x:c r="A346" s="5" t="str">
+        <x:v>Prop_Ocean_TideSkiff</x:v>
+      </x:c>
+      <x:c r="B346" s="5" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C346" s="5" t="str">
+        <x:v>Ocean Realm</x:v>
+      </x:c>
+      <x:c r="D346" s="5" t="str">
+        <x:v>Dock boat; helm/boarding presentation</x:v>
+      </x:c>
+      <x:c r="E346" s="5" t="n">
+        <x:v>1766</x:v>
+      </x:c>
+      <x:c r="F346" s="5" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G346" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H346" s="32" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I346" s="32" t="str">
+        <x:v>Private import</x:v>
+      </x:c>
+      <x:c r="J346" s="5" t="str">
+        <x:v>Dock travel binding pending</x:v>
+      </x:c>
+      <x:c r="K346" s="5" t="str">
+        <x:v>ocean-vessels/Prop_Ocean_TideSkiff.glb</x:v>
+      </x:c>
+      <x:c r="L346" s="5" t="str">
+        <x:v>9f34d5b569225a847599283e0d65d62e348b171305a09167fb4554fd2a1b2b18</x:v>
+      </x:c>
+      <x:c r="M346" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N346" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O346" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P346" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q346" s="5" t="str">
+        <x:v>Original Codex Blender mesh; private Unreal inspection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347">
+      <x:c r="A347" s="5" t="str">
+        <x:v>Prop_Ocean_CoralSubmarine</x:v>
+      </x:c>
+      <x:c r="B347" s="5" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C347" s="5" t="str">
+        <x:v>Ocean Realm</x:v>
+      </x:c>
+      <x:c r="D347" s="5" t="str">
+        <x:v>Submerged dock vessel; dive/helm presentation</x:v>
+      </x:c>
+      <x:c r="E347" s="5" t="n">
+        <x:v>6676</x:v>
+      </x:c>
+      <x:c r="F347" s="5" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G347" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H347" s="32" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I347" s="32" t="str">
+        <x:v>Private import</x:v>
+      </x:c>
+      <x:c r="J347" s="5" t="str">
+        <x:v>Dock travel binding pending</x:v>
+      </x:c>
+      <x:c r="K347" s="5" t="str">
+        <x:v>ocean-vessels/Prop_Ocean_CoralSubmarine.glb</x:v>
+      </x:c>
+      <x:c r="L347" s="5" t="str">
+        <x:v>f96f8b14a75d87bc92dd44b841790a7da36fb87f22c7827ebe8dd6da658fab82</x:v>
+      </x:c>
+      <x:c r="M347" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N347" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O347" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P347" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q347" s="5" t="str">
+        <x:v>Original Codex Blender mesh; private Unreal inspection</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348">
+      <x:c r="A348" s="5" t="str">
+        <x:v>Prop_Ocean_HarbourDock</x:v>
+      </x:c>
+      <x:c r="B348" s="5" t="str">
+        <x:v>Prop</x:v>
+      </x:c>
+      <x:c r="C348" s="5" t="str">
+        <x:v>Ocean Realm</x:v>
+      </x:c>
+      <x:c r="D348" s="5" t="str">
+        <x:v>Modular harbour dressing; existing pier collision presentation</x:v>
+      </x:c>
+      <x:c r="E348" s="5" t="n">
+        <x:v>8352</x:v>
+      </x:c>
+      <x:c r="F348" s="5" t="str">
+        <x:v>static</x:v>
+      </x:c>
+      <x:c r="G348" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H348" s="32" t="str">
+        <x:v>Validated</x:v>
+      </x:c>
+      <x:c r="I348" s="32" t="str">
+        <x:v>Private import</x:v>
+      </x:c>
+      <x:c r="J348" s="5" t="str">
+        <x:v>Dock travel binding pending</x:v>
+      </x:c>
+      <x:c r="K348" s="5" t="str">
+        <x:v>ocean-vessels/Prop_Ocean_HarbourDock.glb</x:v>
+      </x:c>
+      <x:c r="L348" s="5" t="str">
+        <x:v>bc25893595a78c78553b45f74e04496aacfc2e619d4b7d6f44ea919276af9a73</x:v>
+      </x:c>
+      <x:c r="M348" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N348" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="O348" s="5" t="str">
+        <x:v>n.a.</x:v>
+      </x:c>
+      <x:c r="P348" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q348" s="5" t="str">
+        <x:v>Original Codex Blender mesh; private Unreal inspection</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18989,12 +19148,22 @@
       <x:c r="K49" s="2"/>
       <x:c r="L49" s="2"/>
     </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="2"/>
-      <x:c r="B50" s="2"/>
-      <x:c r="C50" s="2"/>
-      <x:c r="D50" s="2"/>
-      <x:c r="E50" s="2"/>
+    <x:row r="50" ht="88" customHeight="1">
+      <x:c r="A50" s="4" t="str">
+        <x:v>OCE10</x:v>
+      </x:c>
+      <x:c r="B50" s="4" t="str">
+        <x:v>Boat and submarine boarding at docks</x:v>
+      </x:c>
+      <x:c r="C50" s="4" t="str">
+        <x:v>Original skiff, submarine and dock; waterline pivots and +X forward</x:v>
+      </x:c>
+      <x:c r="D50" s="4" t="str">
+        <x:v>3 static exports validated; private Unreal harbor capture verified</x:v>
+      </x:c>
+      <x:c r="E50" s="4" t="str">
+        <x:v>Boarding, hull collision and destination streaming acceptance pending</x:v>
+      </x:c>
       <x:c r="F50" s="2"/>
       <x:c r="G50" s="2"/>
       <x:c r="H50" s="2"/>
@@ -19247,14 +19416,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D30,"Verified")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(D8:D31,"Verified")</x:f>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D30,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D31,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -19860,6 +20029,32 @@
       </x:c>
       <x:c r="H30" s="5" t="str">
         <x:v>Clear revision removes old mesh; appearance/travel pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="88" customHeight="1">
+      <x:c r="A31" s="5" t="str">
+        <x:v>HARBOR-RENDER</x:v>
+      </x:c>
+      <x:c r="B31" s="5" t="str">
+        <x:v>Private Ocean harbor inspection</x:v>
+      </x:c>
+      <x:c r="C31" s="5" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D31" s="30" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E31" s="29" t="n">
+        <x:v>34.656</x:v>
+      </x:c>
+      <x:c r="F31" s="5" t="str">
+        <x:v>Java server startup plus native engine startup and HTTP scenario</x:v>
+      </x:c>
+      <x:c r="G31" s="5" t="str">
+        <x:v>ocean-scene-http-proof.json</x:v>
+      </x:c>
+      <x:c r="H31" s="5" t="str">
+        <x:v>64 chunks and 3 props rendered; controls and realm transfer pending</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Verify fitted Ocean hulls in native physics and remote clients
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R0a1380cdfba0446d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R8f3663ecf7064541"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rbf9a92559ed64729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R9b3a8cafae154b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Rc6237692198f4263"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R80b3d52017f14f99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R23ae81e83a7045a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rf48d8d8c7c9d4cbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -132,7 +132,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -215,6 +215,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -19172,12 +19178,22 @@
       <x:c r="K50" s="2"/>
       <x:c r="L50" s="2"/>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
-      <x:c r="E51" s="2"/>
+    <x:row r="51" ht="64" customHeight="1">
+      <x:c r="A51" s="4" t="str">
+        <x:v>OCE11</x:v>
+      </x:c>
+      <x:c r="B51" s="4" t="str">
+        <x:v>Vessel body collision fits its art</x:v>
+      </x:c>
+      <x:c r="C51" s="4" t="str">
+        <x:v>Bounded unoccupied authority configuration replicated to peers</x:v>
+      </x:c>
+      <x:c r="D51" s="4" t="str">
+        <x:v>Native wall sweeps and two-process profile replication verified</x:v>
+      </x:c>
+      <x:c r="E51" s="4" t="str">
+        <x:v>Rendered piloting, rotation clearance and dock travel pending</x:v>
+      </x:c>
       <x:c r="F51" s="2"/>
       <x:c r="G51" s="2"/>
       <x:c r="H51" s="2"/>
@@ -19416,14 +19432,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D31,"Verified")</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTIF(D8:D34,"Verified")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D31,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D34,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20055,6 +20071,84 @@
       </x:c>
       <x:c r="H31" s="5" t="str">
         <x:v>64 chunks and 3 props rendered; controls and realm transfer pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="64" customHeight="1">
+      <x:c r="A32" s="4" t="str">
+        <x:v>BUILD-HULL</x:v>
+      </x:c>
+      <x:c r="B32" s="4" t="str">
+        <x:v>Full plugin with configurable hulls</x:v>
+      </x:c>
+      <x:c r="C32" s="4" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D32" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E32" s="38" t="n">
+        <x:v>210.96</x:v>
+      </x:c>
+      <x:c r="F32" s="4" t="str">
+        <x:v>Full 136-file source snapshot</x:v>
+      </x:c>
+      <x:c r="G32" s="4" t="str">
+        <x:v>ocean-hull-profile-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H32" s="4" t="str">
+        <x:v>No shared editor or fixture overlay in production build</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="64" customHeight="1">
+      <x:c r="A33" s="4" t="str">
+        <x:v>HULL-PROFILE</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="str">
+        <x:v>Daedalus.Ocean.HullProfile</x:v>
+      </x:c>
+      <x:c r="C33" s="4" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D33" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E33" s="38" t="n">
+        <x:v>0.014085199683904648</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="str">
+        <x:v>Native test body; excludes startup</x:v>
+      </x:c>
+      <x:c r="G33" s="4" t="str">
+        <x:v>ocean-hull-profile-runtime-proof.json</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="str">
+        <x:v>Bounds, overlap, occupied refusal and real wall sweeps</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="64" customHeight="1">
+      <x:c r="A34" s="4" t="str">
+        <x:v>HULL-NET</x:v>
+      </x:c>
+      <x:c r="B34" s="4" t="str">
+        <x:v>Replicated boat and submarine body dimensions</x:v>
+      </x:c>
+      <x:c r="C34" s="4" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D34" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E34" s="38" t="n">
+        <x:v>47.797</x:v>
+      </x:c>
+      <x:c r="F34" s="4" t="str">
+        <x:v>Sum of two separate server/client scenarios</x:v>
+      </x:c>
+      <x:c r="G34" s="4" t="str">
+        <x:v>ocean-hull-profile-network-proof.json</x:v>
+      </x:c>
+      <x:c r="H34" s="4" t="str">
+        <x:v>Both client colliders match; client resize refused; rendered travel pending</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(ocean): prove effective URL refusal through real Unreal HTTP requests
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="Rc6237692198f4263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R80b3d52017f14f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R23ae81e83a7045a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rf48d8d8c7c9d4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R61ebf4714d8f4139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rbb4d10df70254f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rd4597cadbf674f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R37ea79fe416446fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19202,12 +19202,22 @@
       <x:c r="K51" s="2"/>
       <x:c r="L51" s="2"/>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="2"/>
-      <x:c r="B52" s="2"/>
-      <x:c r="C52" s="2"/>
-      <x:c r="D52" s="2"/>
-      <x:c r="E52" s="2"/>
+    <x:row r="52" ht="80" customHeight="1">
+      <x:c r="A52" s="4" t="str">
+        <x:v>OCE12</x:v>
+      </x:c>
+      <x:c r="B52" s="4" t="str">
+        <x:v>Accept chunks only from exact requested URL</x:v>
+      </x:c>
+      <x:c r="C52" s="4" t="str">
+        <x:v>Case-sensitive effective URL comparison before payload publication</x:v>
+      </x:c>
+      <x:c r="D52" s="4" t="str">
+        <x:v>Direct accepted. Path, port and path-case redirects refused in actual UE.</x:v>
+      </x:c>
+      <x:c r="E52" s="4" t="str">
+        <x:v>TLS, credential forwarding policy and live authenticated travel remain open.</x:v>
+      </x:c>
       <x:c r="F52" s="2"/>
       <x:c r="G52" s="2"/>
       <x:c r="H52" s="2"/>
@@ -19432,14 +19442,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D34,"Verified")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIF(D8:D36,"Verified")</x:f>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D34,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D36,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20149,6 +20159,58 @@
       </x:c>
       <x:c r="H34" s="4" t="str">
         <x:v>Both client colliders match; client resize refused; rendered travel pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="80" customHeight="1">
+      <x:c r="A35" s="4" t="str">
+        <x:v>BUILD-URL</x:v>
+      </x:c>
+      <x:c r="B35" s="4" t="str">
+        <x:v>Full plugin with effective URL check</x:v>
+      </x:c>
+      <x:c r="C35" s="4" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D35" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E35" s="38" t="n">
+        <x:v>220.56</x:v>
+      </x:c>
+      <x:c r="F35" s="4" t="str">
+        <x:v>148-file production snapshot dab439d6</x:v>
+      </x:c>
+      <x:c r="G35" s="4" t="str">
+        <x:v>ocean-effective-url-build-proof.json</x:v>
+      </x:c>
+      <x:c r="H35" s="4" t="str">
+        <x:v>Five native Ocean tests passed. Later main metadata fixes are outside this snapshot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="80" customHeight="1">
+      <x:c r="A36" s="4" t="str">
+        <x:v>HTTP-URL</x:v>
+      </x:c>
+      <x:c r="B36" s="4" t="str">
+        <x:v>Direct response and three redirect refusals</x:v>
+      </x:c>
+      <x:c r="C36" s="4" t="str">
+        <x:v>Ocean</x:v>
+      </x:c>
+      <x:c r="D36" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E36" s="38" t="n">
+        <x:v>38.407000000000004</x:v>
+      </x:c>
+      <x:c r="F36" s="4" t="str">
+        <x:v>Four sequential UE loopback processes</x:v>
+      </x:c>
+      <x:c r="G36" s="4" t="str">
+        <x:v>ocean-effective-url-redirect-proof.json</x:v>
+      </x:c>
+      <x:c r="H36" s="4" t="str">
+        <x:v>Fixture build 261.13s. Same-origin credential forwarded. TLS and pre-forward prevention unproven.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: track scoped battle cast build and native clip verification
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R61ebf4714d8f4139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rbb4d10df70254f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rd4597cadbf674f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R37ea79fe416446fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R5447bfec101a49cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rcaa0a83154e1447c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdbc655ec6b854b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R7d87b4eb1ce0478f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19226,12 +19226,22 @@
       <x:c r="K52" s="2"/>
       <x:c r="L52" s="2"/>
     </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="2"/>
-      <x:c r="B53" s="2"/>
-      <x:c r="C53" s="2"/>
-      <x:c r="D53" s="2"/>
-      <x:c r="E53" s="2"/>
+    <x:row r="53" ht="80" customHeight="1">
+      <x:c r="A53" s="4" t="str">
+        <x:v>PORT11</x:v>
+      </x:c>
+      <x:c r="B53" s="4" t="str">
+        <x:v>Each battle character uses its own skeleton clips</x:v>
+      </x:c>
+      <x:c r="C53" s="4" t="str">
+        <x:v>Bounded folder-local discovery with compatible explicit overrides</x:v>
+      </x:c>
+      <x:c r="D53" s="4" t="str">
+        <x:v>Synthetic native selection verified for two distinct skeletons</x:v>
+      </x:c>
+      <x:c r="E53" s="4" t="str">
+        <x:v>Imported clip names, director wiring, idle return and rendered battle still pending.</x:v>
+      </x:c>
       <x:c r="F53" s="2"/>
       <x:c r="G53" s="2"/>
       <x:c r="H53" s="2"/>
@@ -19442,14 +19452,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D36,"Verified")</x:f>
-        <x:v>24</x:v>
+        <x:f>COUNTIF(D8:D38,"Verified")</x:f>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D36,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D38,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20211,6 +20221,58 @@
       </x:c>
       <x:c r="H36" s="4" t="str">
         <x:v>Fixture build 261.13s. Same-origin credential forwarded. TLS and pre-forward prevention unproven.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="80" customHeight="1">
+      <x:c r="A37" s="4" t="str">
+        <x:v>BUILD-CAST</x:v>
+      </x:c>
+      <x:c r="B37" s="4" t="str">
+        <x:v>Full plugin with per-mesh battle clips</x:v>
+      </x:c>
+      <x:c r="C37" s="4" t="str">
+        <x:v>All casts</x:v>
+      </x:c>
+      <x:c r="D37" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E37" s="38" t="n">
+        <x:v>236.33</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="str">
+        <x:v>151-file snapshot c419b8b4</x:v>
+      </x:c>
+      <x:c r="G37" s="4" t="str">
+        <x:v>battle-cast-animation-proof.json</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="str">
+        <x:v>Later utility interfaces are outside this build snapshot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="80" customHeight="1">
+      <x:c r="A38" s="4" t="str">
+        <x:v>CAST-CLIPS</x:v>
+      </x:c>
+      <x:c r="B38" s="4" t="str">
+        <x:v>Daedalus.Battle.CastAnimations</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="str">
+        <x:v>All casts</x:v>
+      </x:c>
+      <x:c r="D38" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E38" s="38" t="n">
+        <x:v>0.03842709958553314</x:v>
+      </x:c>
+      <x:c r="F38" s="4" t="str">
+        <x:v>Native synthetic two-skeleton test body</x:v>
+      </x:c>
+      <x:c r="G38" s="4" t="str">
+        <x:v>battle-cast-animation-proof.json</x:v>
+      </x:c>
+      <x:c r="H38" s="4" t="str">
+        <x:v>Own clips, override compatibility, missing/null refusal. Imported art and rendered battle remain open.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: broaden verification heading to cover battle and Ocean
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R5447bfec101a49cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rcaa0a83154e1447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdbc655ec6b854b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R7d87b4eb1ce0478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R40f9503f8eaf4d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rc20c7c3cfb1141f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdc2ad958fb1542c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R6698e629f5d04dba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19439,7 +19439,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="26" t="str">
-        <x:v>Native ocean verification runs</x:v>
+        <x:v>Native runtime verification runs</x:v>
       </x:c>
     </x:row>
     <x:row r="4">

</xml_diff>

<commit_message>
test(battle): prove all thirteen actual imported Gallery clip bindings
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R40f9503f8eaf4d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="Rc20c7c3cfb1141f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rdc2ad958fb1542c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R6698e629f5d04dba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R023e7bd6bf6e4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R54f6b29730f54968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rff315c26aff3466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R3dcce4388f9e4f39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19237,10 +19237,10 @@
         <x:v>Bounded folder-local discovery with compatible explicit overrides</x:v>
       </x:c>
       <x:c r="D53" s="4" t="str">
-        <x:v>Synthetic native selection verified for two distinct skeletons</x:v>
+        <x:v>Two synthetic skeletons plus 13 actual imported Gallery casts verified</x:v>
       </x:c>
       <x:c r="E53" s="4" t="str">
-        <x:v>Imported clip names, director wiring, idle return and rendered battle still pending.</x:v>
+        <x:v>Director wiring, idle return, playback, cooking and rendered battle still pending.</x:v>
       </x:c>
       <x:c r="F53" s="2"/>
       <x:c r="G53" s="2"/>
@@ -19452,14 +19452,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D38,"Verified")</x:f>
-        <x:v>26</x:v>
+        <x:f>COUNTIF(D8:D39,"Verified")</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D38,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D39,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20237,16 +20237,16 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="E37" s="38" t="n">
-        <x:v>236.33</x:v>
+        <x:v>242.56</x:v>
       </x:c>
       <x:c r="F37" s="4" t="str">
-        <x:v>151-file snapshot c419b8b4</x:v>
+        <x:v>159-file snapshot 36adcecc</x:v>
       </x:c>
       <x:c r="G37" s="4" t="str">
         <x:v>battle-cast-animation-proof.json</x:v>
       </x:c>
       <x:c r="H37" s="4" t="str">
-        <x:v>Later utility interfaces are outside this build snapshot.</x:v>
+        <x:v>Later Java cabinets and main fixes are outside this build snapshot.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="80" customHeight="1">
@@ -20263,7 +20263,7 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="E38" s="38" t="n">
-        <x:v>0.03842709958553314</x:v>
+        <x:v>0.02282389998435974</x:v>
       </x:c>
       <x:c r="F38" s="4" t="str">
         <x:v>Native synthetic two-skeleton test body</x:v>
@@ -20272,7 +20272,33 @@
         <x:v>battle-cast-animation-proof.json</x:v>
       </x:c>
       <x:c r="H38" s="4" t="str">
-        <x:v>Own clips, override compatibility, missing/null refusal. Imported art and rendered battle remain open.</x:v>
+        <x:v>Concatenated import names. Test errors/warnings 0/0; editor 0/1 (layout notice).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="80" customHeight="1">
+      <x:c r="A39" s="4" t="str">
+        <x:v>CAST-IMPORT</x:v>
+      </x:c>
+      <x:c r="B39" s="4" t="str">
+        <x:v>13 Gallery meshes and 26 attack/hurt bindings</x:v>
+      </x:c>
+      <x:c r="C39" s="4" t="str">
+        <x:v>Gallery</x:v>
+      </x:c>
+      <x:c r="D39" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E39" s="38" t="n">
+        <x:v>0.68</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="str">
+        <x:v>Commandlet body only, excludes startup</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="str">
+        <x:v>battle-cast-imported-proof.json</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="str">
+        <x:v>152 copied art hashes intact. Editor errors/warnings 0/0. Playback/rendering still pending.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs(realms): track discovery checks without changing prior asset or verification records
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R023e7bd6bf6e4b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R54f6b29730f54968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="Rff315c26aff3466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R3dcce4388f9e4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R8d59d978cc504f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R95ce1c4a5dd64fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R6d4af758d069471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R56e7db0ea2334850"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19250,12 +19250,22 @@
       <x:c r="K53" s="2"/>
       <x:c r="L53" s="2"/>
     </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="2"/>
-      <x:c r="B54" s="2"/>
-      <x:c r="C54" s="2"/>
-      <x:c r="D54" s="2"/>
-      <x:c r="E54" s="2"/>
+    <x:row r="54" ht="96" customHeight="1">
+      <x:c r="A54" s="4" t="str">
+        <x:v>SYS01</x:v>
+      </x:c>
+      <x:c r="B54" s="4" t="str">
+        <x:v>Clients discover each realm data provider</x:v>
+      </x:c>
+      <x:c r="C54" s="4" t="str">
+        <x:v>Canonical identity, protocol and same-origin routes without duplicating terrain</x:v>
+      </x:c>
+      <x:c r="D54" s="4" t="str">
+        <x:v>Production JWT HTTP discovery to Ocean chunk read verified</x:v>
+      </x:c>
+      <x:c r="E54" s="4" t="str">
+        <x:v>Player transfer, district routing, Unreal subscription and hosting still pending.</x:v>
+      </x:c>
       <x:c r="F54" s="2"/>
       <x:c r="G54" s="2"/>
       <x:c r="H54" s="2"/>
@@ -19439,7 +19449,7 @@
   <x:sheetData>
     <x:row r="2">
       <x:c r="A2" s="26" t="str">
-        <x:v>Native runtime verification runs</x:v>
+        <x:v>Runtime verification runs</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -19452,14 +19462,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D39,"Verified")</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTIF(D8:D40,"Verified")</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D39,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D40,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20299,6 +20309,32 @@
       </x:c>
       <x:c r="H39" s="4" t="str">
         <x:v>152 copied art hashes intact. Editor errors/warnings 0/0. Playback/rendering still pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="96" customHeight="1">
+      <x:c r="A40" s="4" t="str">
+        <x:v>REALM-DIR</x:v>
+      </x:c>
+      <x:c r="B40" s="4" t="str">
+        <x:v>Authenticated provider discovery and advertised Ocean read</x:v>
+      </x:c>
+      <x:c r="C40" s="4" t="str">
+        <x:v>WorldHub + Ocean</x:v>
+      </x:c>
+      <x:c r="D40" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E40" s="38" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="F40" s="4" t="str">
+        <x:v>Full server reactor verify. 719 core / 796 server tests.</x:v>
+      </x:c>
+      <x:c r="G40" s="4" t="str">
+        <x:v>realm-directory-proof.json</x:v>
+      </x:c>
+      <x:c r="H40" s="4" t="str">
+        <x:v>10 focused checks also pass in 51.582s. No travel, Unreal loading or hosting claim.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(realms): refresh canonical binding proof and tracker from full verification
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R8d59d978cc504f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R95ce1c4a5dd64fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R6d4af758d069471a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="R56e7db0ea2334850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R1856b73b8d034a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R1384d56b748e48e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R4f08c246a48a409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Re29072f8235c4a28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19258,7 +19258,7 @@
         <x:v>Clients discover each realm data provider</x:v>
       </x:c>
       <x:c r="C54" s="4" t="str">
-        <x:v>Canonical identity, protocol and same-origin routes without duplicating terrain</x:v>
+        <x:v>Storage IDs, canonical session/catalog bindings and same-origin routes without duplicating terrain</x:v>
       </x:c>
       <x:c r="D54" s="4" t="str">
         <x:v>Production JWT HTTP discovery to Ocean chunk read verified</x:v>
@@ -20325,16 +20325,16 @@
         <x:v>Verified</x:v>
       </x:c>
       <x:c r="E40" s="38" t="n">
-        <x:v>207</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
-        <x:v>Full server reactor verify. 719 core / 796 server tests.</x:v>
+        <x:v>Full server reactor verify. 719 core / 799 server tests.</x:v>
       </x:c>
       <x:c r="G40" s="4" t="str">
         <x:v>realm-directory-proof.json</x:v>
       </x:c>
       <x:c r="H40" s="4" t="str">
-        <x:v>10 focused checks also pass in 51.582s. No travel, Unreal loading or hosting claim.</x:v>
+        <x:v>13 focused checks also pass in 46.273s. No travel, Unreal loading or hosting claim.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record land API restart proof and update production tracker
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R1856b73b8d034a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R1384d56b748e48e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R4f08c246a48a409f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Re29072f8235c4a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="1" r:id="R8c2e31db28744c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" r:id="R462499fc8ca3499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" r:id="R8225b473ece14fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" r:id="Rbaecf1f2b8f044d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19274,12 +19274,22 @@
       <x:c r="K54" s="2"/>
       <x:c r="L54" s="2"/>
     </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="2"/>
-      <x:c r="B55" s="2"/>
-      <x:c r="C55" s="2"/>
-      <x:c r="D55" s="2"/>
-      <x:c r="E55" s="2"/>
+    <x:row r="55" ht="110" customHeight="1">
+      <x:c r="A55" s="4" t="str">
+        <x:v>SYS02</x:v>
+      </x:c>
+      <x:c r="B55" s="4" t="str">
+        <x:v>Consistent land numbers in every realm</x:v>
+      </x:c>
+      <x:c r="C55" s="4" t="str">
+        <x:v>100x100 spiral and 10x10 districts. Estate identity is independent of current position.</x:v>
+      </x:c>
+      <x:c r="D55" s="4" t="str">
+        <x:v>All 10,000 cells and 40,000 estate candidates agree across languages.</x:v>
+      </x:c>
+      <x:c r="E55" s="4" t="str">
+        <x:v>Grid addresses do not establish mintable supply or ownership.</x:v>
+      </x:c>
       <x:c r="F55" s="2"/>
       <x:c r="G55" s="2"/>
       <x:c r="H55" s="2"/>
@@ -19288,12 +19298,22 @@
       <x:c r="K55" s="2"/>
       <x:c r="L55" s="2"/>
     </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="2"/>
-      <x:c r="B56" s="2"/>
-      <x:c r="C56" s="2"/>
-      <x:c r="D56" s="2"/>
-      <x:c r="E56" s="2"/>
+    <x:row r="56" ht="110" customHeight="1">
+      <x:c r="A56" s="4" t="str">
+        <x:v>SYS03</x:v>
+      </x:c>
+      <x:c r="B56" s="4" t="str">
+        <x:v>Estates can move while retaining identity</x:v>
+      </x:c>
+      <x:c r="C56" s="4" t="str">
+        <x:v>Explicit hub reservation and overlap checks. Atomic local snapshots and revision conflicts.</x:v>
+      </x:c>
+      <x:c r="D56" s="4" t="str">
+        <x:v>Restart and 10,000-estate persistence verified.</x:v>
+      </x:c>
+      <x:c r="E56" s="4" t="str">
+        <x:v>Authorized move API, production backups and distributed authority remain pending.</x:v>
+      </x:c>
       <x:c r="F56" s="2"/>
       <x:c r="G56" s="2"/>
       <x:c r="H56" s="2"/>
@@ -19302,12 +19322,22 @@
       <x:c r="K56" s="2"/>
       <x:c r="L56" s="2"/>
     </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="2"/>
-      <x:c r="B57" s="2"/>
-      <x:c r="C57" s="2"/>
-      <x:c r="D57" s="2"/>
-      <x:c r="E57" s="2"/>
+    <x:row r="57" ht="110" customHeight="1">
+      <x:c r="A57" s="4" t="str">
+        <x:v>SYS04</x:v>
+      </x:c>
+      <x:c r="B57" s="4" t="str">
+        <x:v>Load placed lands one district at a time</x:v>
+      </x:c>
+      <x:c r="C57" s="4" t="str">
+        <x:v>JWT district API returns current cells, seed strings and layout revision.</x:v>
+      </x:c>
+      <x:c r="D57" s="4" t="str">
+        <x:v>Actual HTTP restart and identity-preserving move verified.</x:v>
+      </x:c>
+      <x:c r="E57" s="4" t="str">
+        <x:v>Unreal subscription, terrain generation and editor layout import remain pending.</x:v>
+      </x:c>
       <x:c r="F57" s="2"/>
       <x:c r="G57" s="2"/>
       <x:c r="H57" s="2"/>
@@ -19462,14 +19492,14 @@
         <x:v>Verified runs</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:f>COUNTIF(D8:D40,"Verified")</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIF(D8:D43,"Verified")</x:f>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Pending checks</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>COUNTIF(D8:D40,"Pending")</x:f>
+        <x:f>COUNTIF(D8:D43,"Pending")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -20335,6 +20365,84 @@
       </x:c>
       <x:c r="H40" s="4" t="str">
         <x:v>13 focused checks also pass in 46.273s. No travel, Unreal loading or hosting claim.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="110" customHeight="1">
+      <x:c r="A41" s="4" t="str">
+        <x:v>LAND-GRID</x:v>
+      </x:c>
+      <x:c r="B41" s="4" t="str">
+        <x:v>Shared Java, native and Python plot addressing</x:v>
+      </x:c>
+      <x:c r="C41" s="4" t="str">
+        <x:v>All realms</x:v>
+      </x:c>
+      <x:c r="D41" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E41" s="38" t="n">
+        <x:v>46.197</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="str">
+        <x:v>723 core tests. 10,000 cell and 40,000 estate parity rows.</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="str">
+        <x:v>land-grid-parity-proof.json</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="str">
+        <x:v>Addressing only. Native gcc/clang CI checks Python against the Java-tested digest.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="110" customHeight="1">
+      <x:c r="A42" s="4" t="str">
+        <x:v>LAND-STORE</x:v>
+      </x:c>
+      <x:c r="B42" s="4" t="str">
+        <x:v>Persistent physical estate placement</x:v>
+      </x:c>
+      <x:c r="C42" s="4" t="str">
+        <x:v>All realms</x:v>
+      </x:c>
+      <x:c r="D42" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E42" s="38" t="n">
+        <x:v>50.348</x:v>
+      </x:c>
+      <x:c r="F42" s="4" t="str">
+        <x:v>731 core tests. Restart, overlap, hub and stale-writer checks.</x:v>
+      </x:c>
+      <x:c r="G42" s="4" t="str">
+        <x:v>realm-layout-store-proof.json</x:v>
+      </x:c>
+      <x:c r="H42" s="4" t="str">
+        <x:v>10,000-estate snapshot. No wallet ownership, distributed store or editor-import claim.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="110" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>LAND-API</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>Authenticated district reads after server restart</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>Java host</x:v>
+      </x:c>
+      <x:c r="D43" s="37" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="E43" s="38" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="F43" s="4" t="str">
+        <x:v>731 core / 805 server tests.</x:v>
+      </x:c>
+      <x:c r="G43" s="4" t="str">
+        <x:v>realm-land-api-proof.json</x:v>
+      </x:c>
+      <x:c r="H43" s="4" t="str">
+        <x:v>Actual JWT HTTP restart, move, quota and corruption checks. Unreal consumer integration remains pending.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
registry: Super Island rows WZ08-09
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26772,7 +26772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28726,9 +28726,6 @@
           <t>Each land has a reason to trade: surplus and need</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -28756,9 +28753,6 @@
           <t>Water flows through the air since the shattering</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -28786,9 +28780,6 @@
           <t>Heal the planet; the smith needs copper and iron</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -28816,9 +28807,6 @@
           <t>The Keeper's Broken Circle</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -28846,9 +28834,6 @@
           <t>The inn cooks what the island grows</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -28876,9 +28861,6 @@
           <t>Each culture has an inn and a shop</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -28906,9 +28888,66 @@
           <t>Arks tow lands together</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>WZ08</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plot sockets Connect_E/N/W/S at +-120 m, 10 m deck, 16 m bridges (Lumenwake standard)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>voxel_super_island.py landings/bridges; Ultra's super_island_layout.py</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Blender export + manifest; tug/placement authority pending (ADR-065)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Owners bring purchased plots together by ship</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>WZ09</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Sky rivers as water connectors between member lakes</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>island_cluster._sky_river</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Blender export; Unreal water material pending</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Water flows through the air since the shattering</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ADR-066 Colony Ledger: M.U.L.E. loop + Animal Crossing day book + Arc Raiders raids, driven by realm chemistry and ecology (pure core, 10 tests); Excel tracker rows WZ10-15 + Team Claude sheet; registry
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -8,6 +8,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unreal verification" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemistry" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Claude 2026-10-14" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -26772,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28915,9 +28916,6 @@
           <t>Owners bring purchased plots together by ship</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -28945,9 +28943,186 @@
           <t>Water flows through the air since the shattering</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>WZ10</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Power unit built from island goods (gearbox copper+iron, shaft iron, rotor wind/water, crystal battery); rich/legendary lands start with a broken one to salvage</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Codex codex_salvage_assembly.py PowerUnit 86100; hero island power-unit site; island_chemistry power_unit</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Asset-only + chemistry; wiring/snapping/charge pending</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ENERGY feeds lamps, mill and ark</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>WZ11</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Colony Ledger: M.U.L.E. loop per realm - plots=deeds, outfitted workers (mule/power unit) per good family, production from chemistry x ecology (seral stage, biodiversity, season), energy tax, adjacency bonus</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>tools/economy/colony_ledger.py (pure core, 10 tests)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Core tested; server rounds/persistence/UI pending (ADR-066)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Richer colony -&gt; richer story -&gt; more items</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>WZ12</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Market day double auction per item; shop/inn standing buyers at family floor; sales ship as ark cargo (distance = rounds); prices walk to the crossing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>colony_ledger.market_day/settle_cargo</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Core tested; ADR-020 cargo binding pending</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Why islands trade: surplus and need</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>WZ13</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Round events from the chemistry: meteor (LEGENDARY), blight, raiders (stolen energy becomes a drifting hulk), wampus hunt, festival demand</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>colony_ledger.event</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Core tested</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>The world keeps changing</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>WZ14</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Day book (Animal Crossing): fish by season/hour, bugs by seral stage, fossils/starmetal shards, ripe fruit; collection (museum) first-of-kind bonus; charm; cast requests from the realm population plan (unicorn guides, kings, bakers...)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>colony_ledger.day_book/requests + data/art/&lt;realm&gt;/population-plan.json</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Core tested; NPC binding pending (PORT09 quest core)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Villagers pull items across realms</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>WZ15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Scavenge + defend (Arc Raiders): hulks and rich lands are loot sites; loot flies home as interceptable cargo; fences/lanterns/watchtowers/patrols/traps raise defence; caught raiders lose cargo</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>colony_ledger.raid/defend</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Core tested; native combat/boarding pending</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Raiding is the other way to fix a need</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -30811,4 +30986,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Team Claude deliverables, 2026-10-14 (Blender contest + economy core). Files in engines/unreal/art/claude-islands unless noted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hero island Skyfall</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Island_H39.fbx/.chemistry.json/_a,_b.png</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>tools/blender/hero_island.py (export_hero.py)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Blender exported + previewed</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sky river, waterfall, ocean basin, Heartstone, ores, cave, crater, town, herb ring, orchard, farm, dock+ark, power unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Five island types</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Island_H91_volcano, H124_frost, H125_mesa, H131_mire, H144_crystal</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hero_island.KINDS</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Blender exported + previewed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Five themed clusters</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cluster_{spring,summer,harvest,halloween,christmas}_7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tools/blender/island_cluster.py (export_cluster.py)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Blender exported + previewed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>halloween = LABYRINTH realm (LAB09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Super Island (Ultra standard)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SuperIsland_C3.fbx/.super-island.json</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_super_island.py (export_super.py)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Blender exported + previewed</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>256 m pitch, sockets +-120 m, 10 m deck, 16 m bridges</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Seeded chemistry</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tools/blender/island_chemistry.py + Chemistry sheet</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>profile(seed, realm)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Pure Python</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>per-realm tables; power_unit; goods surplus/need</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Colony Ledger core</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tools/economy/colony_ledger.py + test_colony_ledger.py</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADR-066</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>10/10 tests</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>M.U.L.E. + Animal Crossing day book + Arc Raiders raids</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>World Zero placed islands (editor contest, suspended)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ClaudeIsland_240..368 actors in DaedalusWorld</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>daedalus_claude_islands.py</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>129 saved</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>docs/mechanics/MECHANICS-REGISTRY.md, docs/adr/ADR-066-colony-ledger.md, docs/production/HANDOFF-2026-10-14-team-claude.md, UNREAL-RESEARCH-2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>on main</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ADR-066: fishing spots + sky-sea boats on the sky-river network (core + tests, rows WZ16-17)
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28970,9 +28970,6 @@
           <t>ENERGY feeds lamps, mill and ark</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -29000,9 +28997,6 @@
           <t>Richer colony -&gt; richer story -&gt; more items</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -29030,9 +29024,6 @@
           <t>Why islands trade: surplus and need</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -29060,9 +29051,6 @@
           <t>The world keeps changing</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -29090,9 +29078,6 @@
           <t>Villagers pull items across realms</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -29120,9 +29105,66 @@
           <t>Raiding is the other way to fix a need</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>WZ16</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Fishing off every island: lake, stream, pier, sky river, ocean basin spots; fish by chemistry water.fish, season, hour; rare catches to the collection</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>colony_ledger.fishing; hero island pier/dock/lake</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Core tested; rod/cast minigame pending</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>The Fisher buys the rest</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>WZ17</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Sky-sea boats: float on the water that floats in the sky (sky rivers, lakes, basins), cannot fly, must stay in water; sky-river network = travel graph; hull from plank+iron, sails from wool</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>colony_ledger.water_network; island_cluster/voxel_super_island sky rivers; hero island boat</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Core tested; vessel physics pending (OCE01/OCE10 boats)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Water sockets open sea lanes when plots are tugged together</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31079,7 +31121,6 @@
           <t>Blender exported + previewed</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -31210,7 +31251,6 @@
           <t>129 saved</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -31223,13 +31263,11 @@
           <t>docs/mechanics/MECHANICS-REGISTRY.md, docs/adr/ADR-066-colony-ledger.md, docs/production/HANDOFF-2026-10-14-team-claude.md, UNREAL-RESEARCH-2026-10-14.md</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>on main</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
tracker: WZ18 characters + Team Claude sheet rows; registry
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29132,9 +29132,6 @@
           <t>The Fisher buys the rest</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -29162,9 +29159,36 @@
           <t>Water sockets open sea lanes when plots are tugged together</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>WZ18</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Small characters that move: 64 voxel species (animals, birds, bees, carnivorous plants) on the shared 8-bone rig with Idle/Walk/Attack/Hurt; plants snap on Attack; ecology decides which live where (bees need meadow, hens scrub edge, deer old forest)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_creatures.py -&gt; engines/unreal/art/claude-creatures</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>GLB+FBX exported; native import/AI pending</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Birds and bees make the island feel alive; carnivorous plants guard and help (LAB10)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31036,7 +31060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31269,6 +31293,83 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hero batch 60 islands</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>claude-islands/heroes/Island_H1000..1059_&lt;kind&gt;.fbx + png + chemistry</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>export_heroes.py</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Blender exported</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>kind = seed % 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>64 voxel characters</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>claude-creatures/Creature_*.glb/.fbx/.json + contact sheet</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>voxel_creatures.py / export_creatures.py</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Blender exported, rigged + 4 clips</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>24 animals, 18 birds, 9 bees, 13 carnivorous plants</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Colony Ledger + fishing + boats</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tools/economy/colony_ledger.py</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ADR-066</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>11/11 tests</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
zombie waves in the ledger (5 escalating waves vs defence, salvage drops); tracker WZ19-20; registry
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29186,9 +29186,66 @@
           <t>Birds and bees make the island feel alive; carnivorous plants guard and help (LAB10)</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>WZ19</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Zombie apocalypse in waves: 24 zombie types (villager/farmer/miner/knight/king/pirate/bloated/crawler/runner/... frost/ember/crystal/mud, ghoul, wraith) arrive in 5 escalating waves; defence (WZ15) holds the line; fallen zombies drop salvage</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>voxel_creatures.ZOMBIES; colony_ledger.event zombie_wave</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Rigged GLB/FBX exporting; core tested; native spawning/combat pending (ADR-037)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Why you build walls, lanterns and towers</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>WZ20</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Dinosaurs (10) and sea creatures (19) + 70 animals incl. extinct ones; sea creatures live in sky-sea basins and ocean realm (OCE); dinos on legendary/old-forest lands</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>voxel_creatures.DINOS/SEA/ANIMALS</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Rigged GLB/FBX exporting; habitat binding via ecology pending</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Fishing, boating and exploring have something to meet</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31060,7 +31117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31368,7 +31425,33 @@
           <t>11/11 tests</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>171 voxel characters (v3)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>claude-creatures/</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>voxel_creatures.py</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>70 animals, 18 birds, 9 bees, 13 carnivorous plants, 8 fish, 24 zombies, 10 dinos, 19 sea</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
tracker WZ21-22 + sheet rows; architecture 14.6 dresser props, 206 species
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29213,9 +29213,6 @@
           <t>Why you build walls, lanterns and towers</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -29243,9 +29240,66 @@
           <t>Fishing, boating and exploring have something to meet</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>WZ21</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Dresser props library: 21 tree species x 4 stages (Prop_Tree_&lt;Species&gt;_&lt;Stage&gt;), 33 plants incl. crops + the six RingInfusion herbs, 12 shrubs, 18 cloud types/colours (storm, thunder, aurora, rainbow, rain, snow, ash, sunset...)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_flora.py -&gt; engines/unreal/art/claude-flora (ADR-054 names, bottom-centre pivots)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>FBX exporting; joins Dress() by name</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Species by ground (sand palms/saguaro, stone pines, grass the rest) per ADR-054</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>WZ22</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Insects (19) and burrowers (16): butterflies/dragonflies/fireflies hover, ants/spiders/scorpions crawl, worms/snails; moles/gophers/prairie dogs/meerkats/wombats/pangolins live in the ground (dig mechanic ADR-049 finds them)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>voxel_creatures INSECTS + ANIMALS burrowers</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Rigged GLB/FBX exporting</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Bugs by seral stage feed the day book; burrowers are what the pick turns up</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31117,7 +31171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31453,6 +31507,79 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>147 dresser props (flora + clouds)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>claude-flora/Prop_*.fbx/.json + sheet-&lt;family&gt;.png</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>voxel_flora.py / export_flora.py</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>206 voxel characters (v4)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>claude-creatures/</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>voxel_creatures.py</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>+19 insects, +16 burrowers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>200 hero islands + 20 clusters</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>claude-islands/heroes, clusters</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>export_heroes.py / export_clusters.py</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>heroes done; clusters finishing</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tracker WZ23 + sheet; architecture 14.7 farm kit
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29267,9 +29267,6 @@
           <t>Species by ground (sand palms/saguaro, stone pines, grass the rest) per ADR-054</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -29297,9 +29294,36 @@
           <t>Bugs by seral stage feed the day book; burrowers are what the pick turns up</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>WZ23</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Farming kit: 21 machines (tractors, plough, seeder, harrow, harvester, baler, sprayer, mower, wagons, pumps, windpump, tank - wheels spin), 16 buildings (barns, silos, coop, hives, greenhouse, pens, dovecote, sheds, smokehouse, dairy), 27 tools/fixtures (fences, gates, bales, troughs, churns, press, loom, anvil, stall...), 35 crops (vines/trellises, roots, greens, berries, grains, paddies, orchard rows)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_farm.py -&gt; engines/unreal/art/claude-farm</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>FBX exporting</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Farming = FOOD production in the Colony Ledger; machines are outfitted workers; crops follow the chemistry's soil/crops</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31171,7 +31195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31528,7 +31552,6 @@
           <t>exporting</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -31578,7 +31601,29 @@
           <t>heroes done; clusters finishing</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>99 farm props</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>claude-farm/Prop_{Machine,Farm,Crop}_*.fbx/.json + sheets</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>voxel_farm.py / export_farm.py</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: eggs/house-grave-sports/Sims realm — architecture §14.8–14.10, registry, tracker WZ24–26, handoff
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29321,9 +29321,87 @@
           <t>Farming = FOOD production in the Colony Ledger; machines are outfitted workers; crops follow the chemistry's soil/crops</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>WZ24</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Egg hatching (Adopt-Me style, PORT06 egg stages): 49 egg types (gemstone, diamond, gold, silver, silk, obsidian, ice, lava, cloud, holiday...) x Intact/Cracked/Hatching + Shiny = 196 props; rarity odds common 70/rare 22/legendary 7/ultra 1; each type hatches from a creature family rolled by the realm's ecology</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_eggs.py -&gt; engines/unreal/art/claude-eggs + eggs.manifest.json</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>FBX exporting</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Eggs are scavenge/fishing/festival finds in the Colony Ledger; hatched species joins the island population</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>WZ25</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>House equipment (69: beds, sofas, bathtubs, kitchen, lamps, fireplace, TV...), tombstones/graveyard (29: stones, crypt, coffin, open grave, zombie hand = zombie-wave spawn dressing), sports equipment (52: baseball, basketball, football, dodgeball, soccer, tennis, hockey, golf, bowling, bleachers, scoreboard) with throwable flags</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_props.py -&gt; engines/unreal/art/claude-props</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>FBX exporting</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Minigames catch / dodgeball / baseball / basketball / football use the throwable set; graves mark where waves rise</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>WZ26</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Sims realm complete build-out: 26-piece house kit (floors/walls/roofs/stairs/porch/pool/fence/mailbox), 18 practical machines mapped to real apps (scanner-&gt;PhotosToPDFPC, fax-&gt;fax-trident, photo bench-&gt;image-optimizer, study desk-&gt;synapse, server rack-&gt;LoadBalancerPro), 21 appliances (needs loop), House_Sims_Starter furnished 10x8 m house in 6 part meshes</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_sims.py -&gt; engines/unreal/art/claude-sims; docs/PRACTICAL-APPS.md</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>FBX exporting</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Lot = kit footprint on a PARCELS plot; machines run the practical apps; appliances feed FOOD/ENERGY needs in the ledger</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31195,7 +31273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31623,7 +31701,72 @@
           <t>exporting</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>196 egg props</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>claude-eggs/Prop_Egg_*.fbx/.json + eggs.manifest.json + sheet-egg.png</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>voxel_eggs.py / export_catalog.py eggs</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>150 house/grave/sport props</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>claude-props/Prop_{House,Grave,Sport}_* + sheets</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>voxel_props.py / export_catalog.py props</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>66 Sims assets + starter house</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>claude-sims/Build_Sims_*, Prop_Sims_*, House_Sims_Starter_* + sheets</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>voxel_sims.py / export_catalog.py sims</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: dragons — architecture §14.11, registry, tracker WZ27, handoff
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29400,6 +29400,33 @@
       <c r="E91" t="inlineStr">
         <is>
           <t>Lot = kit footprint on a PARCELS plot; machines run the practical apps; appliances feed FOOD/ENERGY needs in the ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>WZ27</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Flying dragons: 504 rigged (12 elements x 6 forms x 7 variants) - hover/cruise/dive/launch/lunge/breath clips; element matches realm chemistry (fire~volcano, ice~frost, crystal~crystal, gold~LEGENDARY)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_dragons.py -&gt; engines/unreal/art/claude-dragons + dragons.manifest.json</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>GLB/FBX exporting</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Raid event source in the Colony Ledger; tameable mount; fairy form hatches from dragon eggs (WZ24)</t>
         </is>
       </c>
     </row>
@@ -31273,7 +31300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31768,6 +31795,28 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>504 flying dragons</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>claude-dragons/Creature_Dragon*.glb/.fbx/.json + sheet-&lt;element&gt;.png</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>voxel_dragons.py / export_dragons.py</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: owls, HD island recipe, octets — architecture §14.12-14.14, registry, tracker WZ28-30, handoff, lessons
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29427,6 +29427,87 @@
       <c r="E92" t="inlineStr">
         <is>
           <t>Raid event source in the Colony Ledger; tameable mount; fairy form hatches from dragon eggs (WZ24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>WZ28</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Owls: 504 rigged (14 species x 6 plumages x 6 variants) - head-swivel idle, flight, silent-swoop action; night hunters/scouts</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_owls.py -&gt; engines/unreal/art/claude-owls + owls.manifest.json</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>GLB/FBX exported (379 s)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Ecology: hunt burrowers/insects, roost in Ancient trees; scouts in Living Island Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>WZ29</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>High-end islands: smooth authored terrain, strata keel with ore veins + Heartstone, clipped water, waterfall, sky-river tube, instanced foliage, lit town/farm/dock/shrine, UCX, LOD1/2, named PBR materials</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>tools/blender/hd_island.py -&gt; engines/unreal/art/claude-hd-islands</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>GLB/FBX exporting</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Same chemistry + terrace roles as voxel islands; addresses Codex audit gaps (materials, water slot, collision)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>WZ30</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Octets: 10 Super Islands of 8 connected HD islands (hub + ring of 7 at 256 m pitch), 14 rope bridges, 7 ring sky-streams, seasonal/holiday themes</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>tools/blender/hd_cluster.py -&gt; engines/unreal/art/claude-octets</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>GLB/FBX exporting</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Deeds stay per plot (Ultra standard); bridges = travel, sky streams = water network / sky-sea boat routes</t>
         </is>
       </c>
     </row>
@@ -31300,7 +31381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31817,6 +31898,50 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>504 owls</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>claude-owls/Creature_Owl*.glb/.fbx/.json + sheets</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>voxel_owls.py / export_owls.py</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>exported</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10 octets (80 HD islands)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>claude-octets/Octet_&lt;Theme&gt;_&lt;seed&gt;_*</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>hd_island.py / hd_cluster.py</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: HD island v2 gameplay hooks, kind landmarks, 20x speed path, 10k batch run — architecture §14.15, lessons, tracker WZ31
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29508,6 +29508,33 @@
       <c r="E95" t="inlineStr">
         <is>
           <t>Deeds stay per plot (Ultra standard); bridges = travel, sky streams = water network / sky-sea boat routes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>WZ31</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10,000 HD islands (seeds 10000-19999), each built from chemistry + mechanics data (gameplay hooks with cited sources: spawn, NPCs, ark, water, fishing, herbs/brews, orchard, livestock, crops, ore nodes, caves, crater, Power Unit, shop/inn, ledger goods, defense, nests, quests) + kind landmarks</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>tools/blender/hd_island.py + hd_batch.py -&gt; engines/unreal/art/claude-hd-islands/batch/&lt;thousands&gt;/ + index-worker*.jsonl</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>running (4 workers, ~1 island/s)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Every island json lists its mechanics_sources; Codex/Unreal can place NPCs, ores, water, quests from the gameplay rows</t>
         </is>
       </c>
     </row>
@@ -31381,7 +31408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31942,6 +31969,28 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10,000 HD islands</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>claude-hd-islands/batch/&lt;thousands&gt;/HDIsland_&lt;Kind&gt;_&lt;seed&gt;.*</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>hd_batch.py (4 workers)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: RPG realm casts — architecture §14.16, registry, tracker WZ32-33; prism item sheet spacing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29535,6 +29535,60 @@
       <c r="E96" t="inlineStr">
         <is>
           <t>Every island json lists its mechanics_sources; Codex/Unreal can place NPCs, ores, water, quests from the gameplay rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>WZ32</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Portal Realm cast: every Planned row of the population plan (49 enemy types, 50 friendly types incl. unicorn roles, 10 individuals each = 990) + 5 proposal bosses, rigged voxel bodies with 8 clips</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>tools/blender/realm_rpg_cast.py + export_rpg_cast.py -&gt; engines/unreal/art/claude-portal-cast (Mob_Portal_&lt;TYPE&gt;_Voxel_NN)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>jsons carry plan_id/variant_seed for data/art/portal/population-plan.json; native binding stays with Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>WZ33</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Prismheart Realm (ADR-067, original 16-bit crystal-era party RPG): 8 jobs x6 heroes, 30 monsters x5, 8 summons, 48 townsfolk, Duneback mounts, 12 structures (shrine, waystone, Skyfarer airship, castle gate, inn/shops/spell tower/chapel, dock), 24 items (chests, job weapons, potions, shards); realm chemistry</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>realm_rpg_cast.py, realm_prism_props.py, island_chemistry REALMS['PRISMHEART'] -&gt; claude-prism-cast, claude-prism-props</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>PRISM01-04 mechanics; REALMS.md row; battle rules / economy not decided</t>
         </is>
       </c>
     </row>
@@ -31408,7 +31462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31991,6 +32045,28 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Portal cast 995 + Prismheart 258 cast + 36 props</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>claude-portal-cast/, claude-prism-cast/, claude-prism-props/</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>realm_rpg_cast.py / realm_prism_props.py</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: random encounters — architecture §14.17, registry, tracker WZ34
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29589,6 +29589,33 @@
       <c r="E98" t="inlineStr">
         <is>
           <t>PRISM01-04 mechanics; REALMS.md row; battle rules / economy not decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>WZ34</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Random encounters for the Portal + Prismheart realms: 320 original enemy types (40 lines x 4 palette-swap tiers) with stats/behaviour/element/zones, encounter tables (zone step rates, weighted 1-6 enemy formations), 412 pixel battle sprites (8-bit and 16-bit styles), 320 rigged bodies</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_bestiary.py + render_battle_sprites.py -&gt; data/rpg/*.json, engines/unreal/art/claude-battle-sprites/&lt;realm&gt;/, claude-bestiary/&lt;realm&gt;/</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>sprites + data done; rigs exporting</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Battle screen draws sprites from sprites.json; the field rolls 1/steps_mean per step per zone</t>
         </is>
       </c>
     </row>
@@ -31462,7 +31489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32067,6 +32094,28 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>412 battle sprites + 320 bestiary types + encounter tables</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>claude-battle-sprites/, data/rpg/</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>rpg_bestiary.py / render_battle_sprites.py</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: battle-screen kit — architecture §14.18, lessons (AgX, Non-Color, numpy pixel art), tracker WZ32-35
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29556,7 +29556,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>exporting</t>
+          <t>exported (995 / 258 rigs)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -29583,7 +29583,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>exporting</t>
+          <t>exported (995 / 258 rigs)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -29610,12 +29610,39 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>sprites + data done; rigs exporting</t>
+          <t>done (412 sprites, 329 rigs incl. bosses)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
           <t>Battle screen draws sprites from sprites.json; the field rolls 1/steps_mean per step per zone</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>WZ35</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Battle-screen kit for both RPG realms: 35 zone backdrops (8-bit and 16-bit), party sprites (8 Prismheart jobs + Portal hero/sage/scout), 9 original Prismheart bosses (rigged + sprites + data/rpg/prism-bosses.json), 24 item icons</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_battle_kit.py, pixel_art.py, rpg_bosses.py -&gt; engines/unreal/art/claude-battle-kit/, claude-battle-sprites/prism/, claude-bestiary/prism-bosses/</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Battle screen = backdrop(zone) + enemy sprites(formation) + party sprites; bosses per shard dungeon</t>
         </is>
       </c>
     </row>
@@ -31489,7 +31516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32116,6 +32143,28 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Battle kit: 35 backdrops, 11 party, 9 bosses, 24 icons</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>claude-battle-kit/</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>rpg_battle_kit.py</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Docs: architecture 14.19 wildlife + tracker WZ36
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29643,6 +29643,33 @@
       <c r="E100" t="inlineStr">
         <is>
           <t>Battle screen = backdrop(zone) + enemy sprites(formation) + party sprites; bosses per shard dungeon</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>WZ36</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Wildlife: 504 rigged wolves (12 kinds x 6 coats x 7) + 504 rigged rabbits (12 breeds x 6 coats x 7) with new wolf/rabbit clips and predator-prey ecology; 258 aquatic plant props (43 species x 6 growth stages) tied to fish, spring purity, herbs and goods</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>tools/blender/voxel_wolves.py, voxel_rabbits.py, voxel_aquatic.py, export_wildlife.py -&gt; engines/unreal/art/claude-wolves, claude-rabbits, claude-aquatic</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>exporting</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Spawn tables read ECOLOGY (islands, pack size, warrens); place aquatic props by pivot family</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: architecture 14.20 spells + overworld, tracker WZ36 done, WZ37
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29664,12 +29664,39 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>exporting</t>
+          <t>done (504 wolves, 504 rabbits, 258 aquatic)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
           <t>Spawn tables read ECOLOGY (islands, pack size, warrens); place aquatic props by pivot family</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>WZ37</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>RPG realms: 51 animated battle spells (17 effects x 3 tiers) in 8-bit and 16-bit styles; overworld tile sets (23 terrain incl. animated water/lava/coasts + 14 landmarks) with encounter zones per tile and a demo overworld</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_spell_fx.py, rpg_world_map.py, pixel_png.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/spells, worldmap; data/rpg/spells.json, worldmap-tiles.json</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Field map = tiles; stepping on a tile rolls its encounter_zone; battle menu reads spells.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: merge 7 uncommitted Team-Claude-2026-10-14 rows found on the PC checkout (Copperfall, Willowglass, Miri v3, nursery station, SUPERPOLISH lane, native closeout, Sunspool) with WZ36/WZ37
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -31570,7 +31570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31580,6 +31580,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -32216,6 +32217,195 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Copperfall Ark Rest | 842401</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>task/floating-islands/copperfall-ark-rest-842401/</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>build_copperfall.py | uncommitted SHA256 1ecfa42b28008b7f6050ee16eb704654b8cec56b3643c8ce889f4f8c13e12d50</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SOURCE_AUTHORED; BAR_READ; RESOURCE_SLOT_PENDING</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>WORLD-ZERO / Aetherflow district. Owner production_checkpoint_evidence. Seven planned role groups/four sockets; counts unmeasured. Blend/FBX/GLB/render/native not run. Root coordinator verified source; comparable rendered BAR review required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Willowglass Refuge | 842402</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>task/floating-islands/willowglass-refuge-842402/</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>build_willowglass.py | uncommitted SHA256 79183615f7362451895d65749d5280a11ca671d3cff5ec868ff8a94a9a60e8c0</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>WATER_BAR_CORRECTION_AUTHORED; RESOURCE_SLOT_PENDING</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>WORLD-ZERO / Aetherflow district. Owner held_rainlight_dragons_audit. Suspended pond/underside/depth/two-scale ripples authored; ten roles/nine sockets planned. No Blend/export/render/native; measurements and comparisons pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Miri v3 | 160814</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>task/character-upgrades/miri-v3/</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>build_miri_v3.py | uncommitted SHA256 7597c4f711c397b0887ee896d3307b48db949f017fae477a478847162e62f6bb</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SOURCE_AUTHORED; BAR_READ; RESOURCE_SLOT_PENDING</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Owner claude_standards_audit; preserve original author. Existing courier/17 bones/three clips; four joint covers/two sole refinements planned. Emberthread/16-bit realm mapping remains provisional. No v3 Blend/export/render/native; native v2 untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Aetherflow nursery station | 617024</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>task/character-upgrades/aetherflow-habitat-r1/</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>build_nursery_station.py | uncommitted SHA256 1a5f8c3e5b66bd3fb59f68b7d1ac270bac4b1d771c686d41167ebdf7889052d0</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SOURCE_AUTHORED; BAR_READ; RESOURCE_SLOT_PENDING</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>WORLD-ZERO / Aetherflow district. Owner closeout_asset_count. Nine source fingerprints; fish/pond reference-only, excluded station export. No scene/export/render/native; day/dusk/player/jetty comparisons pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SUPERPOLISH reference lane</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Seven registry realms / fourteen PROVISIONAL reference slots</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ultra task 01a13bd0-4127-7dd1-b74f-7f3750012b9c; turn 01a13db1-70c0-74f3-ba56-f9e1c2253046; direct semantic ACK</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>ULTRA_ACCEPTED_SUPERPOLISH_LEAD; REFERENCES_PROVISIONAL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Island + land per realm; original asset owners retained; other builders bulk. Seven source IDs do NOT cover all named 8-bit/16-bit/N64/Hushveil requests. Reconcile those mappings with owners; OCEAN missing Chemistry. No reference READY/BAR/runtime pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Native closeout / remaining backlog</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CodexContest/codex-arcade-gameplay-0344.checkpoint.json</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PR147 a1bfd563736537ce065b6ccd461a828e5a21ab7d | receipt SHA20bbe284f767a99fac1e5e6cbeaf69f3b494d00c98d6954339f2d1787ea1b90a</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>39_BOUNDED_NATIVE_CHECKS_PASS; HUD_DEFECT_OPEN</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Operator owner report31503: production map/all101actors/user saves restored; physical controller unverified. HUD source owner resumed separately. App compile resource-pending; TMOG contract/tool-blocked. Photo notices closed PR4 83118805. Eighteen held packets unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sunspool Refuge | 861503</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-13/task-3/sunspool-refuge/r1/Sunspool_Refuge.blend; exports/Sunspool_Refuge.glb + .fbx</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>build source f7b9f82a + foliage 92abfb98; manifest SHA256 131af600f2b8ad9ae6cd2c19d7f82d71615d67ea4d1a34179028d6686f505bd1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>BLENDER_SAVED_EXPORTED; VISUAL_REVIEW_PENDING; NATIVE_FALSE</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>WORLD-ZERO; owner pootscoot. One authorized CPU2 Blender4.3.1 job exit0; 49,438 evaluated triangles/273 mesh-curve objects, 91.06x70.15x49.05m. Internal construct/export2.203s; peak not measured. Root verified Blend523805B c79df0a6..., GLB2714040B 9f6cca5f..., FBX1491292B cde7ae22.... Zero rendered views; separate review-render window31509 pending; no READY/intake grant.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: merge the PC checkout's uncommitted Team-Claude rows (native closeout update, Bulrush Sprout)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -31570,7 +31570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31580,6 +31580,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -32367,17 +32368,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PR147 a1bfd563736537ce065b6ccd461a828e5a21ab7d | receipt SHA20bbe284f767a99fac1e5e6cbeaf69f3b494d00c98d6954339f2d1787ea1b90a</t>
+          <t>HUD source integrated PR147 b8faf601. Latest asset receipt c97f17db. Game acceptance a1bfd563 is pre-fix.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>39_BOUNDED_NATIVE_CHECKS_PASS; HUD_DEFECT_OPEN</t>
+          <t>39_PRE_FIX_CHECKS_PASS; HUD_BUILD_PENDING</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Operator owner report31503: production map/all101actors/user saves restored; physical controller unverified. HUD source owner resumed separately. App compile resource-pending; TMOG contract/tool-blocked. Photo notices closed PR4 83118805. Eighteen held packets unchanged.</t>
+          <t>Sole operator codex-play-guard accepted ONE HUD serial build then release/app-next31542. At05:19UTC four hd_batch workers remain active,7230/10000 exports; no producer no-next-heavy ACK. Fresh3.77GiB physical/1.92GiB virtual free is not a build grant. No post-fix compile/load/visual proof. Physical controller unverified. Eighteen holds unchanged; global READY unknown. TMOG UI-tool blocked. Photo notices closed.</t>
         </is>
       </c>
     </row>
@@ -32405,6 +32406,33 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>WORLD-ZERO; owner pootscoot. One authorized CPU2 Blender4.3.1 job exit0; 49,438 evaluated triangles/273 mesh-curve objects, 91.06x70.15x49.05m. Internal construct/export2.203s; peak not measured. Root verified Blend523805B c79df0a6..., GLB2714040B 9f6cca5f..., FBX1491292B cde7ae22.... Zero rendered views; separate review-render window31509 pending; no READY/intake grant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bulrush Sprout | 1035e10d</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CodexContest/codex-bulrush-intake-0504.checkpoint.json; AquaticBulrushR1/known-save-readback.json</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Claude retained FBX1035e10dfad9afc65a5b442a530b2163c82d57cbfefbbf59973751e005ef6cbd. Importer codex-play-guard. PR147 c97f17db32b2cd36defcc38aa768b6e92f9dadc6.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>NATIVE_SAVED_ASSET_ONLY; APPEARANCE_REVIEW_PENDING</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Observed05:04:28UTC; one36-triangle StaticMesh saved true,39726B SHAd8d5f8d5b2331ab75f24ec00ce4cef423dfd472d192e0abb30d41f8776caa7ff.103Static+17Miri=120tracked packages;119prior hashes/101actors/camera/map unchanged. Import0.415584s/save0.229938s are native phases. No replay after late guard halt. Zero placement/world save. Appearance/collision/ecosystem unverified. Not an island or blanket READY.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: architecture 14.21 walkable towns, tracker WZ38
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29697,6 +29697,33 @@
       <c r="E102" t="inlineStr">
         <is>
           <t>Field map = tiles; stepping on a tile rolls its encounter_zone; battle menu reads spells.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>WZ38</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>RPG realms: walkable towns — 42 town tiles (walls, roofs, shop signs, furniture, fountain, chests), 8 villager types x 4 directions x 2 walk frames, demo town per realm; also battle UI kit + 5x7 pixel font</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_town.py, rpg_battle_ui.py, pixel_font.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/town, ui; data/rpg/town-tiles.json</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Town scene = tile grid from town-tiles.json; interact codes drive shops/inn/chests; NPC strips 8 frames</t>
         </is>
       </c>
     </row>
@@ -31580,7 +31607,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Docs: architecture 14.22 interiors, tracker WZ39
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29724,6 +29724,33 @@
       <c r="E103" t="inlineStr">
         <is>
           <t>Town scene = tile grid from town-tiles.json; interact codes drive shops/inn/chests; NPC strips 8 frames</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>WZ39</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>RPG realms: building interiors — item, weapon, armour/magic shops, inn, castle hall per realm; doors linked from the demo town; shop stock with prices/stats; magic shop sells tier-1/2 spells</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_interiors.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/interiors; data/rpg/interiors.json</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Door tile in town -&gt; interiors.json opened_by; exit mat returns to that door</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: architecture 14.23 dungeons, tracker WZ40
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29751,6 +29751,33 @@
       <c r="E104" t="inlineStr">
         <is>
           <t>Door tile in town -&gt; interiors.json opened_by; exit mat returns to that door</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>WZ40</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>RPG realms: dungeons — 7 themed tile sets, seeded multi-floor generator; 5 Portal dungeons + 9 Prismheart boss dungeons (46 floors) with stairs, chests/loot, hazards, encounter zones, sealed boss chambers</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_dungeon.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/dungeons; data/rpg/dungeons.json</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>done (reachability verified)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Floor grid + stair links drive the dungeon scene; encounter zone per floor rolls battles; BossGate opens the boss fight</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: architecture 14.24 menus + party, tracker WZ41
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29778,6 +29778,33 @@
       <c r="E105" t="inlineStr">
         <is>
           <t>Floor grid + stair links drive the dungeon scene; encounter zone per floor rolls battles; BossGate opens the boss fight</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>WZ41</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RPG realms: field menus (menu, status, equip, items, shop, save) x2 realms + starting party data (11 named heroes, stats, growth, gear, spells, join points) + 16 item icons</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_menus.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/menus; data/rpg/party.json, menus.json</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Engine builds the menus from menus.json windows/fields; party.json seeds a new game</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: architecture 14.25 music + sfx, tracker WZ42
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29805,6 +29805,33 @@
       <c r="E106" t="inlineStr">
         <is>
           <t>Engine builds the menus from menus.json windows/fields; party.json seeds a new game</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>WZ42</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>RPG realms: original chiptune music — 9 tracks in 8-bit (Portal) and 16-bit (Prismheart) arrangements with loop points — and 15 sound effects per realm</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_audio.py -&gt; engines/unreal/art/claude-audio/&lt;realm&gt;/; data/rpg/audio.json</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Map/screen -&gt; track via audio.json used_by; loop_end in samples</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: merge the PC checkout's uncommitted Team-Claude rows (night run)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -31705,7 +31705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31715,6 +31715,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -32480,12 +32481,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ULTRA_ACCEPTED_SUPERPOLISH_LEAD; REFERENCES_PROVISIONAL</t>
+          <t>ULTRA_ACCEPTED_LEAD; 14_PROVISIONAL_SLOTS; NEW_REQUEST_DELIVERED</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Island + land per realm; original asset owners retained; other builders bulk. Seven source IDs do NOT cover all named 8-bit/16-bit/N64/Hushveil requests. Reconcile those mappings with owners; OCEAN missing Chemistry. No reference READY/BAR/runtime pass.</t>
+          <t>Owner Ultra / buckwild-sol. Existing direct lead ACK retained. One island + land area per canonical realm. Seven registry IDs do not resolve every named 8-bit/16-bit/N64/Hushveil mapping. OCEAN uses floating harbor + seabed sector. Hub31701 requests continuous polish, ecology exemplar and owned repairs. Current request ACK/job/ETA pending. No reference BAR/native acceptance.</t>
         </is>
       </c>
     </row>
@@ -32502,17 +32503,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HUD source integrated PR147 b8faf601. Latest asset receipt c97f17db. Game acceptance a1bfd563 is pre-fix.</t>
+          <t>Sole operator codex-play-guard. Current accepted184-file source PR147074c519b. First new asset save receipt31733, DeliveryHeroView/readback.json and saved-production-baseline.json.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>39_PRE_FIX_CHECKS_PASS; HUD_BUILD_PENDING</t>
+          <t>FIRST_NEW_NATIVE_SAVE_3_OF_3; TRACKED123; TARGETED_UI_PASS</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sole operator codex-play-guard accepted ONE HUD serial build then release/app-next31542. At05:19UTC four hd_batch workers remain active,7230/10000 exports; no producer no-next-heavy ACK. Fresh3.77GiB physical/1.92GiB virtual free is not a build grant. No post-fix compile/load/visual proof. Physical controller unverified. Eighteen holds unchanged; global READY unknown. TMOG UI-tool blocked. Photo notices closed.</t>
+          <t>Actual three native saves true2026-10-15T14:51:43.691578UTC: YellowIris4,Pickerelweed4,Cattail4.123 tracked packages =106StaticMesh+17Miri. Prior120 preserved,184 source/DLL/runtime,map5690 and101actors clean. World placement0/map save0 as of receipt. HeroR4 shore-flower fitting is a separate active step, not yet saved in this evidence.80/80 build exit0 and targeted HUD/7unpaired panels accepted10:16. Paired workflows, hardware/DPI/multiuser and explicit focus reacquisition remain open.</t>
         </is>
       </c>
     </row>
@@ -32534,12 +32535,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>BLENDER_SAVED_EXPORTED; VISUAL_REVIEW_PENDING; NATIVE_FALSE</t>
+          <t>FIRST_HERO_RENDERED; BELOW_BAR; R2_POLISH_ACTIVE; NATIVE_FALSE</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WORLD-ZERO; owner pootscoot. One authorized CPU2 Blender4.3.1 job exit0; 49,438 evaluated triangles/273 mesh-curve objects, 91.06x70.15x49.05m. Internal construct/export2.203s; peak not measured. Root verified Blend523805B c79df0a6..., GLB2714040B 9f6cca5f..., FBX1491292B cde7ae22.... Zero rendered views; separate review-render window31509 pending; no READY/intake grant.</t>
+          <t>WORLD-ZERO. Owner pootscoot retained and resumed31691/31692. Hub31707 at14:45:25UTC: r1/views/Sunspool_hero.png personally viewed,1100x900,24samples,1164366B. CPU2 render19.67s, Blender peak179.36MB, not Windows peak. Flat plateau, pointed path overlaps, hidden Heartstone and sparse fronts require focused R2 polish. Original exported files retained. Render lease31698 released. No READY/native acceptance.</t>
         </is>
       </c>
     </row>
@@ -32567,6 +32568,222 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>Observed05:04:28UTC; one36-triangle StaticMesh saved true,39726B SHAd8d5f8d5b2331ab75f24ec00ce4cef423dfd472d192e0abb30d41f8776caa7ff.103Static+17Miri=120tracked packages;119prior hashes/101actors/camera/map unchanged. Import0.415584s/save0.229938s are native phases. No replay after late guard halt. Zero placement/world save. Appearance/collision/ecosystem unverified. Not an island or blanket READY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Reviewed asset holds</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>qualified-intake/held-payload-reconciliation-20261015-144913.json</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ultra / buckwild-sol owns16. Team Claude / unreal-team owns2 dragons. Reconciliation saved/read back14:49:13UTC.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>18_HELD; 28_OF_28_PAYLOAD_HASHES_UNCHANGED; ZERO_CLEARED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3 fish +7 water +6 Rainlight +2 dragons. Receipt SHA256b363df09a79ce848e3f53ec99787a5b419a8b69d7db73389f90a0d6b2f5372e0. Rainlight v4 GLBs remain byte-identical to v3 and no FBX; no proven font defect. Dragon Walk clips have zero changing channels in inspected exports. Hub31701 routes16 to retained owner,31700 routes2 dragons. No accepted repaired packet/native result. Global qualified READY unknown.1266 source catalogue entries are not blanket READY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Young Bulrush qualification</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>task/qualified-intake/AquaticBulrushYoungR1/import-dispatch.json</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Owner canonical_workbook_audit. Task ACK14:44UTC. Packet saved14:48:10UTC and root rehashed. Original source author Claude retained.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SOURCE_PACKET_SAVED; OPERATOR_ACK31746; TRANSLATION_ACTIVE</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Dispatch JSON13580B SHA2564f2d63cdd9e204dcfa27975c1bab22fa088bbd8312ae7be0020d3a778f7b1bb1. Receipt SHA25637ec3a6af1164fed67a74aa2e2b0bb0c0563d64c65012fe652c9b2b9c298e71d. FBX15276B SHA2564a2b332eeb243bfd6b5e22467406b45241d9c3c4921b2c56691e60c6e452670c. Operator ACK31746 owns translation/helper. Packet is source preflight data, not executable native API. Its120package/101actor guard is historical after Marsh3 save; reconcile actual123package and post-placement baseline before execution. No native/BAR/world pass for Young.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TMOG live diagnostics</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>tmog-diagnostics-readonly/manifest.json and TMOG-READONLY-DIAGNOSTICS.md</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Owner closeout_asset_count. Bounded investigation complete. Manifest SHA256b5a6f23013243b8621eee5c36ce42825b7aa603648c88683cac34b799c80a1b5.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>INVESTIGATION_COMPLETE; LIVE_APP_DIAGNOSTICS_BLOCKED</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BLACKBEARD14:44:12-15UTC PID56912/version1.0.1.0. OS working set124.375 to127.0625MiB,124threads/1210handles are OS measurements, not app readings. No node_repl/@oai/sky and CUA native APIs disabled. Summary/Processes/Performance/minimized freshness untested and no window state changed.421 text files plus primary c1ce262d harness inspected; no supported TMOG export/IPC contract surfaced. Need supported native UI runtime or authoritative TMOG data contract. No adapter fabricated/source edits/process control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Photo / Image / SynapseFax workflows</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Existing task5 evidence/practical-paired-acceptance synthetic fixture lane</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Owner pootscoot-practical-apps. Explicit semantic acceptance hub31710 at14:46:52UTC of root31704. Native owner codex-play-guard.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IMAGE_PROTOCOL_OWNER_PASS; OTHER_FIXTURES_ACTIVE; NATIVE_PAIR_FALSE</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Owner reports Image114HTTP/375assertions/3persisted outputs/4hashes reread in separate JVM and six canonical guard cases passed. Root did not rerun. GUI/native pair remains false. Photo loopback/hardlink sandbox denial is not a product failure; narrow retry under review. Synapse preparing. Fax lacks accepted backend credential/config. Consolidated packet ETA10minutes from14:46:52UTC, not delivery proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Team Claude Blender sprint</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>October15 deadline19:00UTC / noon Pacific. Existing builders and BAR.md recipes.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Owner Team Claude / unreal-team. Hub31700 request and31706 supported ping delivered.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>DELIVERED; TASK_ACK_OWNERS_ETA_PENDING</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Request concrete non-overlapping builder assignments: owned dragon repairs, realm characters/biomes/modular floating-world islands and small reviewed import packets. Include seed, source/export paths, unit/material budgets and previews. Follow Ultra reference recipes and actual hardware capacity. Delivery does not establish acceptance or completed output. Sole Unreal writer remains Codex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ultra ecology source authoring</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>44 species /11 style-location families /3 growth stages. Existing request31687 / allocation31712.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Owner Ultra / buckwild-sol. Existing SUPERPOLISH lead ACK retained. Exact current allocation ACK/start pending.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ONE_CPU2_AUTHOR_JOB_ALLOCATED; OWNER_ACK_START_PENDING</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Source realm_ecology_pack.py SHA256117fd02dc3749ddf1d4a6f8cbd434c94dc8ec6ceb840657363312917e8bea4bb inspected. Author CLI serially resets11families, no family selector. One --mode author job to primary/artifacts/ecology/realm-plants-fungi-v1. Owner must acquire free lease and recheck resources, preserving Sunspool R2. No exports/renders grant and no root execution. No READY/native acceptance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Continuous qualified native intake</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>task-2/native-ingestion/MarshPlantersR1/DeliveryHeroView/readback.json + saved-production-baseline.json</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sole native operator codex-play-guard. Actual save report31733. Sourceexact YellowIris4/Pickerelweed4/Cattail4. Original Claude source credit retained.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>NATIVE_3_OF_3_SAVED; TRACKED123; WORLD_PLACEMENT_SEPARATE</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>True saves2026-10-15T14:51:43.691578UTC. Native668/172/290tri, exact colors/bounds/material/options accepted.123 packages =106StaticMesh+17Miri. Prior120 hashes,184 source/DLL/runtime,map5690/101actors preserved and clean. Worldplaced0/mapsave0 as of this receipt. Operator fitting new HeroR4 shore-flower detail; placement/save remains separately unverified here. Young31746 translation accepted; refresh current123 and actual post-placement protection before its execution. Source qualification/native asset save/world BAR remain separate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Owner docs / peer discussion</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Existing hub topic production-improvements-20261015. Requests31726operator,31727Sunspool,31728apps,31729Claude,31730Ultra,31731Grok,31732arcade.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Root/Poot DOCS_SAVED14:54:48UTC. Canonical BOARD/LESSONS-LEARNED-UNREAL.md SHA3287e16f36d879eae1164eb67afe1c5b13c471e1e59fe244cfa6eb6105830f30 and existing MESSAGES/art-handoff.md SHAb3ff808540986c0ff5600ca97edf54ca0cfd1d846ae48eef39b49fc701110f62. Readback receipt coordination-docs-append-1454-receipt.json.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>7_DELIVERED; CODEX_SUNSPOOL_OWNER_ACK; PEER_DOCS_PENDING; DISCUSSION_PENDING</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>codex-play-guard31726: delivered, owner ACK31745, docs pending, response pending. Active guard_auditDOCS + app_retry_packet_audit/Young translation; docs ETA10minutes from ACK. pootscoot/Sunspool31727: delivered, owner ACK31736, docs pending, response pending. Active model/render/handoff + cash_import_contract_review; docs ETA about1minute after views. pootscoot-practical-apps31728: delivered, owner ACK pending, docs pending, response pending. unreal-team/Claude31729: delivered, owner ACK pending, docs pending, response pending. buckwild-sol/Ultra31730: delivered, owner ACK pending, docs pending, response pending. Grok31731: delivered, owner ACK pending, docs pending, response pending; active roster unconfirmed. pootscoot-desktop-games31732: delivered, owner ACK pending, docs pending, response pending. Each lead must supply active-member individual ACKs, saved doc paths/hashes, actual measurements/recipes/failures and prioritized fixes, then read another owner and give actionable proposal/agreed owner. Root docs saved; root peer response/consensus pending. Production continues at safe checkpoints.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: realm audio into rd-jukebox (audit + seeds), tracker WZ43
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29832,6 +29832,33 @@
       <c r="E107" t="inlineStr">
         <is>
           <t>Map/screen -&gt; track via audio.json used_by; loop_end in samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>WZ43</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Realm music fed into the existing rd-jukebox as guest seed songs (20 MP3 + webp covers, cue manifest); sound for every realm event (54). Audit: rd-jukebox branch unmerged, off by default, no cue route for {cue, changed, sfx} yet</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_jukebox_seeds.py, rpg_audio.py -&gt; engines/unreal/art/claude-audio/jukebox-seeds; data/rpg/jukebox.json</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>done (verified on rd-jukebox build); cue route = jukebox owner</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Enable: DAEDALUS_JUKEBOX_ENABLED=true + SEED_SONGS_DIR; merge rd-jukebox; add a cue route that reads realm-cues.json</t>
         </is>
       </c>
     </row>
@@ -31715,7 +31742,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Docs: architecture 14.26 title + name entry, tracker WZ44
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29859,6 +29859,33 @@
       <c r="E108" t="inlineStr">
         <is>
           <t>Enable: DAEDALUS_JUKEBOX_ENABLED=true + SEED_SONGS_DIR; merge rd-jukebox; add a cue route that reads realm-cues.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>WZ44</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>RPG realms: animated title screens (scene, emblem, logo, menu, PRESS START) + name entry for both realms</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_title.py -&gt; engines/unreal/art/claude-battle-kit/&lt;realm&gt;/title; data/rpg/title.json</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Boot -&gt; Title (cue TITLE) -&gt; NEW GAME -&gt; name entry -&gt; party.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: WZ45-WZ51 (Prismheart demo, controllers, settings, start screen, name entry, shard quest, controller contract); keeps the PC's newer Team Claude rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DK9VUiyxsxHGgBLGV1tcPP
</commit_message>
<xml_diff>
--- a/docs/production/Realm-production-2026-10-13.xlsx
+++ b/docs/production/Realm-production-2026-10-13.xlsx
@@ -26773,7 +26773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29886,6 +29886,160 @@
       <c r="E109" t="inlineStr">
         <is>
           <t>Boot -&gt; Title (cue TITLE) -&gt; NEW GAME -&gt; name entry -&gt; party.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>WZ45</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Prismheart playable browser demo built only from the realm's own art, data and jukebox cues; ADR-052 {cue, changed, sfx} bodies drive a WebAudio jukebox</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>tools/rpg_demo/build_demo.py, index.html, play_test.py; artifact 'Prismheart Playable Demo'</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>done (playthrough PASS, seeded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>WZ46</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Controllers everywhere: shared web module DaedalusPad + mega controller bundle (SDL_GameControllerDB 1,018 USB pads + 145 curated models: Razer, GameSir, Nintendo, Sega, Atari, arcade); realm.html, demo and Java explore (GLFW) use it</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>static/controllers/daedalus-pad.js, controller-bundle.json; tools/controllers/*; daedalus-explore PadMappings; docs/controllers.md</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>done (pads 46/46, realm 13/13, explore 85/85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>WZ47</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Settings like Halo Infinite (Controller, Keyboard/Mouse, Video, Audio, Gameplay, Accessibility): one schema built from DaedalusSettings.cpp + hero layout tables, modular web store + panel; native follow-ups listed (Audio tab, cross-shaped stick dead zone)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>data/settings/settings-schema.json; tools/settings/*; static/settings/daedalus-settings.js; docs/settings.md</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>done web; native rows = Unreal operator</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>WZ48</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Prismheart start screen: full-screen display, live title menu (NEW GAME / CONTINUE / OPTIONS), all controls in the Settings tabs, inn save + CONTINUE, touch controls on phones only</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>tools/blender/rpg_title.py (TitleBg + menu_geometry); tools/rpg_demo/index.html, title_test.py</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>done (title 23/23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>WZ49</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Prismheart name entry (pad, keyboard, tap); realm Devices rows (connected pads, Teach Buttons)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>tools/rpg_demo/index.html; static/realm.js</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>WZ50</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Prismheart shard quest: Cinder Forge, Windcut Aerie, Sunwell Sanctum, The Shattered Heart; 3 Wardens + half-formed Prism Devourer (scaled openly for 3 of 6 shards), ending</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>tools/rpg_demo/build_demo.py, index.html, bot.py, quest_test.py; docs 14.28</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>done (quest 24/24, 3 seeds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>WZ51</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Controller contract v1 (frozen) + conformance vectors run on the web module and Codex's DaedalusPortalControls.h (generated C++, g++ C++20)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>data/controllers/controller-contract.json; tools/controllers/contract_*.py/js; docs/controller-contract.md</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>done (web 12/12, native 10/10); wiring into SDaedalusRealm = Unreal operator</t>
         </is>
       </c>
     </row>
@@ -32416,22 +32570,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>task/floating-islands/copperfall-ark-rest-842401/</t>
+          <t>task-3/copperfall-ark-rest-polish-842401/before/manifest.json; before-hero-resume-export-r2.process.json; before/renders/hero.png</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>build_copperfall.py | uncommitted SHA256 1ecfa42b28008b7f6050ee16eb704654b8cec56b3643c8ce889f4f8c13e12d50</t>
+          <t>Original creator production_checkpoint_evidence; additive overlay pootscoot, original8inputs unchanged. Retained Blend2787504B SHA2f2479083d994364d60cfbc8136dacccd895772afd5eed9153253a3d7ecde43f,269meshes/10000tri. Corrected own review driver SHA4db77cc7aaba9c09c29e6c9d5a306947e90fd6bfa9689d6edfb3a64fffa9ef25; three team harness responses submitted.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SOURCE_AUTHORED; BAR_READ; RESOURCE_SLOT_PENDING</t>
+          <t>ORIGINAL_BEFORE_EXPORT_HERO_SAVED;OWNER_VIEWED;AFTER_NATIVE_PENDING</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>WORLD-ZERO / Aetherflow district. Owner production_checkpoint_evidence. Seven planned role groups/four sockets; counts unmeasured. Blend/FBX/GLB/render/native not run. Root coordinator verified source; comparable rendered BAR review required.</t>
+          <t>Corrected recovery actual16:53:12UTC exit0/19.008s,CPU2; retained scene reopened without geometry rebuild. GLB812404B SHA87ac937eb27a422cc04fb5c1b0f785091df3f5b62d1e8e5df1e30987829a0117; FBX1031084B SHAe753b26946dacd078f8d2d20c1f46f457b9884328278f56b826152155048756c; hero892900B SHA071393291241d48f37a8812c7ab5e56cde1ab10b22ca99535a206dc982738e36. Prior export guard4.145s and unusedCAR_lamp recovery1.183s failures retained. Compute released32025. Fresh owner view identifies abrupt/raised route bends and checker-like grass; canopy joins need fitting. AFTER absent, native0, no BAR/playability acceptance.</t>
         </is>
       </c>
     </row>
@@ -32497,22 +32651,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>task/character-upgrades/aetherflow-habitat-r1/</t>
+          <t>task/character-upgrades/aetherflow-habitat-r1/polish-r1/{before-preview-r1,after-preview-r1}/; after-preview-r1-job/execution.json</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>build_nursery_station.py | uncommitted SHA256 1a5f8c3e5b66bd3fb59f68b7d1ac270bac4b1d771c686d41167ebdf7889052d0</t>
+          <t>Owner closeout_asset_count. Actual BEFORE16:20:14 exit0/16.363s; matched AFTER16:49:08.5235056UTC exit0/16.389s. Same hero_day,2CPU/8samples/800x600; station hidden vs visible. Original16pins retained;20plan/source/baseline checks passed per child report. Final child readback owner-reported SHA9fee21208a919da6434024290a4dd84da276f01c3238954e5a7a0db64de1417c; canonical nursery lesson saved16:55:47UTC.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SOURCE_AUTHORED; BAR_READ; RESOURCE_SLOT_PENDING</t>
+          <t>MATCHED_BEFORE_AFTER_SAVED_ROOT_VIEWED;SOURCE_ONLY;BAR_NATIVE_PENDING</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WORLD-ZERO / Aetherflow district. Owner closeout_asset_count. Nine source fingerprints; fish/pond reference-only, excluded station export. No scene/export/render/native; day/dusk/player/jetty comparisons pending.</t>
+          <t>Root viewed actual pair: purposeful additive canopy/lantern/bench/rails/jetty approach; low-sample softness, prop/player readability and refuge markers need further review. AFTER PNG591578B SHAfdf0480ce82cb00689b20f2a7ab280d2d4c0de5ae3cc546edf9f913c7e64c7f2. GLB352904B byte-identical BEFORE/AFTER SHA224af849734273a5afa8b8f05f59957a09032f51231eb2e98ac4f8a60e9a8f48; station97meshes/6388tri/9materials, context excluded. Terminal/release16:49:08.5907195UTC verified. No BAR/native/physics/ecology/READY claim.</t>
         </is>
       </c>
     </row>
@@ -32551,22 +32705,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CodexContest/codex-arcade-gameplay-0344.checkpoint.json</t>
+          <t>task-2/native-ingestion/SunspoolThreeRolesR4/Placement/readback.json + saved-production-baseline.json</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sole operator codex-play-guard. Current accepted184-file source PR147074c519b. First new asset save receipt31733, DeliveryHeroView/readback.json and saved-production-baseline.json.</t>
+          <t>Sole native operator codex-play-guard. Accepted184 source/runtime074c519b retained. Poot original Sunspool source retained. Three-role native placement baseline16:13:57UTC SHA98c689e6a7945133d448a33ba37d4df9305de0500922d635ff8eb6334e47d080. Detailed operations LOCAL.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FIRST_NEW_NATIVE_SAVE_3_OF_3; TRACKED123; TARGETED_UI_PASS</t>
+          <t>131_PACKAGES;124_ACTORS;SUNSPOOL3ROLE_SUBSET_PLACED_MAP_SAVED;TARGETED_UI_ONLY</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Actual three native saves true2026-10-15T14:51:43.691578UTC: YellowIris4,Pickerelweed4,Cattail4.123 tracked packages =106StaticMesh+17Miri. Prior120 preserved,184 source/DLL/runtime,map5690 and101actors clean. World placement0/map save0 as of receipt. HeroR4 shore-flower fitting is a separate active step, not yet saved in this evidence.80/80 build exit0 and targeted HUD/7unpaired panels accepted10:16. Paired workflows, hardware/DPI/multiuser and explicit focus reacquisition remain open.</t>
+          <t>Retained baseline131packages/124actors: six Sunspool packages (3StaticMesh+3ownedMICs) saved16:06:56UTC, then11new decorative actors (3roles+8owned supports), all113prior records unchanged. Map saveTRUE20.232948s;209372448B SHAd0af38071b022fb2688b873a8b709eddf5e3ec77b0b644067489e416c26c45c3. Exact1076tri/material/bounds/save checks passed. Only3of307source meshes delivered. Full scene, final BAR/collision/navigation/playability and paired app acceptance remain unaccepted.</t>
         </is>
       </c>
     </row>
@@ -32578,22 +32732,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-10-13/task-3/sunspool-refuge/r1/Sunspool_Refuge.blend; exports/Sunspool_Refuge.glb + .fbx</t>
+          <t>C:\Users\730ri\Documents\Codex\2026-10-13\task-3\sunspool-refuge\r4\Sunspool_Refuge.blend; C:\Users\730ri\Documents\Codex\2026-10-13\task-3\sunspool-refuge\r4\exports\Sunspool_Refuge.glb + .fbx; actual views C:\Users\730ri\Documents\Codex\2026-10-13\task-3\sunspool-refuge\r4\views</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>build source f7b9f82a + foliage 92abfb98; manifest SHA256 131af600f2b8ad9ae6cd2c19d7f82d71615d67ea4d1a34179028d6686f505bd1</t>
+          <t>R4 manifest SHA256 e4e4e1e8f3897273899b30c8b50845a493a81b8f5df3d8d8f2b7d697d2128d9a; exact source/export/audit pins C:\Users\730ri\Documents\Codex\2026-10-13\task-3\sunspool-refuge\delivery\import-review.json</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FIRST_HERO_RENDERED; BELOW_BAR; R2_POLISH_ACTIVE; NATIVE_FALSE</t>
+          <t>BLENDER_REVIEWED_EXPORTED; NATIVE_PROFILE_HELD; READY_FALSE</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>WORLD-ZERO. Owner pootscoot retained and resumed31691/31692. Hub31707 at14:45:25UTC: r1/views/Sunspool_hero.png personally viewed,1100x900,24samples,1164366B. CPU2 render19.67s, Blender peak179.36MB, not Windows peak. Flat plateau, pointed path overlaps, hidden Heartstone and sparse fronts require focused R2 polish. Original exported files retained. Render lease31698 released. No READY/native acceptance.</t>
+          <t>WORLD-ZERO; owner pootscoot; seed861503; R1/R2/R3 preserved. R4 six actual views personally+independently reviewed,76739tri/307meshes/26PBR,maxGLBusedslots3. Fixed route joins/serrations, keel pinch, Heartstone washout and terrain T-junction seams. Binary8/8comparisons; ground one connected surface/one outerloop/zeroT-junction candidates at1e-5m. Native0; collision/nav/LOD/gameplay unaccepted. Source1m/GLB Y-up/FBXfactor100; native owner profile/unit/material decision required. Peer31757; docs31750; individualmember audits31796.</t>
         </is>
       </c>
     </row>
@@ -32659,22 +32813,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>task/qualified-intake/AquaticBulrushYoungR1/import-dispatch.json</t>
+          <t>task-2/native-ingestion/BulrushYoungR1/Delivery/readback.json; ViewportHeroR4AfterYoung/saved-production-baseline.json</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Owner canonical_workbook_audit. Task ACK14:44UTC. Packet saved14:48:10UTC and root rehashed. Original source author Claude retained.</t>
+          <t>Claude original source retained; canonical_workbook_audit source packet; codex-play-guard/app_retry_packet_audit admission. Source FBX15276B SHA4a2b332eeb243bfd6b5e22467406b45241d9c3c4921b2c56691e60c6e452670c. Actual native receipt31842.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SOURCE_PACKET_SAVED; OPERATOR_ACK31746; TRANSLATION_ACTIVE</t>
+          <t>YOUNG_NATIVE_SAVED_READBACK_COMPLETE;WORLD_PLACEMENT0;BAR_OPEN</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Dispatch JSON13580B SHA2564f2d63cdd9e204dcfa27975c1bab22fa088bbd8312ae7be0020d3a778f7b1bb1. Receipt SHA25637ec3a6af1164fed67a74aa2e2b0bb0c0563d64c65012fe652c9b2b9c298e71d. FBX15276B SHA2564a2b332eeb243bfd6b5e22467406b45241d9c3c4921b2c56691e60c6e452670c. Operator ACK31746 owns translation/helper. Packet is source preflight data, not executable native API. Its120package/101actor guard is historical after Marsh3 save; reconcile actual123package and post-placement baseline before execution. No native/BAR/world pass for Young.</t>
+          <t>True save15:34:00/readback15:34:21UTC. /Game/Daedalus/Art/Islands/CodexContest/Ingestion/Aquatic_Bulrush_Young_4a2b332eeb243bfd/Prop_Aquatic_Marsh_Bulrush_2 saved36868B SHA7df8d64a31359b8863a7e982a16d0f0090eee05adee18dc1b6f3754c068d3d3a.56tri; import0.130762s/saveTRUE0.081899s are native phases. Existing Interchange/build1/M_Voxel route, futureactor.01; world placement0. All124prior packages/113actors/mapc644/184source preserved. Appearance/collision/playability unaccepted; no replay or blanket READY.</t>
         </is>
       </c>
     </row>
@@ -32713,22 +32867,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Existing task5 evidence/practical-paired-acceptance synthetic fixture lane</t>
+          <t>2026-10-13/task-5/evidence/fax-synthetic-backend/joined-b9ac21fd-2151-4081-8a0c-ef70c6f18efb/result.json; JVM-reopen proof covers recorded job/document projection only; full POST/retry/GET tuple+Instant separately passed4 focused tests.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Owner pootscoot-practical-apps. Explicit semantic acceptance hub31710 at14:46:52UTC of root31704. Native owner codex-play-guard.</t>
+          <t>Owner pootscoot-practical-apps; source93d328d5 owner checkpoint. Retained result sourceBaseHead5e005c2afb0b8a46308b069a653da57f2649d5b8 is separately identified. One Fax synthetic2phase process PASS71.279s, exit0, terminal16:51:47.254UTC. Native owner codex-play-guard remains sole writer.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>IMAGE_PROTOCOL_OWNER_PASS; OTHER_FIXTURES_ACTIVE; NATIVE_PAIR_FALSE</t>
+          <t>FAX_SYNTHETIC2PHASE_PASS;COMPANION_FIXTURES_PASS;NATIVE_PROVIDER_UNACCEPTED</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Owner reports Image114HTTP/375assertions/3persisted outputs/4hashes reread in separate JVM and six canonical guard cases passed. Root did not rerun. GUI/native pair remains false. Photo loopback/hardlink sandbox denial is not a product failure; narrow retry under review. Synapse preparing. Fax lacks accepted backend credential/config. Consolidated packet ETA10minutes from14:46:52UTC, not delivery proof.</t>
+          <t>Both synthetic phases downloaded actual page text/QR, JavaZXing/PDFBox verified. Independent JVM reopen verified recorded job/document projection and onejob only, not expiry/recipient; cancellation persisted. Full POST/retry/GET tuple+Instant separately passed4 focused tests. Cleanup completed and8ports refused. Synthetic file-backedH2/test-only statefulRedis mock; no provider transmission, native pairing, production auth, PostgreSQL or realRedis acceptance. Photo/Image/Synapse companion evidence remains separate from native jobs. Source prepare-expiry-microseconds delta recorded, not production-auth proof. Detailed operations LOCAL; no account/provider/config change.</t>
         </is>
       </c>
     </row>
@@ -32794,22 +32948,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>task-2/native-ingestion/MarshPlantersR1/DeliveryHeroView/readback.json + saved-production-baseline.json</t>
+          <t>task-2/native-ingestion/SunspoolThreeRolesR4/Placement/readback.json + saved-production-baseline.json</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sole native operator codex-play-guard. Actual save report31733. Sourceexact YellowIris4/Pickerelweed4/Cattail4. Original Claude source credit retained.</t>
+          <t>Sole native operator codex-play-guard. Poot source subset BronzeSunRim-0.4/DyeHouse_FabricBolt0/DyeHouse_FoldedTealRoof retained,1076tri. Six new saved packages =3static+3ownedMICs; eleven new owned decorative actors.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>NATIVE_3_OF_3_SAVED; TRACKED123; WORLD_PLACEMENT_SEPARATE</t>
+          <t>SUNSPOOL3ROLE_SUBSET_NATIVE_SAVED_PLACED;131PACKAGES;124ACTORS</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>True saves2026-10-15T14:51:43.691578UTC. Native668/172/290tri, exact colors/bounds/material/options accepted.123 packages =106StaticMesh+17Miri. Prior120 hashes,184 source/DLL/runtime,map5690/101actors preserved and clean. Worldplaced0/mapsave0 as of this receipt. Operator fitting new HeroR4 shore-flower detail; placement/save remains separately unverified here. Young31746 translation accepted; refresh current123 and actual post-placement protection before its execution. Source qualification/native asset save/world BAR remain separate.</t>
+          <t>Source GLB33440B SHAabd4fefd3c7bdc2cc312cb4d5428b0f3e82e61143e08afc0991639a7fd9dca97. Three exact source roles saved with owned material instances16:06:56UTC. Placement/readback16:13:58UTC:113prior+11new actors, mapTRUE20.232948s,131packages,184source preserved. Decorative staging only; eight supports are Codex additions. Full307mesh/26PBR source row36 remains its separate held source record. No fullSunspool, collision/navigation/nativeBAR/playability or future generalized importer acceptance.</t>
         </is>
       </c>
     </row>
@@ -32826,17 +32980,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Root/Poot DOCS_SAVED14:54:48UTC. Canonical BOARD/LESSONS-LEARNED-UNREAL.md SHA3287e16f36d879eae1164eb67afe1c5b13c471e1e59fe244cfa6eb6105830f30 and existing MESSAGES/art-handoff.md SHAb3ff808540986c0ff5600ca97edf54ca0cfd1d846ae48eef39b49fc701110f62. Readback receipt coordination-docs-append-1454-receipt.json.</t>
+          <t>Root/Poot DOCS_SAVED14:54:48UTC. Canonical BOARD/LESSONS-LEARNED-UNREAL.md SHA3287e16f36d879eae1164eb67afe1c5b13c471e1e59fe244cfa6eb6105830f30 and existing MESSAGES/art-handoff.md SHAb3ff808540986c0ff5600ca97edf54ca0cfd1d846ae48eef39b49fc701110f62. Readback receipt coordination-docs-append-1454-receipt.json. Later individual audit receipts:20known complete = coordination6 + Sunspool3 + native4 + apps7; global member denominator unknown. Native31833-31836, Sunspool31796, apps31801-31806/31811; separate nursery-preflight-review completed15:59:15UTC SHA87394de395a2c82fec1ce56b11b603cc52f75c3c96b352892fb34e988e02baae. Each has bounded read scope/time; no lead-to-whole-team completion inference.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>7_DELIVERED; CODEX_SUNSPOOL_OWNER_ACK; PEER_DOCS_PENDING; DISCUSSION_PENDING</t>
+          <t>20_INDIVIDUAL_AUDITS_COMPLETE;GLOBAL_DENOMINATOR_UNKNOWN;3_LEADS_DOCS_PEER_RESPONSE</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>codex-play-guard31726: delivered, owner ACK31745, docs pending, response pending. Active guard_auditDOCS + app_retry_packet_audit/Young translation; docs ETA10minutes from ACK. pootscoot/Sunspool31727: delivered, owner ACK31736, docs pending, response pending. Active model/render/handoff + cash_import_contract_review; docs ETA about1minute after views. pootscoot-practical-apps31728: delivered, owner ACK pending, docs pending, response pending. unreal-team/Claude31729: delivered, owner ACK pending, docs pending, response pending. buckwild-sol/Ultra31730: delivered, owner ACK pending, docs pending, response pending. Grok31731: delivered, owner ACK pending, docs pending, response pending; active roster unconfirmed. pootscoot-desktop-games31732: delivered, owner ACK pending, docs pending, response pending. Each lead must supply active-member individual ACKs, saved doc paths/hashes, actual measurements/recipes/failures and prioritized fixes, then read another owner and give actionable proposal/agreed owner. Root docs saved; root peer response/consensus pending. Production continues at safe checkpoints.</t>
+          <t>codex-play-guard31726: OWNER_ACK31745; DOCS_SAVED31780/31848; PEER_RESPONSE31780; four individual bounded receipts31833-31836. Current131packages/124actors/mapd0af; exact3role Sunspool subset saved/placed, full scene not delivered. pootscoot/Sunspool31727: owner ACK31736; DOCS_SAVED31750; PEER_DISCUSSION31757; individual3member bounded audit receipts31796. Root/pootscoot source polish/handoff; cash_import_contract_review binaryaudit; tmog_official_interface actual-view review. R4 final6views reviewed,76739tri/307meshes/26PBR; native profile held. Exact handoff task-3/sunspool-refuge/handoff.json. pootscoot-practical-apps31728: OWNER_ACK/DOCS_SAVED/PEER_RESPONSE31754; seven individual bounded audit receipts31801-31806/31811. Fax synthetic2phase PASS16:51:47UTC/71.279s, actual joined-b9ac21fd result; crossJVM job/document projection only, not expiry/recipient. Full POST/retry/GET tuple+Instant separately passed4 focused tests. Provider/native/production-auth/PostgreSQL/realRedis unaccepted. Other companion evidence remains separate from native pairing. unreal-team/Claude31729: delivered, owner ACK pending, docs pending, response pending. buckwild-sol/Ultra31730: delivered, owner ACK pending, docs pending, response pending. Grok31731: delivered, owner ACK pending, docs pending, response pending; active roster unconfirmed. pootscoot-desktop-games31732: delivered, owner ACK pending, docs pending, response pending. Each lead must supply active-member individual ACKs, saved doc paths/hashes, actual measurements/recipes/failures and prioritized fixes, then read another owner and give actionable proposal/agreed owner. Root docs saved; root peer response/consensus pending. Production continues at safe checkpoints.</t>
         </is>
       </c>
     </row>

</xml_diff>